<commit_message>
Prepare verified Swahili course checkpoint
</commit_message>
<xml_diff>
--- a/patois_learn_database_1.xlsx
+++ b/patois_learn_database_1.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra25124598cae484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concepts" sheetId="2" r:id="R2d07117495904333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="3" r:id="Rad72d13baffa4c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="course_vocabulary" sheetId="4" r:id="Re0a862d29c0a413c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chapters" sheetId="5" r:id="R7e989f2fb01a4c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="topics" sheetId="6" r:id="R840912dd2d6348c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lesson_steps" sheetId="7" r:id="R9d24f92f20824425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf29364f92b264803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concepts" sheetId="2" r:id="Rd7a96550a7bb4f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="3" r:id="R1fa865f6cc8844bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="course_vocabulary" sheetId="4" r:id="Re662ffe04c864afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chapters" sheetId="5" r:id="R51b8a7d62b3745de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="topics" sheetId="6" r:id="R97396c530be74fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lesson_steps" sheetId="7" r:id="Rb1892027d05d4543"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -387,7 +387,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="lessonstepsTable" displayName="lessonstepsTable" ref="A1:M65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="lessonstepsTable" displayName="lessonstepsTable" ref="A1:M129" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="course_id"/>
     <x:tableColumn id="2" name="topic_id"/>
@@ -1453,7 +1453,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R683d6176ab944ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R936a88d8848f493f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1673,7 +1673,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1037f1897ab4458"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1495842f5454f49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2903,18 +2903,20 @@
       <x:c r="B41" s="26" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="C41" s="26"/>
-      <x:c r="D41" s="26"/>
+      <x:c r="C41" s="26" t="str">
+        <x:v>Ndiyo</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="str">
+        <x:v>N-DEE-yoh</x:v>
+      </x:c>
       <x:c r="E41" s="26"/>
       <x:c r="F41" s="26" t="str">
         <x:v>assets/images/vocab/swahili/yes.png</x:v>
       </x:c>
-      <x:c r="G41" s="26" t="str">
-        <x:v>assets/audio/swahili/yes.mp3</x:v>
-      </x:c>
+      <x:c r="G41" s="26" t="str"/>
       <x:c r="H41" s="26"/>
       <x:c r="I41" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J41" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -2927,18 +2929,20 @@
       <x:c r="B42" s="26" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="C42" s="26"/>
-      <x:c r="D42" s="26"/>
+      <x:c r="C42" s="26" t="str">
+        <x:v>Hapana</x:v>
+      </x:c>
+      <x:c r="D42" s="26" t="str">
+        <x:v>hah-PAH-nah</x:v>
+      </x:c>
       <x:c r="E42" s="26"/>
       <x:c r="F42" s="26" t="str">
         <x:v>assets/images/vocab/swahili/no.png</x:v>
       </x:c>
-      <x:c r="G42" s="26" t="str">
-        <x:v>assets/audio/swahili/no.mp3</x:v>
-      </x:c>
+      <x:c r="G42" s="26" t="str"/>
       <x:c r="H42" s="26"/>
       <x:c r="I42" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J42" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -2951,18 +2955,20 @@
       <x:c r="B43" s="26" t="str">
         <x:v>maybe</x:v>
       </x:c>
-      <x:c r="C43" s="26"/>
-      <x:c r="D43" s="26"/>
+      <x:c r="C43" s="26" t="str">
+        <x:v>Labda</x:v>
+      </x:c>
+      <x:c r="D43" s="26" t="str">
+        <x:v>LAHB-dah</x:v>
+      </x:c>
       <x:c r="E43" s="26"/>
       <x:c r="F43" s="26" t="str">
         <x:v>assets/images/vocab/swahili/maybe.png</x:v>
       </x:c>
-      <x:c r="G43" s="26" t="str">
-        <x:v>assets/audio/swahili/maybe.mp3</x:v>
-      </x:c>
+      <x:c r="G43" s="26" t="str"/>
       <x:c r="H43" s="26"/>
       <x:c r="I43" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J43" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -2975,18 +2981,20 @@
       <x:c r="B44" s="26" t="str">
         <x:v>okay</x:v>
       </x:c>
-      <x:c r="C44" s="26"/>
-      <x:c r="D44" s="26"/>
+      <x:c r="C44" s="26" t="str">
+        <x:v>Sawa</x:v>
+      </x:c>
+      <x:c r="D44" s="26" t="str">
+        <x:v>SAH-wah</x:v>
+      </x:c>
       <x:c r="E44" s="26"/>
       <x:c r="F44" s="26" t="str">
         <x:v>assets/images/vocab/swahili/okay.png</x:v>
       </x:c>
-      <x:c r="G44" s="26" t="str">
-        <x:v>assets/audio/swahili/okay.mp3</x:v>
-      </x:c>
+      <x:c r="G44" s="26" t="str"/>
       <x:c r="H44" s="26"/>
       <x:c r="I44" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J44" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -2999,18 +3007,20 @@
       <x:c r="B45" s="26" t="str">
         <x:v>again</x:v>
       </x:c>
-      <x:c r="C45" s="26"/>
-      <x:c r="D45" s="26"/>
+      <x:c r="C45" s="26" t="str">
+        <x:v>Tena</x:v>
+      </x:c>
+      <x:c r="D45" s="26" t="str">
+        <x:v>TEH-nah</x:v>
+      </x:c>
       <x:c r="E45" s="26"/>
       <x:c r="F45" s="26" t="str">
         <x:v>assets/images/vocab/swahili/again.png</x:v>
       </x:c>
-      <x:c r="G45" s="26" t="str">
-        <x:v>assets/audio/swahili/again.mp3</x:v>
-      </x:c>
+      <x:c r="G45" s="26" t="str"/>
       <x:c r="H45" s="26"/>
       <x:c r="I45" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J45" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3023,18 +3033,20 @@
       <x:c r="B46" s="26" t="str">
         <x:v>good-afternoon</x:v>
       </x:c>
-      <x:c r="C46" s="26"/>
-      <x:c r="D46" s="26"/>
+      <x:c r="C46" s="26" t="str">
+        <x:v>Habari ya mchana</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>hah-BAH-ree yah m-CHAH-nah</x:v>
+      </x:c>
       <x:c r="E46" s="26"/>
       <x:c r="F46" s="26" t="str">
         <x:v>assets/images/vocab/swahili/good-afternoon.png</x:v>
       </x:c>
-      <x:c r="G46" s="26" t="str">
-        <x:v>assets/audio/swahili/good-afternoon.mp3</x:v>
-      </x:c>
+      <x:c r="G46" s="26" t="str"/>
       <x:c r="H46" s="26"/>
       <x:c r="I46" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J46" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3047,18 +3059,20 @@
       <x:c r="B47" s="26" t="str">
         <x:v>nice-to-meet-you</x:v>
       </x:c>
-      <x:c r="C47" s="26"/>
-      <x:c r="D47" s="26"/>
+      <x:c r="C47" s="26" t="str">
+        <x:v>Nimefurahi kukutana nawe</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>nee-meh-foo-RAH-hee koo-koo-TAH-nah NAH-weh</x:v>
+      </x:c>
       <x:c r="E47" s="26"/>
       <x:c r="F47" s="26" t="str">
         <x:v>assets/images/vocab/swahili/nice-to-meet-you.png</x:v>
       </x:c>
-      <x:c r="G47" s="26" t="str">
-        <x:v>assets/audio/swahili/nice-to-meet-you.mp3</x:v>
-      </x:c>
+      <x:c r="G47" s="26" t="str"/>
       <x:c r="H47" s="26"/>
       <x:c r="I47" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J47" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3071,18 +3085,20 @@
       <x:c r="B48" s="26" t="str">
         <x:v>long-time-no-see</x:v>
       </x:c>
-      <x:c r="C48" s="26"/>
-      <x:c r="D48" s="26"/>
+      <x:c r="C48" s="26" t="str">
+        <x:v>Hatujaonana kwa muda mrefu</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>hah-too-jah-oh-NAH-nah kwah MOO-dah m-REH-foo</x:v>
+      </x:c>
       <x:c r="E48" s="26"/>
       <x:c r="F48" s="26" t="str">
         <x:v>assets/images/vocab/swahili/long-time-no-see.png</x:v>
       </x:c>
-      <x:c r="G48" s="26" t="str">
-        <x:v>assets/audio/swahili/long-time-no-see.mp3</x:v>
-      </x:c>
+      <x:c r="G48" s="26" t="str"/>
       <x:c r="H48" s="26"/>
       <x:c r="I48" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J48" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3095,18 +3111,20 @@
       <x:c r="B49" s="26" t="str">
         <x:v>how-is-your-day</x:v>
       </x:c>
-      <x:c r="C49" s="26"/>
-      <x:c r="D49" s="26"/>
+      <x:c r="C49" s="26" t="str">
+        <x:v>Siku yako inaendeleaje?</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>SEE-koo YAH-koh ee-nah-ehn-deh-leh-AH-jeh</x:v>
+      </x:c>
       <x:c r="E49" s="26"/>
       <x:c r="F49" s="26" t="str">
         <x:v>assets/images/vocab/swahili/how-is-your-day.png</x:v>
       </x:c>
-      <x:c r="G49" s="26" t="str">
-        <x:v>assets/audio/swahili/how-is-your-day.mp3</x:v>
-      </x:c>
+      <x:c r="G49" s="26" t="str"/>
       <x:c r="H49" s="26"/>
       <x:c r="I49" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J49" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3119,18 +3137,20 @@
       <x:c r="B50" s="26" t="str">
         <x:v>have-a-good-day</x:v>
       </x:c>
-      <x:c r="C50" s="26"/>
-      <x:c r="D50" s="26"/>
+      <x:c r="C50" s="26" t="str">
+        <x:v>Uwe na siku njema</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>OO-weh nah SEE-koo N-JEH-mah</x:v>
+      </x:c>
       <x:c r="E50" s="26"/>
       <x:c r="F50" s="26" t="str">
         <x:v>assets/images/vocab/swahili/have-a-good-day.png</x:v>
       </x:c>
-      <x:c r="G50" s="26" t="str">
-        <x:v>assets/audio/swahili/have-a-good-day.mp3</x:v>
-      </x:c>
+      <x:c r="G50" s="26" t="str"/>
       <x:c r="H50" s="26"/>
       <x:c r="I50" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J50" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3143,18 +3163,20 @@
       <x:c r="B51" s="26" t="str">
         <x:v>what-is-your-name</x:v>
       </x:c>
-      <x:c r="C51" s="26"/>
-      <x:c r="D51" s="26"/>
+      <x:c r="C51" s="26" t="str">
+        <x:v>Jina lako ni nani?</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>JEE-nah LAH-koh nee NAH-nee</x:v>
+      </x:c>
       <x:c r="E51" s="26"/>
       <x:c r="F51" s="26" t="str">
         <x:v>assets/images/vocab/swahili/what-is-your-name.png</x:v>
       </x:c>
-      <x:c r="G51" s="26" t="str">
-        <x:v>assets/audio/swahili/what-is-your-name.mp3</x:v>
-      </x:c>
+      <x:c r="G51" s="26" t="str"/>
       <x:c r="H51" s="26"/>
       <x:c r="I51" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J51" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3167,18 +3189,20 @@
       <x:c r="B52" s="26" t="str">
         <x:v>my-name-is</x:v>
       </x:c>
-      <x:c r="C52" s="26"/>
-      <x:c r="D52" s="26"/>
+      <x:c r="C52" s="26" t="str">
+        <x:v>Jina langu ni...</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>JEE-nah LAHN-goo nee</x:v>
+      </x:c>
       <x:c r="E52" s="26"/>
       <x:c r="F52" s="26" t="str">
         <x:v>assets/images/vocab/swahili/my-name-is.png</x:v>
       </x:c>
-      <x:c r="G52" s="26" t="str">
-        <x:v>assets/audio/swahili/my-name-is.mp3</x:v>
-      </x:c>
+      <x:c r="G52" s="26" t="str"/>
       <x:c r="H52" s="26"/>
       <x:c r="I52" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J52" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3191,18 +3215,20 @@
       <x:c r="B53" s="26" t="str">
         <x:v>i-am-a-student</x:v>
       </x:c>
-      <x:c r="C53" s="26"/>
-      <x:c r="D53" s="26"/>
+      <x:c r="C53" s="26" t="str">
+        <x:v>Mimi ni mwanafunzi</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>MEE-mee nee mwah-nah-FOON-zee</x:v>
+      </x:c>
       <x:c r="E53" s="26"/>
       <x:c r="F53" s="26" t="str">
         <x:v>assets/images/vocab/swahili/i-am-a-student.png</x:v>
       </x:c>
-      <x:c r="G53" s="26" t="str">
-        <x:v>assets/audio/swahili/i-am-a-student.mp3</x:v>
-      </x:c>
+      <x:c r="G53" s="26" t="str"/>
       <x:c r="H53" s="26"/>
       <x:c r="I53" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J53" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3215,18 +3241,20 @@
       <x:c r="B54" s="26" t="str">
         <x:v>i-am-learning</x:v>
       </x:c>
-      <x:c r="C54" s="26"/>
-      <x:c r="D54" s="26"/>
+      <x:c r="C54" s="26" t="str">
+        <x:v>Ninajifunza...</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>nee-nah-jee-FOON-zah</x:v>
+      </x:c>
       <x:c r="E54" s="26"/>
       <x:c r="F54" s="26" t="str">
         <x:v>assets/images/vocab/swahili/i-am-learning.png</x:v>
       </x:c>
-      <x:c r="G54" s="26" t="str">
-        <x:v>assets/audio/swahili/i-am-learning.mp3</x:v>
-      </x:c>
+      <x:c r="G54" s="26" t="str"/>
       <x:c r="H54" s="26"/>
       <x:c r="I54" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J54" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3239,18 +3267,20 @@
       <x:c r="B55" s="26" t="str">
         <x:v>i-speak</x:v>
       </x:c>
-      <x:c r="C55" s="26"/>
-      <x:c r="D55" s="26"/>
+      <x:c r="C55" s="26" t="str">
+        <x:v>Ninazungumza...</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>nee-nah-zoon-GOOM-zah</x:v>
+      </x:c>
       <x:c r="E55" s="26"/>
       <x:c r="F55" s="26" t="str">
         <x:v>assets/images/vocab/swahili/i-speak.png</x:v>
       </x:c>
-      <x:c r="G55" s="26" t="str">
-        <x:v>assets/audio/swahili/i-speak.mp3</x:v>
-      </x:c>
+      <x:c r="G55" s="26" t="str"/>
       <x:c r="H55" s="26"/>
       <x:c r="I55" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J55" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3263,18 +3293,20 @@
       <x:c r="B56" s="26" t="str">
         <x:v>where-are-you-from</x:v>
       </x:c>
-      <x:c r="C56" s="26"/>
-      <x:c r="D56" s="26"/>
+      <x:c r="C56" s="26" t="str">
+        <x:v>Unatoka wapi?</x:v>
+      </x:c>
+      <x:c r="D56" s="26" t="str">
+        <x:v>oo-nah-TOH-kah WAH-pee</x:v>
+      </x:c>
       <x:c r="E56" s="26"/>
       <x:c r="F56" s="26" t="str">
         <x:v>assets/images/vocab/swahili/where-are-you-from.png</x:v>
       </x:c>
-      <x:c r="G56" s="26" t="str">
-        <x:v>assets/audio/swahili/where-are-you-from.mp3</x:v>
-      </x:c>
+      <x:c r="G56" s="26" t="str"/>
       <x:c r="H56" s="26"/>
       <x:c r="I56" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J56" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3287,18 +3319,20 @@
       <x:c r="B57" s="26" t="str">
         <x:v>i-am-from</x:v>
       </x:c>
-      <x:c r="C57" s="26"/>
-      <x:c r="D57" s="26"/>
+      <x:c r="C57" s="26" t="str">
+        <x:v>Ninatoka...</x:v>
+      </x:c>
+      <x:c r="D57" s="26" t="str">
+        <x:v>nee-nah-TOH-kah</x:v>
+      </x:c>
       <x:c r="E57" s="26"/>
       <x:c r="F57" s="26" t="str">
         <x:v>assets/images/vocab/swahili/i-am-from.png</x:v>
       </x:c>
-      <x:c r="G57" s="26" t="str">
-        <x:v>assets/audio/swahili/i-am-from.mp3</x:v>
-      </x:c>
+      <x:c r="G57" s="26" t="str"/>
       <x:c r="H57" s="26"/>
       <x:c r="I57" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J57" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3311,18 +3345,20 @@
       <x:c r="B58" s="26" t="str">
         <x:v>where-do-you-live</x:v>
       </x:c>
-      <x:c r="C58" s="26"/>
-      <x:c r="D58" s="26"/>
+      <x:c r="C58" s="26" t="str">
+        <x:v>Unaishi wapi?</x:v>
+      </x:c>
+      <x:c r="D58" s="26" t="str">
+        <x:v>oo-nah-EE-shee WAH-pee</x:v>
+      </x:c>
       <x:c r="E58" s="26"/>
       <x:c r="F58" s="26" t="str">
         <x:v>assets/images/vocab/swahili/where-do-you-live.png</x:v>
       </x:c>
-      <x:c r="G58" s="26" t="str">
-        <x:v>assets/audio/swahili/where-do-you-live.mp3</x:v>
-      </x:c>
+      <x:c r="G58" s="26" t="str"/>
       <x:c r="H58" s="26"/>
       <x:c r="I58" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J58" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3335,18 +3371,20 @@
       <x:c r="B59" s="26" t="str">
         <x:v>i-live-in</x:v>
       </x:c>
-      <x:c r="C59" s="26"/>
-      <x:c r="D59" s="26"/>
+      <x:c r="C59" s="26" t="str">
+        <x:v>Ninaishi...</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>nee-nah-EE-shee</x:v>
+      </x:c>
       <x:c r="E59" s="26"/>
       <x:c r="F59" s="26" t="str">
         <x:v>assets/images/vocab/swahili/i-live-in.png</x:v>
       </x:c>
-      <x:c r="G59" s="26" t="str">
-        <x:v>assets/audio/swahili/i-live-in.mp3</x:v>
-      </x:c>
+      <x:c r="G59" s="26" t="str"/>
       <x:c r="H59" s="26"/>
       <x:c r="I59" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J59" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3359,18 +3397,20 @@
       <x:c r="B60" s="26" t="str">
         <x:v>which-language-do-you-speak</x:v>
       </x:c>
-      <x:c r="C60" s="26"/>
-      <x:c r="D60" s="26"/>
+      <x:c r="C60" s="26" t="str">
+        <x:v>Unazungumza lugha gani?</x:v>
+      </x:c>
+      <x:c r="D60" s="26" t="str">
+        <x:v>oo-nah-zoon-GOOM-zah LOO-ghah GAH-nee</x:v>
+      </x:c>
       <x:c r="E60" s="26"/>
       <x:c r="F60" s="26" t="str">
         <x:v>assets/images/vocab/swahili/which-language-do-you-speak.png</x:v>
       </x:c>
-      <x:c r="G60" s="26" t="str">
-        <x:v>assets/audio/swahili/which-language-do-you-speak.mp3</x:v>
-      </x:c>
+      <x:c r="G60" s="26" t="str"/>
       <x:c r="H60" s="26"/>
       <x:c r="I60" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J60" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3383,18 +3423,20 @@
       <x:c r="B61" s="26" t="str">
         <x:v>family</x:v>
       </x:c>
-      <x:c r="C61" s="26"/>
-      <x:c r="D61" s="26"/>
+      <x:c r="C61" s="26" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="D61" s="26" t="str">
+        <x:v>fah-MEE-lee-ah</x:v>
+      </x:c>
       <x:c r="E61" s="26"/>
       <x:c r="F61" s="26" t="str">
         <x:v>assets/images/vocab/swahili/family.png</x:v>
       </x:c>
-      <x:c r="G61" s="26" t="str">
-        <x:v>assets/audio/swahili/family.mp3</x:v>
-      </x:c>
+      <x:c r="G61" s="26" t="str"/>
       <x:c r="H61" s="26"/>
       <x:c r="I61" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J61" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3407,18 +3449,20 @@
       <x:c r="B62" s="26" t="str">
         <x:v>parents</x:v>
       </x:c>
-      <x:c r="C62" s="26"/>
-      <x:c r="D62" s="26"/>
+      <x:c r="C62" s="26" t="str">
+        <x:v>Wazazi</x:v>
+      </x:c>
+      <x:c r="D62" s="26" t="str">
+        <x:v>wah-ZAH-zee</x:v>
+      </x:c>
       <x:c r="E62" s="26"/>
       <x:c r="F62" s="26" t="str">
         <x:v>assets/images/vocab/swahili/parents.png</x:v>
       </x:c>
-      <x:c r="G62" s="26" t="str">
-        <x:v>assets/audio/swahili/parents.mp3</x:v>
-      </x:c>
+      <x:c r="G62" s="26" t="str"/>
       <x:c r="H62" s="26"/>
       <x:c r="I62" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J62" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3431,18 +3475,20 @@
       <x:c r="B63" s="26" t="str">
         <x:v>husband</x:v>
       </x:c>
-      <x:c r="C63" s="26"/>
-      <x:c r="D63" s="26"/>
+      <x:c r="C63" s="26" t="str">
+        <x:v>Mume</x:v>
+      </x:c>
+      <x:c r="D63" s="26" t="str">
+        <x:v>MOO-meh</x:v>
+      </x:c>
       <x:c r="E63" s="26"/>
       <x:c r="F63" s="26" t="str">
         <x:v>assets/images/vocab/swahili/husband.png</x:v>
       </x:c>
-      <x:c r="G63" s="26" t="str">
-        <x:v>assets/audio/swahili/husband.mp3</x:v>
-      </x:c>
+      <x:c r="G63" s="26" t="str"/>
       <x:c r="H63" s="26"/>
       <x:c r="I63" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J63" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3455,18 +3501,20 @@
       <x:c r="B64" s="26" t="str">
         <x:v>wife</x:v>
       </x:c>
-      <x:c r="C64" s="26"/>
-      <x:c r="D64" s="26"/>
+      <x:c r="C64" s="26" t="str">
+        <x:v>Mke</x:v>
+      </x:c>
+      <x:c r="D64" s="26" t="str">
+        <x:v>m-KEH</x:v>
+      </x:c>
       <x:c r="E64" s="26"/>
       <x:c r="F64" s="26" t="str">
         <x:v>assets/images/vocab/swahili/wife.png</x:v>
       </x:c>
-      <x:c r="G64" s="26" t="str">
-        <x:v>assets/audio/swahili/wife.mp3</x:v>
-      </x:c>
+      <x:c r="G64" s="26" t="str"/>
       <x:c r="H64" s="26"/>
       <x:c r="I64" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J64" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3479,18 +3527,20 @@
       <x:c r="B65" s="26" t="str">
         <x:v>son</x:v>
       </x:c>
-      <x:c r="C65" s="26"/>
-      <x:c r="D65" s="26"/>
+      <x:c r="C65" s="26" t="str">
+        <x:v>Mtoto wa kiume</x:v>
+      </x:c>
+      <x:c r="D65" s="26" t="str">
+        <x:v>m-TOH-toh wah kee-OO-meh</x:v>
+      </x:c>
       <x:c r="E65" s="26"/>
       <x:c r="F65" s="26" t="str">
         <x:v>assets/images/vocab/swahili/son.png</x:v>
       </x:c>
-      <x:c r="G65" s="26" t="str">
-        <x:v>assets/audio/swahili/son.mp3</x:v>
-      </x:c>
+      <x:c r="G65" s="26" t="str"/>
       <x:c r="H65" s="26"/>
       <x:c r="I65" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J65" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3503,18 +3553,20 @@
       <x:c r="B66" s="26" t="str">
         <x:v>daughter</x:v>
       </x:c>
-      <x:c r="C66" s="26"/>
-      <x:c r="D66" s="26"/>
+      <x:c r="C66" s="26" t="str">
+        <x:v>Binti</x:v>
+      </x:c>
+      <x:c r="D66" s="26" t="str">
+        <x:v>BEEN-tee</x:v>
+      </x:c>
       <x:c r="E66" s="26"/>
       <x:c r="F66" s="26" t="str">
         <x:v>assets/images/vocab/swahili/daughter.png</x:v>
       </x:c>
-      <x:c r="G66" s="26" t="str">
-        <x:v>assets/audio/swahili/daughter.mp3</x:v>
-      </x:c>
+      <x:c r="G66" s="26" t="str"/>
       <x:c r="H66" s="26"/>
       <x:c r="I66" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J66" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3527,18 +3579,20 @@
       <x:c r="B67" s="26" t="str">
         <x:v>grandfather</x:v>
       </x:c>
-      <x:c r="C67" s="26"/>
-      <x:c r="D67" s="26"/>
+      <x:c r="C67" s="26" t="str">
+        <x:v>Babu</x:v>
+      </x:c>
+      <x:c r="D67" s="26" t="str">
+        <x:v>BAH-boo</x:v>
+      </x:c>
       <x:c r="E67" s="26"/>
       <x:c r="F67" s="26" t="str">
         <x:v>assets/images/vocab/swahili/grandfather.png</x:v>
       </x:c>
-      <x:c r="G67" s="26" t="str">
-        <x:v>assets/audio/swahili/grandfather.mp3</x:v>
-      </x:c>
+      <x:c r="G67" s="26" t="str"/>
       <x:c r="H67" s="26"/>
       <x:c r="I67" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J67" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3551,18 +3605,20 @@
       <x:c r="B68" s="26" t="str">
         <x:v>please</x:v>
       </x:c>
-      <x:c r="C68" s="26"/>
-      <x:c r="D68" s="26"/>
+      <x:c r="C68" s="26" t="str">
+        <x:v>Tafadhali</x:v>
+      </x:c>
+      <x:c r="D68" s="26" t="str">
+        <x:v>tah-fah-DHAH-lee</x:v>
+      </x:c>
       <x:c r="E68" s="26"/>
       <x:c r="F68" s="26" t="str">
         <x:v>assets/images/vocab/swahili/please.png</x:v>
       </x:c>
-      <x:c r="G68" s="26" t="str">
-        <x:v>assets/audio/swahili/please.mp3</x:v>
-      </x:c>
+      <x:c r="G68" s="26" t="str"/>
       <x:c r="H68" s="26"/>
       <x:c r="I68" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J68" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3575,18 +3631,20 @@
       <x:c r="B69" s="26" t="str">
         <x:v>thank-you</x:v>
       </x:c>
-      <x:c r="C69" s="26"/>
-      <x:c r="D69" s="26"/>
+      <x:c r="C69" s="26" t="str">
+        <x:v>Asante</x:v>
+      </x:c>
+      <x:c r="D69" s="26" t="str">
+        <x:v>ah-SAHN-teh</x:v>
+      </x:c>
       <x:c r="E69" s="26"/>
       <x:c r="F69" s="26" t="str">
         <x:v>assets/images/vocab/swahili/thank-you.png</x:v>
       </x:c>
-      <x:c r="G69" s="26" t="str">
-        <x:v>assets/audio/swahili/thank-you.mp3</x:v>
-      </x:c>
+      <x:c r="G69" s="26" t="str"/>
       <x:c r="H69" s="26"/>
       <x:c r="I69" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J69" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3599,18 +3657,20 @@
       <x:c r="B70" s="26" t="str">
         <x:v>no-problem</x:v>
       </x:c>
-      <x:c r="C70" s="26"/>
-      <x:c r="D70" s="26"/>
+      <x:c r="C70" s="26" t="str">
+        <x:v>Hakuna shida</x:v>
+      </x:c>
+      <x:c r="D70" s="26" t="str">
+        <x:v>hah-KOO-nah SHEE-dah</x:v>
+      </x:c>
       <x:c r="E70" s="26"/>
       <x:c r="F70" s="26" t="str">
         <x:v>assets/images/vocab/swahili/no-problem.png</x:v>
       </x:c>
-      <x:c r="G70" s="26" t="str">
-        <x:v>assets/audio/swahili/no-problem.mp3</x:v>
-      </x:c>
+      <x:c r="G70" s="26" t="str"/>
       <x:c r="H70" s="26"/>
       <x:c r="I70" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J70" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3623,18 +3683,20 @@
       <x:c r="B71" s="26" t="str">
         <x:v>excuse-me</x:v>
       </x:c>
-      <x:c r="C71" s="26"/>
-      <x:c r="D71" s="26"/>
+      <x:c r="C71" s="26" t="str">
+        <x:v>Niwie radhi</x:v>
+      </x:c>
+      <x:c r="D71" s="26" t="str">
+        <x:v>nee-WEE-eh RAH-dhee</x:v>
+      </x:c>
       <x:c r="E71" s="26"/>
       <x:c r="F71" s="26" t="str">
         <x:v>assets/images/vocab/swahili/excuse-me.png</x:v>
       </x:c>
-      <x:c r="G71" s="26" t="str">
-        <x:v>assets/audio/swahili/excuse-me.mp3</x:v>
-      </x:c>
+      <x:c r="G71" s="26" t="str"/>
       <x:c r="H71" s="26"/>
       <x:c r="I71" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J71" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3647,18 +3709,20 @@
       <x:c r="B72" s="26" t="str">
         <x:v>sorry</x:v>
       </x:c>
-      <x:c r="C72" s="26"/>
-      <x:c r="D72" s="26"/>
+      <x:c r="C72" s="26" t="str">
+        <x:v>Samahani</x:v>
+      </x:c>
+      <x:c r="D72" s="26" t="str">
+        <x:v>sah-mah-HAH-nee</x:v>
+      </x:c>
       <x:c r="E72" s="26"/>
       <x:c r="F72" s="26" t="str">
         <x:v>assets/images/vocab/swahili/sorry.png</x:v>
       </x:c>
-      <x:c r="G72" s="26" t="str">
-        <x:v>assets/audio/swahili/sorry.mp3</x:v>
-      </x:c>
+      <x:c r="G72" s="26" t="str"/>
       <x:c r="H72" s="26"/>
       <x:c r="I72" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J72" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3671,18 +3735,20 @@
       <x:c r="B73" s="26" t="str">
         <x:v>this-is-my-family</x:v>
       </x:c>
-      <x:c r="C73" s="26"/>
-      <x:c r="D73" s="26"/>
+      <x:c r="C73" s="26" t="str">
+        <x:v>Hii ni familia yangu</x:v>
+      </x:c>
+      <x:c r="D73" s="26" t="str">
+        <x:v>HEE nee fah-MEE-lee-ah YAH-ngoo</x:v>
+      </x:c>
       <x:c r="E73" s="26"/>
       <x:c r="F73" s="26" t="str">
         <x:v>assets/images/vocab/swahili/this-is-my-family.png</x:v>
       </x:c>
-      <x:c r="G73" s="26" t="str">
-        <x:v>assets/audio/swahili/this-is-my-family.mp3</x:v>
-      </x:c>
+      <x:c r="G73" s="26" t="str"/>
       <x:c r="H73" s="26"/>
       <x:c r="I73" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J73" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3695,18 +3761,20 @@
       <x:c r="B74" s="26" t="str">
         <x:v>this-is-my-husband</x:v>
       </x:c>
-      <x:c r="C74" s="26"/>
-      <x:c r="D74" s="26"/>
+      <x:c r="C74" s="26" t="str">
+        <x:v>Huyu ni mume wangu</x:v>
+      </x:c>
+      <x:c r="D74" s="26" t="str">
+        <x:v>HOO-yoo nee MOO-meh WAH-ngoo</x:v>
+      </x:c>
       <x:c r="E74" s="26"/>
       <x:c r="F74" s="26" t="str">
         <x:v>assets/images/vocab/swahili/this-is-my-husband.png</x:v>
       </x:c>
-      <x:c r="G74" s="26" t="str">
-        <x:v>assets/audio/swahili/this-is-my-husband.mp3</x:v>
-      </x:c>
+      <x:c r="G74" s="26" t="str"/>
       <x:c r="H74" s="26"/>
       <x:c r="I74" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J74" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3719,18 +3787,20 @@
       <x:c r="B75" s="26" t="str">
         <x:v>this-is-my-wife</x:v>
       </x:c>
-      <x:c r="C75" s="26"/>
-      <x:c r="D75" s="26"/>
+      <x:c r="C75" s="26" t="str">
+        <x:v>Huyu ni mke wangu</x:v>
+      </x:c>
+      <x:c r="D75" s="26" t="str">
+        <x:v>HOO-yoo nee m-KEH WAH-ngoo</x:v>
+      </x:c>
       <x:c r="E75" s="26"/>
       <x:c r="F75" s="26" t="str">
         <x:v>assets/images/vocab/swahili/this-is-my-wife.png</x:v>
       </x:c>
-      <x:c r="G75" s="26" t="str">
-        <x:v>assets/audio/swahili/this-is-my-wife.mp3</x:v>
-      </x:c>
+      <x:c r="G75" s="26" t="str"/>
       <x:c r="H75" s="26"/>
       <x:c r="I75" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J75" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3743,18 +3813,20 @@
       <x:c r="B76" s="26" t="str">
         <x:v>he-lives-here</x:v>
       </x:c>
-      <x:c r="C76" s="26"/>
-      <x:c r="D76" s="26"/>
+      <x:c r="C76" s="26" t="str">
+        <x:v>Anaishi hapa</x:v>
+      </x:c>
+      <x:c r="D76" s="26" t="str">
+        <x:v>ah-nah-EE-shee HAH-pah</x:v>
+      </x:c>
       <x:c r="E76" s="26"/>
       <x:c r="F76" s="26" t="str">
         <x:v>assets/images/vocab/swahili/he-lives-here.png</x:v>
       </x:c>
-      <x:c r="G76" s="26" t="str">
-        <x:v>assets/audio/swahili/he-lives-here.mp3</x:v>
-      </x:c>
+      <x:c r="G76" s="26" t="str"/>
       <x:c r="H76" s="26"/>
       <x:c r="I76" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J76" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3767,18 +3839,20 @@
       <x:c r="B77" s="26" t="str">
         <x:v>she-works-here</x:v>
       </x:c>
-      <x:c r="C77" s="26"/>
-      <x:c r="D77" s="26"/>
+      <x:c r="C77" s="26" t="str">
+        <x:v>Anafanya kazi hapa</x:v>
+      </x:c>
+      <x:c r="D77" s="26" t="str">
+        <x:v>ah-nah-FAHN-yah KAH-zee HAH-pah</x:v>
+      </x:c>
       <x:c r="E77" s="26"/>
       <x:c r="F77" s="26" t="str">
         <x:v>assets/images/vocab/swahili/she-works-here.png</x:v>
       </x:c>
-      <x:c r="G77" s="26" t="str">
-        <x:v>assets/audio/swahili/she-works-here.mp3</x:v>
-      </x:c>
+      <x:c r="G77" s="26" t="str"/>
       <x:c r="H77" s="26"/>
       <x:c r="I77" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J77" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3791,18 +3865,20 @@
       <x:c r="B78" s="26" t="str">
         <x:v>we-speak</x:v>
       </x:c>
-      <x:c r="C78" s="26"/>
-      <x:c r="D78" s="26"/>
+      <x:c r="C78" s="26" t="str">
+        <x:v>Tunazungumza...</x:v>
+      </x:c>
+      <x:c r="D78" s="26" t="str">
+        <x:v>too-nah-zoon-GOOM-zah</x:v>
+      </x:c>
       <x:c r="E78" s="26"/>
       <x:c r="F78" s="26" t="str">
         <x:v>assets/images/vocab/swahili/we-speak.png</x:v>
       </x:c>
-      <x:c r="G78" s="26" t="str">
-        <x:v>assets/audio/swahili/we-speak.mp3</x:v>
-      </x:c>
+      <x:c r="G78" s="26" t="str"/>
       <x:c r="H78" s="26"/>
       <x:c r="I78" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J78" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -3815,18 +3891,20 @@
       <x:c r="B79" s="26" t="str">
         <x:v>they-are-from</x:v>
       </x:c>
-      <x:c r="C79" s="26"/>
-      <x:c r="D79" s="26"/>
+      <x:c r="C79" s="26" t="str">
+        <x:v>Wanatoka...</x:v>
+      </x:c>
+      <x:c r="D79" s="26" t="str">
+        <x:v>wah-nah-TOH-kah</x:v>
+      </x:c>
       <x:c r="E79" s="26"/>
       <x:c r="F79" s="26" t="str">
         <x:v>assets/images/vocab/swahili/they-are-from.png</x:v>
       </x:c>
-      <x:c r="G79" s="26" t="str">
-        <x:v>assets/audio/swahili/they-are-from.mp3</x:v>
-      </x:c>
+      <x:c r="G79" s="26" t="str"/>
       <x:c r="H79" s="26"/>
       <x:c r="I79" s="26" t="str">
-        <x:v>backlog</x:v>
+        <x:v>needs-native-review</x:v>
       </x:c>
       <x:c r="J79" s="26" t="str">
         <x:v>unavailable</x:v>
@@ -10395,7 +10473,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a7603189e8f44b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f7730052e424de6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10646,7 +10724,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa75ce2ff5c84efb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R899310f50cac4503"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12553,7 +12631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66b9c82e8e164a54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af8ef0876a34a01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15224,10 +15302,2488 @@
         <x:v>preview</x:v>
       </x:c>
     </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>swahili-getting-started-01-yes</x:v>
+      </x:c>
+      <x:c r="D66" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>What does "Ndiyo" mean?</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>["no","okay","maybe"]</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>["yes"]</x:v>
+      </x:c>
+      <x:c r="K66" t="str"/>
+      <x:c r="L66" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M66" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>swahili-getting-started-02-no</x:v>
+      </x:c>
+      <x:c r="D67" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>Build the Swahili phrase for "no".</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>Hapana</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>["Labda","Tena","Sawa"]</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>["no"]</x:v>
+      </x:c>
+      <x:c r="K67" t="str"/>
+      <x:c r="L67" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>swahili-getting-started-03-match</x:v>
+      </x:c>
+      <x:c r="D68" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I68"/>
+      <x:c r="J68" t="str">
+        <x:v>["yes","no","maybe","okay"]</x:v>
+      </x:c>
+      <x:c r="K68" t="str"/>
+      <x:c r="L68" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>swahili-getting-started-04-maybe</x:v>
+      </x:c>
+      <x:c r="D69" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>Build the English meaning of "Labda".</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>maybe</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>["yes","okay","no"]</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>maybe</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>["maybe"]</x:v>
+      </x:c>
+      <x:c r="K69" t="str"/>
+      <x:c r="L69" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>swahili-getting-started-05-okay</x:v>
+      </x:c>
+      <x:c r="D70" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>Choose the Swahili for "okay".</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Sawa</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>["Hapana","Tena","Labda"]</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>okay</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>["okay"]</x:v>
+      </x:c>
+      <x:c r="K70" t="str"/>
+      <x:c r="L70" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>getting-started</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>swahili-getting-started-06-again</x:v>
+      </x:c>
+      <x:c r="D71" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>again</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>["yes","okay","maybe"]</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>again</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>["again"]</x:v>
+      </x:c>
+      <x:c r="K71" t="str"/>
+      <x:c r="L71" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>swahili-easy-greetings-01-good-afternoon</x:v>
+      </x:c>
+      <x:c r="D72" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>What does "Habari ya mchana" mean?</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>good afternoon</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>["nice to meet you","have a good day","how is your day"]</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>good-afternoon</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>["good-afternoon"]</x:v>
+      </x:c>
+      <x:c r="K72" t="str"/>
+      <x:c r="L72" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>swahili-easy-greetings-02-nice-to-meet-you</x:v>
+      </x:c>
+      <x:c r="D73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>Build the Swahili phrase for "nice to meet you".</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Nimefurahi kukutana nawe</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>["Siku yako inaendeleaje?","Uwe na siku njema","Habari ya mchana"]</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>nice-to-meet-you</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>["nice-to-meet-you"]</x:v>
+      </x:c>
+      <x:c r="K73" t="str"/>
+      <x:c r="L73" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>swahili-easy-greetings-03-match</x:v>
+      </x:c>
+      <x:c r="D74" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I74"/>
+      <x:c r="J74" t="str">
+        <x:v>["good-afternoon","nice-to-meet-you","long-time-no-see","how-is-your-day"]</x:v>
+      </x:c>
+      <x:c r="K74" t="str"/>
+      <x:c r="L74" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>swahili-easy-greetings-04-long-time-no-see</x:v>
+      </x:c>
+      <x:c r="D75" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>Build the English meaning of "Hatujaonana kwa muda mrefu".</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>long time no see</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>["how is your day","have a good day","nice to meet you"]</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>long-time-no-see</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>["long-time-no-see"]</x:v>
+      </x:c>
+      <x:c r="K75" t="str"/>
+      <x:c r="L75" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>swahili-easy-greetings-05-how-is-your-day</x:v>
+      </x:c>
+      <x:c r="D76" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Choose the Swahili for "how is your day".</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>Siku yako inaendeleaje?</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>["Habari ya mchana","Hatujaonana kwa muda mrefu","Uwe na siku njema"]</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>how-is-your-day</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>["how-is-your-day"]</x:v>
+      </x:c>
+      <x:c r="K76" t="str"/>
+      <x:c r="L76" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>easy-greetings</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>swahili-easy-greetings-06-have-a-good-day</x:v>
+      </x:c>
+      <x:c r="D77" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>have a good day</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>["good afternoon","nice to meet you","long time no see"]</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>have-a-good-day</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>["have-a-good-day"]</x:v>
+      </x:c>
+      <x:c r="K77" t="str"/>
+      <x:c r="L77" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>swahili-introducing-yourself-01-what-is-your-name</x:v>
+      </x:c>
+      <x:c r="D78" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>What does "Jina lako ni nani?" mean?</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>what is your name</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>["my name is...","I am a student","I am learning..."]</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>what-is-your-name</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>["what-is-your-name"]</x:v>
+      </x:c>
+      <x:c r="K78" t="str"/>
+      <x:c r="L78" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M78" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>swahili-introducing-yourself-02-my-name-is</x:v>
+      </x:c>
+      <x:c r="D79" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Build the Swahili phrase for "my name is...".</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>Jina langu ni...</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>["Mimi ni mwanafunzi","Ninazungumza...","Ninajifunza..."]</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>my-name-is</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>["my-name-is"]</x:v>
+      </x:c>
+      <x:c r="K79" t="str"/>
+      <x:c r="L79" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>swahili-introducing-yourself-03-match</x:v>
+      </x:c>
+      <x:c r="D80" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I80"/>
+      <x:c r="J80" t="str">
+        <x:v>["what-is-your-name","my-name-is","i-am-a-student","i-am-learning"]</x:v>
+      </x:c>
+      <x:c r="K80" t="str"/>
+      <x:c r="L80" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>swahili-introducing-yourself-04-i-am-a-student</x:v>
+      </x:c>
+      <x:c r="D81" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Build the English meaning of "Mimi ni mwanafunzi".</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>I am a student</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>["what is your name","I am learning...","my name is..."]</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>i-am-a-student</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>["i-am-a-student"]</x:v>
+      </x:c>
+      <x:c r="K81" t="str"/>
+      <x:c r="L81" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>swahili-introducing-yourself-05-i-am-learning</x:v>
+      </x:c>
+      <x:c r="D82" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Choose the Swahili for "I am learning...".</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>Ninajifunza...</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>["Jina lako ni nani?","Mimi ni mwanafunzi","Ninazungumza..."]</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>i-am-learning</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>["i-am-learning"]</x:v>
+      </x:c>
+      <x:c r="K82" t="str"/>
+      <x:c r="L82" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M82" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>introducing-yourself</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>swahili-introducing-yourself-06-i-speak</x:v>
+      </x:c>
+      <x:c r="D83" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>I speak...</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>["what is your name","I am a student","my name is..."]</x:v>
+      </x:c>
+      <x:c r="I83" t="str">
+        <x:v>i-speak</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>["i-speak"]</x:v>
+      </x:c>
+      <x:c r="K83" t="str"/>
+      <x:c r="L83" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M83" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>swahili-your-background-01-where-are-you-from</x:v>
+      </x:c>
+      <x:c r="D84" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>What does "Unatoka wapi?" mean?</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>where are you from</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>["I am from...","where do you live","I live in..."]</x:v>
+      </x:c>
+      <x:c r="I84" t="str">
+        <x:v>where-are-you-from</x:v>
+      </x:c>
+      <x:c r="J84" t="str">
+        <x:v>["where-are-you-from"]</x:v>
+      </x:c>
+      <x:c r="K84" t="str"/>
+      <x:c r="L84" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M84" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>swahili-your-background-02-i-am-from</x:v>
+      </x:c>
+      <x:c r="D85" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Build the Swahili phrase for "I am from...".</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Ninatoka...</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>["Unaishi wapi?","Unazungumza lugha gani?","Ninaishi..."]</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>i-am-from</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>["i-am-from"]</x:v>
+      </x:c>
+      <x:c r="K85" t="str"/>
+      <x:c r="L85" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M85" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>swahili-your-background-03-match</x:v>
+      </x:c>
+      <x:c r="D86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I86"/>
+      <x:c r="J86" t="str">
+        <x:v>["where-are-you-from","i-am-from","where-do-you-live","i-live-in"]</x:v>
+      </x:c>
+      <x:c r="K86" t="str"/>
+      <x:c r="L86" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>swahili-your-background-04-where-do-you-live</x:v>
+      </x:c>
+      <x:c r="D87" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Build the English meaning of "Unaishi wapi?".</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>where do you live</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>["where are you from","I live in...","I am from..."]</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>where-do-you-live</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>["where-do-you-live"]</x:v>
+      </x:c>
+      <x:c r="K87" t="str"/>
+      <x:c r="L87" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M87" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>swahili-your-background-05-i-live-in</x:v>
+      </x:c>
+      <x:c r="D88" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Choose the Swahili for "I live in...".</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Ninaishi...</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>["Ninatoka...","Unazungumza lugha gani?","Unatoka wapi?"]</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>i-live-in</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>["i-live-in"]</x:v>
+      </x:c>
+      <x:c r="K88" t="str"/>
+      <x:c r="L88" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>your-background</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>swahili-your-background-06-which-language-do-you-speak</x:v>
+      </x:c>
+      <x:c r="D89" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>which language do you speak</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>["where do you live","I live in...","I am from..."]</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>which-language-do-you-speak</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>["which-language-do-you-speak"]</x:v>
+      </x:c>
+      <x:c r="K89" t="str"/>
+      <x:c r="L89" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M89" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>swahili-family-members-01-family</x:v>
+      </x:c>
+      <x:c r="D90" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>What does "Familia" mean?</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>family</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>["husband","daughter","wife"]</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>family</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>["family"]</x:v>
+      </x:c>
+      <x:c r="K90" t="str"/>
+      <x:c r="L90" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>swahili-family-members-02-parents</x:v>
+      </x:c>
+      <x:c r="D91" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Build the Swahili phrase for "parents".</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Wazazi</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>["Mume","Binti","Mtoto wa kiume"]</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>parents</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>["parents"]</x:v>
+      </x:c>
+      <x:c r="K91" t="str"/>
+      <x:c r="L91" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>swahili-family-members-03-match</x:v>
+      </x:c>
+      <x:c r="D92" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I92"/>
+      <x:c r="J92" t="str">
+        <x:v>["family","parents","husband","wife"]</x:v>
+      </x:c>
+      <x:c r="K92" t="str"/>
+      <x:c r="L92" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>swahili-family-members-04-husband</x:v>
+      </x:c>
+      <x:c r="D93" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Build the English meaning of "Mume".</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>husband</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>["parents","wife","daughter"]</x:v>
+      </x:c>
+      <x:c r="I93" t="str">
+        <x:v>husband</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>["husband"]</x:v>
+      </x:c>
+      <x:c r="K93" t="str"/>
+      <x:c r="L93" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M93" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>swahili-family-members-05-wife</x:v>
+      </x:c>
+      <x:c r="D94" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Choose the Swahili for "wife".</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Mke</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>["Familia","Mtoto wa kiume","Binti"]</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>wife</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>["wife"]</x:v>
+      </x:c>
+      <x:c r="K94" t="str"/>
+      <x:c r="L94" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M94" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>swahili-family-members-06-son</x:v>
+      </x:c>
+      <x:c r="D95" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>son</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>["family","daughter","husband"]</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>son</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>["son"]</x:v>
+      </x:c>
+      <x:c r="K95" t="str"/>
+      <x:c r="L95" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>swahili-family-members-07-daughter</x:v>
+      </x:c>
+      <x:c r="D96" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Choose the Swahili for "daughter".</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Binti</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>["Babu","Mtoto wa kiume","Wazazi"]</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>daughter</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>["daughter"]</x:v>
+      </x:c>
+      <x:c r="K96" t="str"/>
+      <x:c r="L96" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M96" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>family-members</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>swahili-family-members-08-grandfather</x:v>
+      </x:c>
+      <x:c r="D97" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Choose the Swahili for "grandfather".</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Babu</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>["Mume","Mtoto wa kiume","Familia"]</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>grandfather</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>["grandfather"]</x:v>
+      </x:c>
+      <x:c r="K97" t="str"/>
+      <x:c r="L97" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M97" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>swahili-polite-conversation-01-please</x:v>
+      </x:c>
+      <x:c r="D98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>What does "Tafadhali" mean?</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>please</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>["thank you","sorry","excuse me"]</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>please</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>["please"]</x:v>
+      </x:c>
+      <x:c r="K98" t="str"/>
+      <x:c r="L98" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M98" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>swahili-polite-conversation-02-thank-you</x:v>
+      </x:c>
+      <x:c r="D99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>Build the Swahili phrase for "thank you".</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Asante</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>["Hakuna shida","Tafadhali","Samahani"]</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>thank-you</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>["thank-you"]</x:v>
+      </x:c>
+      <x:c r="K99" t="str"/>
+      <x:c r="L99" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M99" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>swahili-polite-conversation-03-match</x:v>
+      </x:c>
+      <x:c r="D100" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I100"/>
+      <x:c r="J100" t="str">
+        <x:v>["please","thank-you","no-problem","excuse-me"]</x:v>
+      </x:c>
+      <x:c r="K100" t="str"/>
+      <x:c r="L100" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>swahili-polite-conversation-04-no-problem</x:v>
+      </x:c>
+      <x:c r="D101" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Build the English meaning of "Hakuna shida".</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>no problem</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>["please","excuse me","thank you"]</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>no-problem</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>["no-problem"]</x:v>
+      </x:c>
+      <x:c r="K101" t="str"/>
+      <x:c r="L101" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M101" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>swahili-polite-conversation-05-excuse-me</x:v>
+      </x:c>
+      <x:c r="D102" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Choose the Swahili for "excuse me".</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Niwie radhi</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>["Tafadhali","Hakuna shida","Samahani"]</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>excuse-me</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>["excuse-me"]</x:v>
+      </x:c>
+      <x:c r="K102" t="str"/>
+      <x:c r="L102" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M102" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>polite-conversation</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>swahili-polite-conversation-06-sorry</x:v>
+      </x:c>
+      <x:c r="D103" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>sorry</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>["please","excuse me","no problem"]</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>sorry</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>["sorry"]</x:v>
+      </x:c>
+      <x:c r="K103" t="str"/>
+      <x:c r="L103" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M103" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>swahili-introducing-others-01-this-is-my-family</x:v>
+      </x:c>
+      <x:c r="D104" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>What does "Hii ni familia yangu" mean?</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>this is my family</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>["this is my husband","he lives here","we speak..."]</x:v>
+      </x:c>
+      <x:c r="I104" t="str">
+        <x:v>this-is-my-family</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>["this-is-my-family"]</x:v>
+      </x:c>
+      <x:c r="K104" t="str"/>
+      <x:c r="L104" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M104" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>swahili-introducing-others-02-this-is-my-husband</x:v>
+      </x:c>
+      <x:c r="D105" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>Build the Swahili phrase for "this is my husband".</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Huyu ni mume wangu</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>["Tunazungumza...","Wanatoka...","Anaishi hapa"]</x:v>
+      </x:c>
+      <x:c r="I105" t="str">
+        <x:v>this-is-my-husband</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>["this-is-my-husband"]</x:v>
+      </x:c>
+      <x:c r="K105" t="str"/>
+      <x:c r="L105" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M105" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>swahili-introducing-others-03-match</x:v>
+      </x:c>
+      <x:c r="D106" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I106"/>
+      <x:c r="J106" t="str">
+        <x:v>["this-is-my-family","this-is-my-husband","this-is-my-wife","he-lives-here"]</x:v>
+      </x:c>
+      <x:c r="K106" t="str"/>
+      <x:c r="L106" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M106" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>swahili-introducing-others-04-this-is-my-wife</x:v>
+      </x:c>
+      <x:c r="D107" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Build the English meaning of "Huyu ni mke wangu".</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>this is my wife</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>["this is my family","he lives here","we speak..."]</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>this-is-my-wife</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>["this-is-my-wife"]</x:v>
+      </x:c>
+      <x:c r="K107" t="str"/>
+      <x:c r="L107" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>swahili-introducing-others-05-he-lives-here</x:v>
+      </x:c>
+      <x:c r="D108" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Choose the Swahili for "he lives here".</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Anaishi hapa</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>["Huyu ni mume wangu","Huyu ni mke wangu","Anafanya kazi hapa"]</x:v>
+      </x:c>
+      <x:c r="I108" t="str">
+        <x:v>he-lives-here</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>["he-lives-here"]</x:v>
+      </x:c>
+      <x:c r="K108" t="str"/>
+      <x:c r="L108" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M108" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>swahili-introducing-others-06-she-works-here</x:v>
+      </x:c>
+      <x:c r="D109" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>she works here</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>["this is my family","they are from...","we speak..."]</x:v>
+      </x:c>
+      <x:c r="I109" t="str">
+        <x:v>she-works-here</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>["she-works-here"]</x:v>
+      </x:c>
+      <x:c r="K109" t="str"/>
+      <x:c r="L109" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M109" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>swahili-introducing-others-07-we-speak</x:v>
+      </x:c>
+      <x:c r="D110" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>Choose the Swahili for "we speak...".</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>Tunazungumza...</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>["Huyu ni mke wangu","Anaishi hapa","Anafanya kazi hapa"]</x:v>
+      </x:c>
+      <x:c r="I110" t="str">
+        <x:v>we-speak</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>["we-speak"]</x:v>
+      </x:c>
+      <x:c r="K110" t="str"/>
+      <x:c r="L110" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M110" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>introducing-others</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>swahili-introducing-others-08-they-are-from</x:v>
+      </x:c>
+      <x:c r="D111" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>Choose the Swahili for "they are from...".</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>Wanatoka...</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>["Huyu ni mke wangu","Huyu ni mume wangu","Hii ni familia yangu"]</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>they-are-from</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>["they-are-from"]</x:v>
+      </x:c>
+      <x:c r="K111" t="str"/>
+      <x:c r="L111" s="28" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M111" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>swahili-words-practice-01-yes</x:v>
+      </x:c>
+      <x:c r="D112" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>What does "Ndiyo" mean?</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>["where are you from","excuse me","good afternoon"]</x:v>
+      </x:c>
+      <x:c r="I112" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>["yes"]</x:v>
+      </x:c>
+      <x:c r="K112" t="str"/>
+      <x:c r="L112" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M112" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>swahili-words-practice-02-good-afternoon</x:v>
+      </x:c>
+      <x:c r="D113" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>Build the Swahili phrase for "good afternoon".</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>Habari ya mchana</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>["Anaishi hapa","Familia","Unatoka wapi?"]</x:v>
+      </x:c>
+      <x:c r="I113" t="str">
+        <x:v>good-afternoon</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>["good-afternoon"]</x:v>
+      </x:c>
+      <x:c r="K113" t="str"/>
+      <x:c r="L113" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M113" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>swahili-words-practice-03-match</x:v>
+      </x:c>
+      <x:c r="D114" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H114" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I114"/>
+      <x:c r="J114" t="str">
+        <x:v>["yes","good-afternoon","what-is-your-name","where-are-you-from"]</x:v>
+      </x:c>
+      <x:c r="K114" t="str"/>
+      <x:c r="L114" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M114" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>swahili-words-practice-04-what-is-your-name</x:v>
+      </x:c>
+      <x:c r="D115" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>Build the English meaning of "Jina lako ni nani?".</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>what is your name</x:v>
+      </x:c>
+      <x:c r="H115" t="str">
+        <x:v>["where are you from","family","good afternoon"]</x:v>
+      </x:c>
+      <x:c r="I115" t="str">
+        <x:v>what-is-your-name</x:v>
+      </x:c>
+      <x:c r="J115" t="str">
+        <x:v>["what-is-your-name"]</x:v>
+      </x:c>
+      <x:c r="K115" t="str"/>
+      <x:c r="L115" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M115" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>swahili-words-practice-05-where-are-you-from</x:v>
+      </x:c>
+      <x:c r="D116" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>Choose the Swahili for "where are you from".</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>Unatoka wapi?</x:v>
+      </x:c>
+      <x:c r="H116" t="str">
+        <x:v>["Anaishi hapa","Binti","Jina lako ni nani?"]</x:v>
+      </x:c>
+      <x:c r="I116" t="str">
+        <x:v>where-are-you-from</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>["where-are-you-from"]</x:v>
+      </x:c>
+      <x:c r="K116" t="str"/>
+      <x:c r="L116" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M116" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>swahili-words-practice-06-family</x:v>
+      </x:c>
+      <x:c r="D117" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>family</x:v>
+      </x:c>
+      <x:c r="H117" t="str">
+        <x:v>["what is your name","good afternoon","yes"]</x:v>
+      </x:c>
+      <x:c r="I117" t="str">
+        <x:v>family</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>["family"]</x:v>
+      </x:c>
+      <x:c r="K117" t="str"/>
+      <x:c r="L117" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M117" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>swahili-words-practice-07-daughter</x:v>
+      </x:c>
+      <x:c r="D118" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>Choose the Swahili for "daughter".</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>Binti</x:v>
+      </x:c>
+      <x:c r="H118" t="str">
+        <x:v>["Anaishi hapa","Jina lako ni nani?","Familia"]</x:v>
+      </x:c>
+      <x:c r="I118" t="str">
+        <x:v>daughter</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>["daughter"]</x:v>
+      </x:c>
+      <x:c r="K118" t="str"/>
+      <x:c r="L118" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M118" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>swahili-words-practice-08-excuse-me</x:v>
+      </x:c>
+      <x:c r="D119" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>What does "Niwie radhi" mean?</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>excuse me</x:v>
+      </x:c>
+      <x:c r="H119" t="str">
+        <x:v>["yes","what is your name","he lives here"]</x:v>
+      </x:c>
+      <x:c r="I119" t="str">
+        <x:v>excuse-me</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>["excuse-me"]</x:v>
+      </x:c>
+      <x:c r="K119" t="str"/>
+      <x:c r="L119" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M119" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>words-practice</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>swahili-words-practice-09-he-lives-here</x:v>
+      </x:c>
+      <x:c r="D120" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>Choose the Swahili for "he lives here".</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>Anaishi hapa</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>["Niwie radhi","Ndiyo","Habari ya mchana"]</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>he-lives-here</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>["he-lives-here"]</x:v>
+      </x:c>
+      <x:c r="K120" t="str"/>
+      <x:c r="L120" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>swahili-practice-challenge-01-no</x:v>
+      </x:c>
+      <x:c r="D121" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>What does "Hapana" mean?</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="H121" t="str">
+        <x:v>["I am learning...","parents","no problem"]</x:v>
+      </x:c>
+      <x:c r="I121" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>["no"]</x:v>
+      </x:c>
+      <x:c r="K121" t="str"/>
+      <x:c r="L121" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M121" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>swahili-practice-challenge-02-good-afternoon</x:v>
+      </x:c>
+      <x:c r="D122" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>sentence-build-target</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>Build the Swahili phrase for "good afternoon".</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>Habari ya mchana</x:v>
+      </x:c>
+      <x:c r="H122" t="str">
+        <x:v>["Hapana","Wazazi","Unaishi wapi?"]</x:v>
+      </x:c>
+      <x:c r="I122" t="str">
+        <x:v>good-afternoon</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>["good-afternoon"]</x:v>
+      </x:c>
+      <x:c r="K122" t="str"/>
+      <x:c r="L122" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M122" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>swahili-practice-challenge-03-match</x:v>
+      </x:c>
+      <x:c r="D123" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>match-pairs</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>Match each Swahili phrase to its English meaning.</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>__matched__</x:v>
+      </x:c>
+      <x:c r="H123" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="I123"/>
+      <x:c r="J123" t="str">
+        <x:v>["no","good-afternoon","have-a-good-day","i-am-learning"]</x:v>
+      </x:c>
+      <x:c r="K123" t="str"/>
+      <x:c r="L123" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M123" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>swahili-practice-challenge-04-have-a-good-day</x:v>
+      </x:c>
+      <x:c r="D124" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>word-tray-meaning</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Build the English meaning of "Uwe na siku njema".</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>have a good day</x:v>
+      </x:c>
+      <x:c r="H124" t="str">
+        <x:v>["daughter","no problem","good afternoon"]</x:v>
+      </x:c>
+      <x:c r="I124" t="str">
+        <x:v>have-a-good-day</x:v>
+      </x:c>
+      <x:c r="J124" t="str">
+        <x:v>["have-a-good-day"]</x:v>
+      </x:c>
+      <x:c r="K124" t="str"/>
+      <x:c r="L124" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M124" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>swahili-practice-challenge-05-i-am-learning</x:v>
+      </x:c>
+      <x:c r="D125" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>Choose the Swahili for "I am learning...".</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>Ninajifunza...</x:v>
+      </x:c>
+      <x:c r="H125" t="str">
+        <x:v>["Wazazi","Uwe na siku njema","Hakuna shida"]</x:v>
+      </x:c>
+      <x:c r="I125" t="str">
+        <x:v>i-am-learning</x:v>
+      </x:c>
+      <x:c r="J125" t="str">
+        <x:v>["i-am-learning"]</x:v>
+      </x:c>
+      <x:c r="K125" t="str"/>
+      <x:c r="L125" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M125" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>swahili-practice-challenge-06-where-do-you-live</x:v>
+      </x:c>
+      <x:c r="D126" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>listen-choice</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>Listen, then choose the English meaning.</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>where do you live</x:v>
+      </x:c>
+      <x:c r="H126" t="str">
+        <x:v>["no","parents","I am learning..."]</x:v>
+      </x:c>
+      <x:c r="I126" t="str">
+        <x:v>where-do-you-live</x:v>
+      </x:c>
+      <x:c r="J126" t="str">
+        <x:v>["where-do-you-live"]</x:v>
+      </x:c>
+      <x:c r="K126" t="str"/>
+      <x:c r="L126" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M126" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>swahili-practice-challenge-07-parents</x:v>
+      </x:c>
+      <x:c r="D127" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>Choose the Swahili for "parents".</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>Wazazi</x:v>
+      </x:c>
+      <x:c r="H127" t="str">
+        <x:v>["Uwe na siku njema","Habari ya mchana","Hapana"]</x:v>
+      </x:c>
+      <x:c r="I127" t="str">
+        <x:v>parents</x:v>
+      </x:c>
+      <x:c r="J127" t="str">
+        <x:v>["parents"]</x:v>
+      </x:c>
+      <x:c r="K127" t="str"/>
+      <x:c r="L127" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M127" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>swahili-practice-challenge-08-daughter</x:v>
+      </x:c>
+      <x:c r="D128" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>translate-to-meaning</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>What does "Binti" mean?</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>daughter</x:v>
+      </x:c>
+      <x:c r="H128" t="str">
+        <x:v>["no","I am learning...","have a good day"]</x:v>
+      </x:c>
+      <x:c r="I128" t="str">
+        <x:v>daughter</x:v>
+      </x:c>
+      <x:c r="J128" t="str">
+        <x:v>["daughter"]</x:v>
+      </x:c>
+      <x:c r="K128" t="str"/>
+      <x:c r="L128" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M128" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>swahili</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>practice-challenge</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>swahili-practice-challenge-09-no-problem</x:v>
+      </x:c>
+      <x:c r="D129" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>translate-to-target</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>Choose the Swahili for "no problem".</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>Hakuna shida</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>["Unaishi wapi?","Habari ya mchana","Hapana"]</x:v>
+      </x:c>
+      <x:c r="I129" t="str">
+        <x:v>no-problem</x:v>
+      </x:c>
+      <x:c r="J129" t="str">
+        <x:v>["no-problem"]</x:v>
+      </x:c>
+      <x:c r="K129" t="str"/>
+      <x:c r="L129" s="28" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M129" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4ab0b5184f4bcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7ebce0e23a4b4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Stage Haitian Creole candidate course artwork
</commit_message>
<xml_diff>
--- a/patois_learn_database_1.xlsx
+++ b/patois_learn_database_1.xlsx
@@ -5183,25 +5183,25 @@
         <v>yes</v>
       </c>
       <c r="C119" t="str">
-        <v/>
+        <v>Wi</v>
       </c>
       <c r="D119" t="str">
-        <v/>
+        <v>wee</v>
       </c>
       <c r="E119" t="str">
-        <v/>
+        <v>oui</v>
       </c>
       <c r="F119" t="str">
         <v>assets/images/vocab/haitian-creole/yes.png</v>
       </c>
       <c r="G119" t="str">
-        <v>assets/audio/haitian-creole/yes.mp3</v>
+        <v/>
       </c>
       <c r="H119" t="str">
         <v/>
       </c>
       <c r="I119" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J119" t="str">
         <v>unavailable</v>
@@ -5215,25 +5215,25 @@
         <v>no</v>
       </c>
       <c r="C120" t="str">
-        <v/>
+        <v>Non</v>
       </c>
       <c r="D120" t="str">
-        <v/>
+        <v>non</v>
       </c>
       <c r="E120" t="str">
-        <v/>
+        <v>non</v>
       </c>
       <c r="F120" t="str">
         <v>assets/images/vocab/haitian-creole/no.png</v>
       </c>
       <c r="G120" t="str">
-        <v>assets/audio/haitian-creole/no.mp3</v>
+        <v/>
       </c>
       <c r="H120" t="str">
         <v/>
       </c>
       <c r="I120" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J120" t="str">
         <v>unavailable</v>
@@ -5247,25 +5247,25 @@
         <v>maybe</v>
       </c>
       <c r="C121" t="str">
-        <v/>
+        <v>Petèt</v>
       </c>
       <c r="D121" t="str">
-        <v/>
+        <v>peh-tet</v>
       </c>
       <c r="E121" t="str">
-        <v/>
+        <v>peut-etre</v>
       </c>
       <c r="F121" t="str">
         <v>assets/images/vocab/haitian-creole/maybe.png</v>
       </c>
       <c r="G121" t="str">
-        <v>assets/audio/haitian-creole/maybe.mp3</v>
+        <v/>
       </c>
       <c r="H121" t="str">
         <v/>
       </c>
       <c r="I121" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J121" t="str">
         <v>unavailable</v>
@@ -5279,25 +5279,25 @@
         <v>okay</v>
       </c>
       <c r="C122" t="str">
-        <v/>
+        <v>Dakò</v>
       </c>
       <c r="D122" t="str">
-        <v/>
+        <v>da-ko</v>
       </c>
       <c r="E122" t="str">
-        <v/>
+        <v>daccord</v>
       </c>
       <c r="F122" t="str">
         <v>assets/images/vocab/haitian-creole/okay.png</v>
       </c>
       <c r="G122" t="str">
-        <v>assets/audio/haitian-creole/okay.mp3</v>
+        <v/>
       </c>
       <c r="H122" t="str">
         <v/>
       </c>
       <c r="I122" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J122" t="str">
         <v>unavailable</v>
@@ -5311,25 +5311,25 @@
         <v>again</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>Ankò</v>
       </c>
       <c r="D123" t="str">
-        <v/>
+        <v>an-ko</v>
       </c>
       <c r="E123" t="str">
-        <v/>
+        <v>encore</v>
       </c>
       <c r="F123" t="str">
         <v>assets/images/vocab/haitian-creole/again.png</v>
       </c>
       <c r="G123" t="str">
-        <v>assets/audio/haitian-creole/again.mp3</v>
+        <v/>
       </c>
       <c r="H123" t="str">
         <v/>
       </c>
       <c r="I123" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J123" t="str">
         <v>unavailable</v>
@@ -5343,25 +5343,25 @@
         <v>good-afternoon</v>
       </c>
       <c r="C124" t="str">
-        <v/>
+        <v>Bon apremidi</v>
       </c>
       <c r="D124" t="str">
-        <v/>
+        <v>bon ap-re-mi-di</v>
       </c>
       <c r="E124" t="str">
-        <v/>
+        <v>bon apres-midi</v>
       </c>
       <c r="F124" t="str">
         <v>assets/images/vocab/haitian-creole/good-afternoon.png</v>
       </c>
       <c r="G124" t="str">
-        <v>assets/audio/haitian-creole/good-afternoon.mp3</v>
+        <v/>
       </c>
       <c r="H124" t="str">
         <v/>
       </c>
       <c r="I124" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J124" t="str">
         <v>unavailable</v>
@@ -5375,25 +5375,25 @@
         <v>nice-to-meet-you</v>
       </c>
       <c r="C125" t="str">
-        <v/>
+        <v>Mwen kontan rankontre ou</v>
       </c>
       <c r="D125" t="str">
-        <v/>
+        <v>mwen kon-tan ran-kon-tre ou</v>
       </c>
       <c r="E125" t="str">
-        <v/>
+        <v>enchante</v>
       </c>
       <c r="F125" t="str">
         <v>assets/images/vocab/haitian-creole/nice-to-meet-you.png</v>
       </c>
       <c r="G125" t="str">
-        <v>assets/audio/haitian-creole/nice-to-meet-you.mp3</v>
+        <v/>
       </c>
       <c r="H125" t="str">
         <v/>
       </c>
       <c r="I125" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J125" t="str">
         <v>unavailable</v>
@@ -5407,25 +5407,25 @@
         <v>long-time-no-see</v>
       </c>
       <c r="C126" t="str">
-        <v/>
+        <v>Sa fè lontan nou pa wè</v>
       </c>
       <c r="D126" t="str">
-        <v/>
+        <v>sa fe lon-tan nou pa we</v>
       </c>
       <c r="E126" t="str">
-        <v/>
+        <v>ca fait longtemps</v>
       </c>
       <c r="F126" t="str">
         <v>assets/images/vocab/haitian-creole/long-time-no-see.png</v>
       </c>
       <c r="G126" t="str">
-        <v>assets/audio/haitian-creole/long-time-no-see.mp3</v>
+        <v/>
       </c>
       <c r="H126" t="str">
         <v/>
       </c>
       <c r="I126" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J126" t="str">
         <v>unavailable</v>
@@ -5439,25 +5439,25 @@
         <v>how-is-your-day</v>
       </c>
       <c r="C127" t="str">
-        <v/>
+        <v>Kijan jounen ou ye?</v>
       </c>
       <c r="D127" t="str">
-        <v/>
+        <v>ki-jan jou-nen ou ye</v>
       </c>
       <c r="E127" t="str">
-        <v/>
+        <v>comment se passe ta journee</v>
       </c>
       <c r="F127" t="str">
         <v>assets/images/vocab/haitian-creole/how-is-your-day.png</v>
       </c>
       <c r="G127" t="str">
-        <v>assets/audio/haitian-creole/how-is-your-day.mp3</v>
+        <v/>
       </c>
       <c r="H127" t="str">
         <v/>
       </c>
       <c r="I127" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J127" t="str">
         <v>unavailable</v>
@@ -5471,25 +5471,25 @@
         <v>have-a-good-day</v>
       </c>
       <c r="C128" t="str">
-        <v/>
+        <v>Pase yon bon jounen</v>
       </c>
       <c r="D128" t="str">
-        <v/>
+        <v>pa-se yon bon jou-nen</v>
       </c>
       <c r="E128" t="str">
-        <v/>
+        <v>bonne journee</v>
       </c>
       <c r="F128" t="str">
         <v>assets/images/vocab/haitian-creole/have-a-good-day.png</v>
       </c>
       <c r="G128" t="str">
-        <v>assets/audio/haitian-creole/have-a-good-day.mp3</v>
+        <v/>
       </c>
       <c r="H128" t="str">
         <v/>
       </c>
       <c r="I128" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J128" t="str">
         <v>unavailable</v>
@@ -5503,25 +5503,25 @@
         <v>what-is-your-name</v>
       </c>
       <c r="C129" t="str">
-        <v/>
+        <v>Kijan ou rele?</v>
       </c>
       <c r="D129" t="str">
-        <v/>
+        <v>ki-jan ou re-le</v>
       </c>
       <c r="E129" t="str">
-        <v/>
+        <v>comment tu tappelles</v>
       </c>
       <c r="F129" t="str">
         <v>assets/images/vocab/haitian-creole/what-is-your-name.png</v>
       </c>
       <c r="G129" t="str">
-        <v>assets/audio/haitian-creole/what-is-your-name.mp3</v>
+        <v/>
       </c>
       <c r="H129" t="str">
         <v/>
       </c>
       <c r="I129" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J129" t="str">
         <v>unavailable</v>
@@ -5535,25 +5535,25 @@
         <v>my-name-is</v>
       </c>
       <c r="C130" t="str">
-        <v/>
+        <v>Mwen rele...</v>
       </c>
       <c r="D130" t="str">
-        <v/>
+        <v>mwen re-le</v>
       </c>
       <c r="E130" t="str">
-        <v/>
+        <v>je mappelle</v>
       </c>
       <c r="F130" t="str">
         <v>assets/images/vocab/haitian-creole/my-name-is.png</v>
       </c>
       <c r="G130" t="str">
-        <v>assets/audio/haitian-creole/my-name-is.mp3</v>
+        <v/>
       </c>
       <c r="H130" t="str">
         <v/>
       </c>
       <c r="I130" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J130" t="str">
         <v>unavailable</v>
@@ -5567,25 +5567,25 @@
         <v>i-am-a-student</v>
       </c>
       <c r="C131" t="str">
-        <v/>
+        <v>Mwen se yon etidyan</v>
       </c>
       <c r="D131" t="str">
-        <v/>
+        <v>mwen se yon e-ti-dyan</v>
       </c>
       <c r="E131" t="str">
-        <v/>
+        <v>je suis etudiant</v>
       </c>
       <c r="F131" t="str">
         <v>assets/images/vocab/haitian-creole/i-am-a-student.png</v>
       </c>
       <c r="G131" t="str">
-        <v>assets/audio/haitian-creole/i-am-a-student.mp3</v>
+        <v/>
       </c>
       <c r="H131" t="str">
         <v/>
       </c>
       <c r="I131" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J131" t="str">
         <v>unavailable</v>
@@ -5599,25 +5599,25 @@
         <v>i-am-learning</v>
       </c>
       <c r="C132" t="str">
-        <v/>
+        <v>M ap aprann...</v>
       </c>
       <c r="D132" t="str">
-        <v/>
+        <v>map ap-rann</v>
       </c>
       <c r="E132" t="str">
-        <v/>
+        <v>japprends</v>
       </c>
       <c r="F132" t="str">
         <v>assets/images/vocab/haitian-creole/i-am-learning.png</v>
       </c>
       <c r="G132" t="str">
-        <v>assets/audio/haitian-creole/i-am-learning.mp3</v>
+        <v/>
       </c>
       <c r="H132" t="str">
         <v/>
       </c>
       <c r="I132" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J132" t="str">
         <v>unavailable</v>
@@ -5631,25 +5631,25 @@
         <v>i-speak</v>
       </c>
       <c r="C133" t="str">
-        <v/>
+        <v>Mwen pale...</v>
       </c>
       <c r="D133" t="str">
-        <v/>
+        <v>mwen pa-le</v>
       </c>
       <c r="E133" t="str">
-        <v/>
+        <v>je parle</v>
       </c>
       <c r="F133" t="str">
         <v>assets/images/vocab/haitian-creole/i-speak.png</v>
       </c>
       <c r="G133" t="str">
-        <v>assets/audio/haitian-creole/i-speak.mp3</v>
+        <v/>
       </c>
       <c r="H133" t="str">
         <v/>
       </c>
       <c r="I133" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J133" t="str">
         <v>unavailable</v>
@@ -5663,25 +5663,25 @@
         <v>where-are-you-from</v>
       </c>
       <c r="C134" t="str">
-        <v/>
+        <v>Ki kote ou soti?</v>
       </c>
       <c r="D134" t="str">
-        <v/>
+        <v>ki ko-te ou so-ti</v>
       </c>
       <c r="E134" t="str">
-        <v/>
+        <v>tu viens dou</v>
       </c>
       <c r="F134" t="str">
         <v>assets/images/vocab/haitian-creole/where-are-you-from.png</v>
       </c>
       <c r="G134" t="str">
-        <v>assets/audio/haitian-creole/where-are-you-from.mp3</v>
+        <v/>
       </c>
       <c r="H134" t="str">
         <v/>
       </c>
       <c r="I134" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J134" t="str">
         <v>unavailable</v>
@@ -5695,25 +5695,25 @@
         <v>i-am-from</v>
       </c>
       <c r="C135" t="str">
-        <v/>
+        <v>Mwen soti...</v>
       </c>
       <c r="D135" t="str">
-        <v/>
+        <v>mwen so-ti</v>
       </c>
       <c r="E135" t="str">
-        <v/>
+        <v>je viens de</v>
       </c>
       <c r="F135" t="str">
         <v>assets/images/vocab/haitian-creole/i-am-from.png</v>
       </c>
       <c r="G135" t="str">
-        <v>assets/audio/haitian-creole/i-am-from.mp3</v>
+        <v/>
       </c>
       <c r="H135" t="str">
         <v/>
       </c>
       <c r="I135" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J135" t="str">
         <v>unavailable</v>
@@ -5727,25 +5727,25 @@
         <v>where-do-you-live</v>
       </c>
       <c r="C136" t="str">
-        <v/>
+        <v>Ki kote ou rete?</v>
       </c>
       <c r="D136" t="str">
-        <v/>
+        <v>ki ko-te ou re-te</v>
       </c>
       <c r="E136" t="str">
-        <v/>
+        <v>ou habites-tu</v>
       </c>
       <c r="F136" t="str">
         <v>assets/images/vocab/haitian-creole/where-do-you-live.png</v>
       </c>
       <c r="G136" t="str">
-        <v>assets/audio/haitian-creole/where-do-you-live.mp3</v>
+        <v/>
       </c>
       <c r="H136" t="str">
         <v/>
       </c>
       <c r="I136" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J136" t="str">
         <v>unavailable</v>
@@ -5759,25 +5759,25 @@
         <v>i-live-in</v>
       </c>
       <c r="C137" t="str">
-        <v/>
+        <v>Mwen rete...</v>
       </c>
       <c r="D137" t="str">
-        <v/>
+        <v>mwen re-te</v>
       </c>
       <c r="E137" t="str">
-        <v/>
+        <v>jhabite a</v>
       </c>
       <c r="F137" t="str">
         <v>assets/images/vocab/haitian-creole/i-live-in.png</v>
       </c>
       <c r="G137" t="str">
-        <v>assets/audio/haitian-creole/i-live-in.mp3</v>
+        <v/>
       </c>
       <c r="H137" t="str">
         <v/>
       </c>
       <c r="I137" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J137" t="str">
         <v>unavailable</v>
@@ -5791,25 +5791,25 @@
         <v>which-language-do-you-speak</v>
       </c>
       <c r="C138" t="str">
-        <v/>
+        <v>Ki lang ou pale?</v>
       </c>
       <c r="D138" t="str">
-        <v/>
+        <v>ki lang ou pa-le</v>
       </c>
       <c r="E138" t="str">
-        <v/>
+        <v>quelle langue parles-tu</v>
       </c>
       <c r="F138" t="str">
         <v>assets/images/vocab/haitian-creole/which-language-do-you-speak.png</v>
       </c>
       <c r="G138" t="str">
-        <v>assets/audio/haitian-creole/which-language-do-you-speak.mp3</v>
+        <v/>
       </c>
       <c r="H138" t="str">
         <v/>
       </c>
       <c r="I138" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J138" t="str">
         <v>unavailable</v>
@@ -5823,25 +5823,25 @@
         <v>family</v>
       </c>
       <c r="C139" t="str">
-        <v/>
+        <v>Fanmi</v>
       </c>
       <c r="D139" t="str">
-        <v/>
+        <v>fan-mi</v>
       </c>
       <c r="E139" t="str">
-        <v/>
+        <v>famille</v>
       </c>
       <c r="F139" t="str">
         <v>assets/images/vocab/haitian-creole/family.png</v>
       </c>
       <c r="G139" t="str">
-        <v>assets/audio/haitian-creole/family.mp3</v>
+        <v/>
       </c>
       <c r="H139" t="str">
         <v/>
       </c>
       <c r="I139" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J139" t="str">
         <v>unavailable</v>
@@ -5855,25 +5855,25 @@
         <v>parents</v>
       </c>
       <c r="C140" t="str">
-        <v/>
+        <v>Paran</v>
       </c>
       <c r="D140" t="str">
-        <v/>
+        <v>pa-ran</v>
       </c>
       <c r="E140" t="str">
-        <v/>
+        <v>parents</v>
       </c>
       <c r="F140" t="str">
         <v>assets/images/vocab/haitian-creole/parents.png</v>
       </c>
       <c r="G140" t="str">
-        <v>assets/audio/haitian-creole/parents.mp3</v>
+        <v/>
       </c>
       <c r="H140" t="str">
         <v/>
       </c>
       <c r="I140" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J140" t="str">
         <v>unavailable</v>
@@ -5887,25 +5887,25 @@
         <v>husband</v>
       </c>
       <c r="C141" t="str">
-        <v/>
+        <v>Mari</v>
       </c>
       <c r="D141" t="str">
-        <v/>
+        <v>ma-ri</v>
       </c>
       <c r="E141" t="str">
-        <v/>
+        <v>mari</v>
       </c>
       <c r="F141" t="str">
         <v>assets/images/vocab/haitian-creole/husband.png</v>
       </c>
       <c r="G141" t="str">
-        <v>assets/audio/haitian-creole/husband.mp3</v>
+        <v/>
       </c>
       <c r="H141" t="str">
         <v/>
       </c>
       <c r="I141" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J141" t="str">
         <v>unavailable</v>
@@ -5919,25 +5919,25 @@
         <v>wife</v>
       </c>
       <c r="C142" t="str">
-        <v/>
+        <v>Madanm</v>
       </c>
       <c r="D142" t="str">
-        <v/>
+        <v>ma-danm</v>
       </c>
       <c r="E142" t="str">
-        <v/>
+        <v>femme</v>
       </c>
       <c r="F142" t="str">
         <v>assets/images/vocab/haitian-creole/wife.png</v>
       </c>
       <c r="G142" t="str">
-        <v>assets/audio/haitian-creole/wife.mp3</v>
+        <v/>
       </c>
       <c r="H142" t="str">
         <v/>
       </c>
       <c r="I142" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J142" t="str">
         <v>unavailable</v>
@@ -5951,25 +5951,25 @@
         <v>son</v>
       </c>
       <c r="C143" t="str">
-        <v/>
+        <v>Pitit gason</v>
       </c>
       <c r="D143" t="str">
-        <v/>
+        <v>pi-tit ga-son</v>
       </c>
       <c r="E143" t="str">
-        <v/>
+        <v>fils</v>
       </c>
       <c r="F143" t="str">
         <v>assets/images/vocab/haitian-creole/son.png</v>
       </c>
       <c r="G143" t="str">
-        <v>assets/audio/haitian-creole/son.mp3</v>
+        <v/>
       </c>
       <c r="H143" t="str">
         <v/>
       </c>
       <c r="I143" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J143" t="str">
         <v>unavailable</v>
@@ -5983,25 +5983,25 @@
         <v>daughter</v>
       </c>
       <c r="C144" t="str">
-        <v/>
+        <v>Pitit fi</v>
       </c>
       <c r="D144" t="str">
-        <v/>
+        <v>pi-tit fi</v>
       </c>
       <c r="E144" t="str">
-        <v/>
+        <v>fille</v>
       </c>
       <c r="F144" t="str">
         <v>assets/images/vocab/haitian-creole/daughter.png</v>
       </c>
       <c r="G144" t="str">
-        <v>assets/audio/haitian-creole/daughter.mp3</v>
+        <v/>
       </c>
       <c r="H144" t="str">
         <v/>
       </c>
       <c r="I144" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J144" t="str">
         <v>unavailable</v>
@@ -6015,25 +6015,25 @@
         <v>grandfather</v>
       </c>
       <c r="C145" t="str">
-        <v/>
+        <v>Granpapa</v>
       </c>
       <c r="D145" t="str">
-        <v/>
+        <v>gran-pa-pa</v>
       </c>
       <c r="E145" t="str">
-        <v/>
+        <v>grand-pere</v>
       </c>
       <c r="F145" t="str">
         <v>assets/images/vocab/haitian-creole/grandfather.png</v>
       </c>
       <c r="G145" t="str">
-        <v>assets/audio/haitian-creole/grandfather.mp3</v>
+        <v/>
       </c>
       <c r="H145" t="str">
         <v/>
       </c>
       <c r="I145" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J145" t="str">
         <v>unavailable</v>
@@ -6047,25 +6047,25 @@
         <v>please</v>
       </c>
       <c r="C146" t="str">
-        <v/>
+        <v>Tanpri</v>
       </c>
       <c r="D146" t="str">
-        <v/>
+        <v>tan-pri</v>
       </c>
       <c r="E146" t="str">
-        <v/>
+        <v>sil te plait</v>
       </c>
       <c r="F146" t="str">
         <v>assets/images/vocab/haitian-creole/please.png</v>
       </c>
       <c r="G146" t="str">
-        <v>assets/audio/haitian-creole/please.mp3</v>
+        <v/>
       </c>
       <c r="H146" t="str">
         <v/>
       </c>
       <c r="I146" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J146" t="str">
         <v>unavailable</v>
@@ -6079,25 +6079,25 @@
         <v>thank-you</v>
       </c>
       <c r="C147" t="str">
-        <v/>
+        <v>Mèsi</v>
       </c>
       <c r="D147" t="str">
-        <v/>
+        <v>me-si</v>
       </c>
       <c r="E147" t="str">
-        <v/>
+        <v>merci</v>
       </c>
       <c r="F147" t="str">
         <v>assets/images/vocab/haitian-creole/thank-you.png</v>
       </c>
       <c r="G147" t="str">
-        <v>assets/audio/haitian-creole/thank-you.mp3</v>
+        <v/>
       </c>
       <c r="H147" t="str">
         <v/>
       </c>
       <c r="I147" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J147" t="str">
         <v>unavailable</v>
@@ -6111,25 +6111,25 @@
         <v>no-problem</v>
       </c>
       <c r="C148" t="str">
-        <v/>
+        <v>Pa gen pwoblèm</v>
       </c>
       <c r="D148" t="str">
-        <v/>
+        <v>pa gen pwo-blem</v>
       </c>
       <c r="E148" t="str">
-        <v/>
+        <v>pas de probleme</v>
       </c>
       <c r="F148" t="str">
         <v>assets/images/vocab/haitian-creole/no-problem.png</v>
       </c>
       <c r="G148" t="str">
-        <v>assets/audio/haitian-creole/no-problem.mp3</v>
+        <v/>
       </c>
       <c r="H148" t="str">
         <v/>
       </c>
       <c r="I148" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J148" t="str">
         <v>unavailable</v>
@@ -6143,25 +6143,25 @@
         <v>excuse-me</v>
       </c>
       <c r="C149" t="str">
-        <v/>
+        <v>Eskize m</v>
       </c>
       <c r="D149" t="str">
-        <v/>
+        <v>es-ki-ze m</v>
       </c>
       <c r="E149" t="str">
-        <v/>
+        <v>excuse-moi</v>
       </c>
       <c r="F149" t="str">
         <v>assets/images/vocab/haitian-creole/excuse-me.png</v>
       </c>
       <c r="G149" t="str">
-        <v>assets/audio/haitian-creole/excuse-me.mp3</v>
+        <v/>
       </c>
       <c r="H149" t="str">
         <v/>
       </c>
       <c r="I149" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J149" t="str">
         <v>unavailable</v>
@@ -6175,25 +6175,25 @@
         <v>sorry</v>
       </c>
       <c r="C150" t="str">
-        <v/>
+        <v>Mwen regrèt</v>
       </c>
       <c r="D150" t="str">
-        <v/>
+        <v>mwen re-gret</v>
       </c>
       <c r="E150" t="str">
-        <v/>
+        <v>je suis desole</v>
       </c>
       <c r="F150" t="str">
         <v>assets/images/vocab/haitian-creole/sorry.png</v>
       </c>
       <c r="G150" t="str">
-        <v>assets/audio/haitian-creole/sorry.mp3</v>
+        <v/>
       </c>
       <c r="H150" t="str">
         <v/>
       </c>
       <c r="I150" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J150" t="str">
         <v>unavailable</v>
@@ -6207,25 +6207,25 @@
         <v>this-is-my-family</v>
       </c>
       <c r="C151" t="str">
-        <v/>
+        <v>Sa a se fanmi mwen</v>
       </c>
       <c r="D151" t="str">
-        <v/>
+        <v>sa a se fan-mi mwen</v>
       </c>
       <c r="E151" t="str">
-        <v/>
+        <v>voici ma famille</v>
       </c>
       <c r="F151" t="str">
         <v>assets/images/vocab/haitian-creole/this-is-my-family.png</v>
       </c>
       <c r="G151" t="str">
-        <v>assets/audio/haitian-creole/this-is-my-family.mp3</v>
+        <v/>
       </c>
       <c r="H151" t="str">
         <v/>
       </c>
       <c r="I151" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J151" t="str">
         <v>unavailable</v>
@@ -6239,25 +6239,25 @@
         <v>this-is-my-husband</v>
       </c>
       <c r="C152" t="str">
-        <v/>
+        <v>Sa a se mari mwen</v>
       </c>
       <c r="D152" t="str">
-        <v/>
+        <v>sa a se ma-ri mwen</v>
       </c>
       <c r="E152" t="str">
-        <v/>
+        <v>voici mon mari</v>
       </c>
       <c r="F152" t="str">
         <v>assets/images/vocab/haitian-creole/this-is-my-husband.png</v>
       </c>
       <c r="G152" t="str">
-        <v>assets/audio/haitian-creole/this-is-my-husband.mp3</v>
+        <v/>
       </c>
       <c r="H152" t="str">
         <v/>
       </c>
       <c r="I152" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J152" t="str">
         <v>unavailable</v>
@@ -6271,25 +6271,25 @@
         <v>this-is-my-wife</v>
       </c>
       <c r="C153" t="str">
-        <v/>
+        <v>Sa a se madanm mwen</v>
       </c>
       <c r="D153" t="str">
-        <v/>
+        <v>sa a se ma-danm mwen</v>
       </c>
       <c r="E153" t="str">
-        <v/>
+        <v>voici ma femme</v>
       </c>
       <c r="F153" t="str">
         <v>assets/images/vocab/haitian-creole/this-is-my-wife.png</v>
       </c>
       <c r="G153" t="str">
-        <v>assets/audio/haitian-creole/this-is-my-wife.mp3</v>
+        <v/>
       </c>
       <c r="H153" t="str">
         <v/>
       </c>
       <c r="I153" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J153" t="str">
         <v>unavailable</v>
@@ -6303,25 +6303,25 @@
         <v>he-lives-here</v>
       </c>
       <c r="C154" t="str">
-        <v/>
+        <v>Li rete isit la</v>
       </c>
       <c r="D154" t="str">
-        <v/>
+        <v>li re-te i-sit la</v>
       </c>
       <c r="E154" t="str">
-        <v/>
+        <v>il habite ici</v>
       </c>
       <c r="F154" t="str">
         <v>assets/images/vocab/haitian-creole/he-lives-here.png</v>
       </c>
       <c r="G154" t="str">
-        <v>assets/audio/haitian-creole/he-lives-here.mp3</v>
+        <v/>
       </c>
       <c r="H154" t="str">
         <v/>
       </c>
       <c r="I154" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J154" t="str">
         <v>unavailable</v>
@@ -6335,25 +6335,25 @@
         <v>she-works-here</v>
       </c>
       <c r="C155" t="str">
-        <v/>
+        <v>Li travay isit la</v>
       </c>
       <c r="D155" t="str">
-        <v/>
+        <v>li tra-vay i-sit la</v>
       </c>
       <c r="E155" t="str">
-        <v/>
+        <v>elle travaille ici</v>
       </c>
       <c r="F155" t="str">
         <v>assets/images/vocab/haitian-creole/she-works-here.png</v>
       </c>
       <c r="G155" t="str">
-        <v>assets/audio/haitian-creole/she-works-here.mp3</v>
+        <v/>
       </c>
       <c r="H155" t="str">
         <v/>
       </c>
       <c r="I155" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J155" t="str">
         <v>unavailable</v>
@@ -6367,25 +6367,25 @@
         <v>we-speak</v>
       </c>
       <c r="C156" t="str">
-        <v/>
+        <v>Nou pale...</v>
       </c>
       <c r="D156" t="str">
-        <v/>
+        <v>nou pa-le</v>
       </c>
       <c r="E156" t="str">
-        <v/>
+        <v>nous parlons</v>
       </c>
       <c r="F156" t="str">
         <v>assets/images/vocab/haitian-creole/we-speak.png</v>
       </c>
       <c r="G156" t="str">
-        <v>assets/audio/haitian-creole/we-speak.mp3</v>
+        <v/>
       </c>
       <c r="H156" t="str">
         <v/>
       </c>
       <c r="I156" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J156" t="str">
         <v>unavailable</v>
@@ -6399,25 +6399,25 @@
         <v>they-are-from</v>
       </c>
       <c r="C157" t="str">
-        <v/>
+        <v>Yo soti...</v>
       </c>
       <c r="D157" t="str">
-        <v/>
+        <v>yo so-ti</v>
       </c>
       <c r="E157" t="str">
-        <v/>
+        <v>ils viennent de</v>
       </c>
       <c r="F157" t="str">
         <v>assets/images/vocab/haitian-creole/they-are-from.png</v>
       </c>
       <c r="G157" t="str">
-        <v>assets/audio/haitian-creole/they-are-from.mp3</v>
+        <v/>
       </c>
       <c r="H157" t="str">
         <v/>
       </c>
       <c r="I157" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J157" t="str">
         <v>unavailable</v>
@@ -14811,7 +14811,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M193"/>
+  <dimension ref="A1:M257"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22726,9 +22726,2633 @@
         <v>unavailable</v>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B194" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C194" t="str">
+        <v>haitian-creole-getting-started-01-yes</v>
+      </c>
+      <c r="D194">
+        <v>1</v>
+      </c>
+      <c r="E194" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F194" t="str">
+        <v>What does "Wi" mean in Haitian Creole?</v>
+      </c>
+      <c r="G194" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H194" t="str">
+        <v>["no","maybe","okay"]</v>
+      </c>
+      <c r="I194" t="str">
+        <v>yes</v>
+      </c>
+      <c r="J194" t="str">
+        <v>["yes"]</v>
+      </c>
+      <c r="K194" t="str">
+        <v/>
+      </c>
+      <c r="L194" t="b">
+        <v>1</v>
+      </c>
+      <c r="M194" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B195" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C195" t="str">
+        <v>haitian-creole-getting-started-02-no</v>
+      </c>
+      <c r="D195">
+        <v>2</v>
+      </c>
+      <c r="E195" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F195" t="str">
+        <v>Build the Haitian Creole phrase for "no".</v>
+      </c>
+      <c r="G195" t="str">
+        <v>Non</v>
+      </c>
+      <c r="H195" t="str">
+        <v>["Wi","Petèt","Dakò"]</v>
+      </c>
+      <c r="I195" t="str">
+        <v>no</v>
+      </c>
+      <c r="J195" t="str">
+        <v>["no"]</v>
+      </c>
+      <c r="K195" t="str">
+        <v/>
+      </c>
+      <c r="L195" t="b">
+        <v>1</v>
+      </c>
+      <c r="M195" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B196" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C196" t="str">
+        <v>haitian-creole-getting-started-03-match</v>
+      </c>
+      <c r="D196">
+        <v>3</v>
+      </c>
+      <c r="E196" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F196" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G196" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H196" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I196" t="str">
+        <v/>
+      </c>
+      <c r="J196" t="str">
+        <v>["yes","no","maybe","okay"]</v>
+      </c>
+      <c r="K196" t="str">
+        <v/>
+      </c>
+      <c r="L196" t="b">
+        <v>0</v>
+      </c>
+      <c r="M196" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B197" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C197" t="str">
+        <v>haitian-creole-getting-started-04-okay</v>
+      </c>
+      <c r="D197">
+        <v>4</v>
+      </c>
+      <c r="E197" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F197" t="str">
+        <v>Build the English meaning of "Dakò".</v>
+      </c>
+      <c r="G197" t="str">
+        <v>okay</v>
+      </c>
+      <c r="H197" t="str">
+        <v>["yes","no","maybe"]</v>
+      </c>
+      <c r="I197" t="str">
+        <v>okay</v>
+      </c>
+      <c r="J197" t="str">
+        <v>["okay"]</v>
+      </c>
+      <c r="K197" t="str">
+        <v/>
+      </c>
+      <c r="L197" t="b">
+        <v>1</v>
+      </c>
+      <c r="M197" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B198" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C198" t="str">
+        <v>haitian-creole-getting-started-05-again</v>
+      </c>
+      <c r="D198">
+        <v>5</v>
+      </c>
+      <c r="E198" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F198" t="str">
+        <v>Choose the Haitian Creole for "again".</v>
+      </c>
+      <c r="G198" t="str">
+        <v>Ankò</v>
+      </c>
+      <c r="H198" t="str">
+        <v>["Wi","Non","Petèt"]</v>
+      </c>
+      <c r="I198" t="str">
+        <v>again</v>
+      </c>
+      <c r="J198" t="str">
+        <v>["again"]</v>
+      </c>
+      <c r="K198" t="str">
+        <v/>
+      </c>
+      <c r="L198" t="b">
+        <v>1</v>
+      </c>
+      <c r="M198" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B199" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C199" t="str">
+        <v>haitian-creole-getting-started-06-again</v>
+      </c>
+      <c r="D199">
+        <v>6</v>
+      </c>
+      <c r="E199" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F199" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G199" t="str">
+        <v>again</v>
+      </c>
+      <c r="H199" t="str">
+        <v>["yes","no","maybe"]</v>
+      </c>
+      <c r="I199" t="str">
+        <v>again</v>
+      </c>
+      <c r="J199" t="str">
+        <v>["again"]</v>
+      </c>
+      <c r="K199" t="str">
+        <v/>
+      </c>
+      <c r="L199" t="b">
+        <v>1</v>
+      </c>
+      <c r="M199" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B200" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C200" t="str">
+        <v>haitian-creole-easy-greetings-01-good-afternoon</v>
+      </c>
+      <c r="D200">
+        <v>1</v>
+      </c>
+      <c r="E200" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F200" t="str">
+        <v>What does "Bon apremidi" mean in Haitian Creole?</v>
+      </c>
+      <c r="G200" t="str">
+        <v>good afternoon</v>
+      </c>
+      <c r="H200" t="str">
+        <v>["nice to meet you","long time no see","how is your day"]</v>
+      </c>
+      <c r="I200" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J200" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K200" t="str">
+        <v/>
+      </c>
+      <c r="L200" t="b">
+        <v>1</v>
+      </c>
+      <c r="M200" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B201" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C201" t="str">
+        <v>haitian-creole-easy-greetings-02-nice-to-meet-you</v>
+      </c>
+      <c r="D201">
+        <v>2</v>
+      </c>
+      <c r="E201" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F201" t="str">
+        <v>Build the Haitian Creole phrase for "nice to meet you".</v>
+      </c>
+      <c r="G201" t="str">
+        <v>Mwen kontan rankontre ou</v>
+      </c>
+      <c r="H201" t="str">
+        <v>["Bon apremidi","Sa fè lontan nou pa wè","Kijan jounen ou ye?"]</v>
+      </c>
+      <c r="I201" t="str">
+        <v>nice-to-meet-you</v>
+      </c>
+      <c r="J201" t="str">
+        <v>["nice-to-meet-you"]</v>
+      </c>
+      <c r="K201" t="str">
+        <v/>
+      </c>
+      <c r="L201" t="b">
+        <v>1</v>
+      </c>
+      <c r="M201" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B202" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C202" t="str">
+        <v>haitian-creole-easy-greetings-03-match</v>
+      </c>
+      <c r="D202">
+        <v>3</v>
+      </c>
+      <c r="E202" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F202" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G202" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H202" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I202" t="str">
+        <v/>
+      </c>
+      <c r="J202" t="str">
+        <v>["good-afternoon","nice-to-meet-you","long-time-no-see","how-is-your-day"]</v>
+      </c>
+      <c r="K202" t="str">
+        <v/>
+      </c>
+      <c r="L202" t="b">
+        <v>0</v>
+      </c>
+      <c r="M202" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B203" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C203" t="str">
+        <v>haitian-creole-easy-greetings-04-how-is-your-day</v>
+      </c>
+      <c r="D203">
+        <v>4</v>
+      </c>
+      <c r="E203" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F203" t="str">
+        <v>Build the English meaning of "Kijan jounen ou ye?".</v>
+      </c>
+      <c r="G203" t="str">
+        <v>how is your day</v>
+      </c>
+      <c r="H203" t="str">
+        <v>["good afternoon","nice to meet you","long time no see"]</v>
+      </c>
+      <c r="I203" t="str">
+        <v>how-is-your-day</v>
+      </c>
+      <c r="J203" t="str">
+        <v>["how-is-your-day"]</v>
+      </c>
+      <c r="K203" t="str">
+        <v/>
+      </c>
+      <c r="L203" t="b">
+        <v>1</v>
+      </c>
+      <c r="M203" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B204" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C204" t="str">
+        <v>haitian-creole-easy-greetings-05-have-a-good-day</v>
+      </c>
+      <c r="D204">
+        <v>5</v>
+      </c>
+      <c r="E204" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F204" t="str">
+        <v>Choose the Haitian Creole for "have a good day".</v>
+      </c>
+      <c r="G204" t="str">
+        <v>Pase yon bon jounen</v>
+      </c>
+      <c r="H204" t="str">
+        <v>["Bon apremidi","Mwen kontan rankontre ou","Sa fè lontan nou pa wè"]</v>
+      </c>
+      <c r="I204" t="str">
+        <v>have-a-good-day</v>
+      </c>
+      <c r="J204" t="str">
+        <v>["have-a-good-day"]</v>
+      </c>
+      <c r="K204" t="str">
+        <v/>
+      </c>
+      <c r="L204" t="b">
+        <v>1</v>
+      </c>
+      <c r="M204" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B205" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C205" t="str">
+        <v>haitian-creole-easy-greetings-06-have-a-good-day</v>
+      </c>
+      <c r="D205">
+        <v>6</v>
+      </c>
+      <c r="E205" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F205" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G205" t="str">
+        <v>have a good day</v>
+      </c>
+      <c r="H205" t="str">
+        <v>["good afternoon","nice to meet you","long time no see"]</v>
+      </c>
+      <c r="I205" t="str">
+        <v>have-a-good-day</v>
+      </c>
+      <c r="J205" t="str">
+        <v>["have-a-good-day"]</v>
+      </c>
+      <c r="K205" t="str">
+        <v/>
+      </c>
+      <c r="L205" t="b">
+        <v>1</v>
+      </c>
+      <c r="M205" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B206" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C206" t="str">
+        <v>haitian-creole-introducing-yourself-01-what-is-your-name</v>
+      </c>
+      <c r="D206">
+        <v>1</v>
+      </c>
+      <c r="E206" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F206" t="str">
+        <v>What does "Kijan ou rele?" mean in Haitian Creole?</v>
+      </c>
+      <c r="G206" t="str">
+        <v>what is your name</v>
+      </c>
+      <c r="H206" t="str">
+        <v>["my name is","i am a student","i am learning"]</v>
+      </c>
+      <c r="I206" t="str">
+        <v>what-is-your-name</v>
+      </c>
+      <c r="J206" t="str">
+        <v>["what-is-your-name"]</v>
+      </c>
+      <c r="K206" t="str">
+        <v/>
+      </c>
+      <c r="L206" t="b">
+        <v>1</v>
+      </c>
+      <c r="M206" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B207" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C207" t="str">
+        <v>haitian-creole-introducing-yourself-02-my-name-is</v>
+      </c>
+      <c r="D207">
+        <v>2</v>
+      </c>
+      <c r="E207" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F207" t="str">
+        <v>Build the Haitian Creole phrase for "my name is".</v>
+      </c>
+      <c r="G207" t="str">
+        <v>Mwen rele...</v>
+      </c>
+      <c r="H207" t="str">
+        <v>["Kijan ou rele?","Mwen se yon etidyan","M ap aprann..."]</v>
+      </c>
+      <c r="I207" t="str">
+        <v>my-name-is</v>
+      </c>
+      <c r="J207" t="str">
+        <v>["my-name-is"]</v>
+      </c>
+      <c r="K207" t="str">
+        <v/>
+      </c>
+      <c r="L207" t="b">
+        <v>1</v>
+      </c>
+      <c r="M207" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B208" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C208" t="str">
+        <v>haitian-creole-introducing-yourself-03-match</v>
+      </c>
+      <c r="D208">
+        <v>3</v>
+      </c>
+      <c r="E208" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F208" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G208" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H208" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I208" t="str">
+        <v/>
+      </c>
+      <c r="J208" t="str">
+        <v>["what-is-your-name","my-name-is","i-am-a-student","i-am-learning"]</v>
+      </c>
+      <c r="K208" t="str">
+        <v/>
+      </c>
+      <c r="L208" t="b">
+        <v>0</v>
+      </c>
+      <c r="M208" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B209" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C209" t="str">
+        <v>haitian-creole-introducing-yourself-04-i-am-learning</v>
+      </c>
+      <c r="D209">
+        <v>4</v>
+      </c>
+      <c r="E209" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F209" t="str">
+        <v>Build the English meaning of "M ap aprann...".</v>
+      </c>
+      <c r="G209" t="str">
+        <v>i am learning</v>
+      </c>
+      <c r="H209" t="str">
+        <v>["what is your name","my name is","i am a student"]</v>
+      </c>
+      <c r="I209" t="str">
+        <v>i-am-learning</v>
+      </c>
+      <c r="J209" t="str">
+        <v>["i-am-learning"]</v>
+      </c>
+      <c r="K209" t="str">
+        <v/>
+      </c>
+      <c r="L209" t="b">
+        <v>1</v>
+      </c>
+      <c r="M209" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B210" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C210" t="str">
+        <v>haitian-creole-introducing-yourself-05-i-speak</v>
+      </c>
+      <c r="D210">
+        <v>5</v>
+      </c>
+      <c r="E210" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F210" t="str">
+        <v>Choose the Haitian Creole for "i speak".</v>
+      </c>
+      <c r="G210" t="str">
+        <v>Mwen pale...</v>
+      </c>
+      <c r="H210" t="str">
+        <v>["Kijan ou rele?","Mwen rele...","Mwen se yon etidyan"]</v>
+      </c>
+      <c r="I210" t="str">
+        <v>i-speak</v>
+      </c>
+      <c r="J210" t="str">
+        <v>["i-speak"]</v>
+      </c>
+      <c r="K210" t="str">
+        <v/>
+      </c>
+      <c r="L210" t="b">
+        <v>1</v>
+      </c>
+      <c r="M210" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B211" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C211" t="str">
+        <v>haitian-creole-introducing-yourself-06-i-speak</v>
+      </c>
+      <c r="D211">
+        <v>6</v>
+      </c>
+      <c r="E211" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F211" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G211" t="str">
+        <v>i speak</v>
+      </c>
+      <c r="H211" t="str">
+        <v>["what is your name","my name is","i am a student"]</v>
+      </c>
+      <c r="I211" t="str">
+        <v>i-speak</v>
+      </c>
+      <c r="J211" t="str">
+        <v>["i-speak"]</v>
+      </c>
+      <c r="K211" t="str">
+        <v/>
+      </c>
+      <c r="L211" t="b">
+        <v>1</v>
+      </c>
+      <c r="M211" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B212" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C212" t="str">
+        <v>haitian-creole-your-background-01-where-are-you-from</v>
+      </c>
+      <c r="D212">
+        <v>1</v>
+      </c>
+      <c r="E212" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F212" t="str">
+        <v>What does "Ki kote ou soti?" mean in Haitian Creole?</v>
+      </c>
+      <c r="G212" t="str">
+        <v>where are you from</v>
+      </c>
+      <c r="H212" t="str">
+        <v>["i am from","where do you live","i live in"]</v>
+      </c>
+      <c r="I212" t="str">
+        <v>where-are-you-from</v>
+      </c>
+      <c r="J212" t="str">
+        <v>["where-are-you-from"]</v>
+      </c>
+      <c r="K212" t="str">
+        <v/>
+      </c>
+      <c r="L212" t="b">
+        <v>1</v>
+      </c>
+      <c r="M212" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B213" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C213" t="str">
+        <v>haitian-creole-your-background-02-i-am-from</v>
+      </c>
+      <c r="D213">
+        <v>2</v>
+      </c>
+      <c r="E213" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F213" t="str">
+        <v>Build the Haitian Creole phrase for "i am from".</v>
+      </c>
+      <c r="G213" t="str">
+        <v>Mwen soti...</v>
+      </c>
+      <c r="H213" t="str">
+        <v>["Ki kote ou soti?","Ki kote ou rete?","Mwen rete..."]</v>
+      </c>
+      <c r="I213" t="str">
+        <v>i-am-from</v>
+      </c>
+      <c r="J213" t="str">
+        <v>["i-am-from"]</v>
+      </c>
+      <c r="K213" t="str">
+        <v/>
+      </c>
+      <c r="L213" t="b">
+        <v>1</v>
+      </c>
+      <c r="M213" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B214" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C214" t="str">
+        <v>haitian-creole-your-background-03-match</v>
+      </c>
+      <c r="D214">
+        <v>3</v>
+      </c>
+      <c r="E214" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G214" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H214" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I214" t="str">
+        <v/>
+      </c>
+      <c r="J214" t="str">
+        <v>["where-are-you-from","i-am-from","where-do-you-live","i-live-in"]</v>
+      </c>
+      <c r="K214" t="str">
+        <v/>
+      </c>
+      <c r="L214" t="b">
+        <v>0</v>
+      </c>
+      <c r="M214" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B215" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C215" t="str">
+        <v>haitian-creole-your-background-04-i-live-in</v>
+      </c>
+      <c r="D215">
+        <v>4</v>
+      </c>
+      <c r="E215" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Build the English meaning of "Mwen rete...".</v>
+      </c>
+      <c r="G215" t="str">
+        <v>i live in</v>
+      </c>
+      <c r="H215" t="str">
+        <v>["where are you from","i am from","where do you live"]</v>
+      </c>
+      <c r="I215" t="str">
+        <v>i-live-in</v>
+      </c>
+      <c r="J215" t="str">
+        <v>["i-live-in"]</v>
+      </c>
+      <c r="K215" t="str">
+        <v/>
+      </c>
+      <c r="L215" t="b">
+        <v>1</v>
+      </c>
+      <c r="M215" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B216" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C216" t="str">
+        <v>haitian-creole-your-background-05-which-language-do-you-speak</v>
+      </c>
+      <c r="D216">
+        <v>5</v>
+      </c>
+      <c r="E216" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Choose the Haitian Creole for "which language do you speak".</v>
+      </c>
+      <c r="G216" t="str">
+        <v>Ki lang ou pale?</v>
+      </c>
+      <c r="H216" t="str">
+        <v>["Ki kote ou soti?","Mwen soti...","Ki kote ou rete?"]</v>
+      </c>
+      <c r="I216" t="str">
+        <v>which-language-do-you-speak</v>
+      </c>
+      <c r="J216" t="str">
+        <v>["which-language-do-you-speak"]</v>
+      </c>
+      <c r="K216" t="str">
+        <v/>
+      </c>
+      <c r="L216" t="b">
+        <v>1</v>
+      </c>
+      <c r="M216" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B217" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C217" t="str">
+        <v>haitian-creole-your-background-06-which-language-do-you-speak</v>
+      </c>
+      <c r="D217">
+        <v>6</v>
+      </c>
+      <c r="E217" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F217" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G217" t="str">
+        <v>which language do you speak</v>
+      </c>
+      <c r="H217" t="str">
+        <v>["where are you from","i am from","where do you live"]</v>
+      </c>
+      <c r="I217" t="str">
+        <v>which-language-do-you-speak</v>
+      </c>
+      <c r="J217" t="str">
+        <v>["which-language-do-you-speak"]</v>
+      </c>
+      <c r="K217" t="str">
+        <v/>
+      </c>
+      <c r="L217" t="b">
+        <v>1</v>
+      </c>
+      <c r="M217" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B218" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C218" t="str">
+        <v>haitian-creole-family-members-01-family</v>
+      </c>
+      <c r="D218">
+        <v>1</v>
+      </c>
+      <c r="E218" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F218" t="str">
+        <v>What does "Fanmi" mean in Haitian Creole?</v>
+      </c>
+      <c r="G218" t="str">
+        <v>family</v>
+      </c>
+      <c r="H218" t="str">
+        <v>["parents","husband","wife"]</v>
+      </c>
+      <c r="I218" t="str">
+        <v>family</v>
+      </c>
+      <c r="J218" t="str">
+        <v>["family"]</v>
+      </c>
+      <c r="K218" t="str">
+        <v/>
+      </c>
+      <c r="L218" t="b">
+        <v>1</v>
+      </c>
+      <c r="M218" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B219" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C219" t="str">
+        <v>haitian-creole-family-members-02-parents</v>
+      </c>
+      <c r="D219">
+        <v>2</v>
+      </c>
+      <c r="E219" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F219" t="str">
+        <v>Build the Haitian Creole phrase for "parents".</v>
+      </c>
+      <c r="G219" t="str">
+        <v>Paran</v>
+      </c>
+      <c r="H219" t="str">
+        <v>["Fanmi","Mari","Madanm"]</v>
+      </c>
+      <c r="I219" t="str">
+        <v>parents</v>
+      </c>
+      <c r="J219" t="str">
+        <v>["parents"]</v>
+      </c>
+      <c r="K219" t="str">
+        <v/>
+      </c>
+      <c r="L219" t="b">
+        <v>1</v>
+      </c>
+      <c r="M219" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B220" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C220" t="str">
+        <v>haitian-creole-family-members-03-match</v>
+      </c>
+      <c r="D220">
+        <v>3</v>
+      </c>
+      <c r="E220" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F220" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G220" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H220" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I220" t="str">
+        <v/>
+      </c>
+      <c r="J220" t="str">
+        <v>["family","parents","husband","wife"]</v>
+      </c>
+      <c r="K220" t="str">
+        <v/>
+      </c>
+      <c r="L220" t="b">
+        <v>0</v>
+      </c>
+      <c r="M220" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B221" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C221" t="str">
+        <v>haitian-creole-family-members-04-wife</v>
+      </c>
+      <c r="D221">
+        <v>4</v>
+      </c>
+      <c r="E221" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F221" t="str">
+        <v>Build the English meaning of "Madanm".</v>
+      </c>
+      <c r="G221" t="str">
+        <v>wife</v>
+      </c>
+      <c r="H221" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I221" t="str">
+        <v>wife</v>
+      </c>
+      <c r="J221" t="str">
+        <v>["wife"]</v>
+      </c>
+      <c r="K221" t="str">
+        <v/>
+      </c>
+      <c r="L221" t="b">
+        <v>1</v>
+      </c>
+      <c r="M221" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B222" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C222" t="str">
+        <v>haitian-creole-family-members-05-son</v>
+      </c>
+      <c r="D222">
+        <v>5</v>
+      </c>
+      <c r="E222" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F222" t="str">
+        <v>Choose the Haitian Creole for "son".</v>
+      </c>
+      <c r="G222" t="str">
+        <v>Pitit gason</v>
+      </c>
+      <c r="H222" t="str">
+        <v>["Fanmi","Paran","Mari"]</v>
+      </c>
+      <c r="I222" t="str">
+        <v>son</v>
+      </c>
+      <c r="J222" t="str">
+        <v>["son"]</v>
+      </c>
+      <c r="K222" t="str">
+        <v/>
+      </c>
+      <c r="L222" t="b">
+        <v>1</v>
+      </c>
+      <c r="M222" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B223" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C223" t="str">
+        <v>haitian-creole-family-members-06-daughter</v>
+      </c>
+      <c r="D223">
+        <v>6</v>
+      </c>
+      <c r="E223" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F223" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G223" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="H223" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I223" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J223" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K223" t="str">
+        <v/>
+      </c>
+      <c r="L223" t="b">
+        <v>1</v>
+      </c>
+      <c r="M223" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B224" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C224" t="str">
+        <v>haitian-creole-family-members-07-grandfather</v>
+      </c>
+      <c r="D224">
+        <v>7</v>
+      </c>
+      <c r="E224" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F224" t="str">
+        <v>Choose the Haitian Creole for "grandfather".</v>
+      </c>
+      <c r="G224" t="str">
+        <v>Granpapa</v>
+      </c>
+      <c r="H224" t="str">
+        <v>["Fanmi","Paran","Mari"]</v>
+      </c>
+      <c r="I224" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="J224" t="str">
+        <v>["grandfather"]</v>
+      </c>
+      <c r="K224" t="str">
+        <v/>
+      </c>
+      <c r="L224" t="b">
+        <v>1</v>
+      </c>
+      <c r="M224" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B225" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C225" t="str">
+        <v>haitian-creole-family-members-08-grandfather</v>
+      </c>
+      <c r="D225">
+        <v>8</v>
+      </c>
+      <c r="E225" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F225" t="str">
+        <v>What does "Granpapa" mean in Haitian Creole?</v>
+      </c>
+      <c r="G225" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="H225" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I225" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="J225" t="str">
+        <v>["grandfather"]</v>
+      </c>
+      <c r="K225" t="str">
+        <v/>
+      </c>
+      <c r="L225" t="b">
+        <v>1</v>
+      </c>
+      <c r="M225" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B226" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C226" t="str">
+        <v>haitian-creole-polite-conversation-01-please</v>
+      </c>
+      <c r="D226">
+        <v>1</v>
+      </c>
+      <c r="E226" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F226" t="str">
+        <v>What does "Tanpri" mean in Haitian Creole?</v>
+      </c>
+      <c r="G226" t="str">
+        <v>please</v>
+      </c>
+      <c r="H226" t="str">
+        <v>["thank you","no problem","excuse me"]</v>
+      </c>
+      <c r="I226" t="str">
+        <v>please</v>
+      </c>
+      <c r="J226" t="str">
+        <v>["please"]</v>
+      </c>
+      <c r="K226" t="str">
+        <v/>
+      </c>
+      <c r="L226" t="b">
+        <v>1</v>
+      </c>
+      <c r="M226" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B227" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C227" t="str">
+        <v>haitian-creole-polite-conversation-02-thank-you</v>
+      </c>
+      <c r="D227">
+        <v>2</v>
+      </c>
+      <c r="E227" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F227" t="str">
+        <v>Build the Haitian Creole phrase for "thank you".</v>
+      </c>
+      <c r="G227" t="str">
+        <v>Mèsi</v>
+      </c>
+      <c r="H227" t="str">
+        <v>["Tanpri","Pa gen pwoblèm","Eskize m"]</v>
+      </c>
+      <c r="I227" t="str">
+        <v>thank-you</v>
+      </c>
+      <c r="J227" t="str">
+        <v>["thank-you"]</v>
+      </c>
+      <c r="K227" t="str">
+        <v/>
+      </c>
+      <c r="L227" t="b">
+        <v>1</v>
+      </c>
+      <c r="M227" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B228" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C228" t="str">
+        <v>haitian-creole-polite-conversation-03-match</v>
+      </c>
+      <c r="D228">
+        <v>3</v>
+      </c>
+      <c r="E228" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F228" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G228" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H228" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I228" t="str">
+        <v/>
+      </c>
+      <c r="J228" t="str">
+        <v>["please","thank-you","no-problem","excuse-me"]</v>
+      </c>
+      <c r="K228" t="str">
+        <v/>
+      </c>
+      <c r="L228" t="b">
+        <v>0</v>
+      </c>
+      <c r="M228" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B229" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C229" t="str">
+        <v>haitian-creole-polite-conversation-04-excuse-me</v>
+      </c>
+      <c r="D229">
+        <v>4</v>
+      </c>
+      <c r="E229" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F229" t="str">
+        <v>Build the English meaning of "Eskize m".</v>
+      </c>
+      <c r="G229" t="str">
+        <v>excuse me</v>
+      </c>
+      <c r="H229" t="str">
+        <v>["please","thank you","no problem"]</v>
+      </c>
+      <c r="I229" t="str">
+        <v>excuse-me</v>
+      </c>
+      <c r="J229" t="str">
+        <v>["excuse-me"]</v>
+      </c>
+      <c r="K229" t="str">
+        <v/>
+      </c>
+      <c r="L229" t="b">
+        <v>1</v>
+      </c>
+      <c r="M229" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B230" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C230" t="str">
+        <v>haitian-creole-polite-conversation-05-sorry</v>
+      </c>
+      <c r="D230">
+        <v>5</v>
+      </c>
+      <c r="E230" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F230" t="str">
+        <v>Choose the Haitian Creole for "sorry".</v>
+      </c>
+      <c r="G230" t="str">
+        <v>Mwen regrèt</v>
+      </c>
+      <c r="H230" t="str">
+        <v>["Tanpri","Mèsi","Pa gen pwoblèm"]</v>
+      </c>
+      <c r="I230" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="J230" t="str">
+        <v>["sorry"]</v>
+      </c>
+      <c r="K230" t="str">
+        <v/>
+      </c>
+      <c r="L230" t="b">
+        <v>1</v>
+      </c>
+      <c r="M230" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B231" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C231" t="str">
+        <v>haitian-creole-polite-conversation-06-sorry</v>
+      </c>
+      <c r="D231">
+        <v>6</v>
+      </c>
+      <c r="E231" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F231" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G231" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="H231" t="str">
+        <v>["please","thank you","no problem"]</v>
+      </c>
+      <c r="I231" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="J231" t="str">
+        <v>["sorry"]</v>
+      </c>
+      <c r="K231" t="str">
+        <v/>
+      </c>
+      <c r="L231" t="b">
+        <v>1</v>
+      </c>
+      <c r="M231" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B232" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C232" t="str">
+        <v>haitian-creole-introducing-others-01-this-is-my-family</v>
+      </c>
+      <c r="D232">
+        <v>1</v>
+      </c>
+      <c r="E232" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F232" t="str">
+        <v>What does "Sa a se fanmi mwen" mean in Haitian Creole?</v>
+      </c>
+      <c r="G232" t="str">
+        <v>this is my family</v>
+      </c>
+      <c r="H232" t="str">
+        <v>["this is my husband","this is my wife","he lives here"]</v>
+      </c>
+      <c r="I232" t="str">
+        <v>this-is-my-family</v>
+      </c>
+      <c r="J232" t="str">
+        <v>["this-is-my-family"]</v>
+      </c>
+      <c r="K232" t="str">
+        <v/>
+      </c>
+      <c r="L232" t="b">
+        <v>1</v>
+      </c>
+      <c r="M232" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B233" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C233" t="str">
+        <v>haitian-creole-introducing-others-02-this-is-my-husband</v>
+      </c>
+      <c r="D233">
+        <v>2</v>
+      </c>
+      <c r="E233" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F233" t="str">
+        <v>Build the Haitian Creole phrase for "this is my husband".</v>
+      </c>
+      <c r="G233" t="str">
+        <v>Sa a se mari mwen</v>
+      </c>
+      <c r="H233" t="str">
+        <v>["Sa a se fanmi mwen","Sa a se madanm mwen","Li rete isit la"]</v>
+      </c>
+      <c r="I233" t="str">
+        <v>this-is-my-husband</v>
+      </c>
+      <c r="J233" t="str">
+        <v>["this-is-my-husband"]</v>
+      </c>
+      <c r="K233" t="str">
+        <v/>
+      </c>
+      <c r="L233" t="b">
+        <v>1</v>
+      </c>
+      <c r="M233" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B234" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C234" t="str">
+        <v>haitian-creole-introducing-others-03-match</v>
+      </c>
+      <c r="D234">
+        <v>3</v>
+      </c>
+      <c r="E234" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F234" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G234" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H234" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I234" t="str">
+        <v/>
+      </c>
+      <c r="J234" t="str">
+        <v>["this-is-my-family","this-is-my-husband","this-is-my-wife","he-lives-here"]</v>
+      </c>
+      <c r="K234" t="str">
+        <v/>
+      </c>
+      <c r="L234" t="b">
+        <v>0</v>
+      </c>
+      <c r="M234" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B235" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C235" t="str">
+        <v>haitian-creole-introducing-others-04-he-lives-here</v>
+      </c>
+      <c r="D235">
+        <v>4</v>
+      </c>
+      <c r="E235" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F235" t="str">
+        <v>Build the English meaning of "Li rete isit la".</v>
+      </c>
+      <c r="G235" t="str">
+        <v>he lives here</v>
+      </c>
+      <c r="H235" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I235" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J235" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K235" t="str">
+        <v/>
+      </c>
+      <c r="L235" t="b">
+        <v>1</v>
+      </c>
+      <c r="M235" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B236" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C236" t="str">
+        <v>haitian-creole-introducing-others-05-she-works-here</v>
+      </c>
+      <c r="D236">
+        <v>5</v>
+      </c>
+      <c r="E236" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F236" t="str">
+        <v>Choose the Haitian Creole for "she works here".</v>
+      </c>
+      <c r="G236" t="str">
+        <v>Li travay isit la</v>
+      </c>
+      <c r="H236" t="str">
+        <v>["Sa a se fanmi mwen","Sa a se mari mwen","Sa a se madanm mwen"]</v>
+      </c>
+      <c r="I236" t="str">
+        <v>she-works-here</v>
+      </c>
+      <c r="J236" t="str">
+        <v>["she-works-here"]</v>
+      </c>
+      <c r="K236" t="str">
+        <v/>
+      </c>
+      <c r="L236" t="b">
+        <v>1</v>
+      </c>
+      <c r="M236" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B237" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C237" t="str">
+        <v>haitian-creole-introducing-others-06-we-speak</v>
+      </c>
+      <c r="D237">
+        <v>6</v>
+      </c>
+      <c r="E237" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F237" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G237" t="str">
+        <v>we speak</v>
+      </c>
+      <c r="H237" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I237" t="str">
+        <v>we-speak</v>
+      </c>
+      <c r="J237" t="str">
+        <v>["we-speak"]</v>
+      </c>
+      <c r="K237" t="str">
+        <v/>
+      </c>
+      <c r="L237" t="b">
+        <v>1</v>
+      </c>
+      <c r="M237" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B238" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C238" t="str">
+        <v>haitian-creole-introducing-others-07-they-are-from</v>
+      </c>
+      <c r="D238">
+        <v>7</v>
+      </c>
+      <c r="E238" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F238" t="str">
+        <v>Choose the Haitian Creole for "they are from".</v>
+      </c>
+      <c r="G238" t="str">
+        <v>Yo soti...</v>
+      </c>
+      <c r="H238" t="str">
+        <v>["Sa a se fanmi mwen","Sa a se mari mwen","Sa a se madanm mwen"]</v>
+      </c>
+      <c r="I238" t="str">
+        <v>they-are-from</v>
+      </c>
+      <c r="J238" t="str">
+        <v>["they-are-from"]</v>
+      </c>
+      <c r="K238" t="str">
+        <v/>
+      </c>
+      <c r="L238" t="b">
+        <v>1</v>
+      </c>
+      <c r="M238" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B239" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C239" t="str">
+        <v>haitian-creole-introducing-others-08-they-are-from</v>
+      </c>
+      <c r="D239">
+        <v>8</v>
+      </c>
+      <c r="E239" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F239" t="str">
+        <v>What does "Yo soti..." mean in Haitian Creole?</v>
+      </c>
+      <c r="G239" t="str">
+        <v>they are from</v>
+      </c>
+      <c r="H239" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I239" t="str">
+        <v>they-are-from</v>
+      </c>
+      <c r="J239" t="str">
+        <v>["they-are-from"]</v>
+      </c>
+      <c r="K239" t="str">
+        <v/>
+      </c>
+      <c r="L239" t="b">
+        <v>1</v>
+      </c>
+      <c r="M239" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B240" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C240" t="str">
+        <v>haitian-creole-words-practice-01-yes</v>
+      </c>
+      <c r="D240">
+        <v>1</v>
+      </c>
+      <c r="E240" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F240" t="str">
+        <v>What does "Wi" mean in Haitian Creole?</v>
+      </c>
+      <c r="G240" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H240" t="str">
+        <v>["good afternoon","what is your name","where are you from"]</v>
+      </c>
+      <c r="I240" t="str">
+        <v>yes</v>
+      </c>
+      <c r="J240" t="str">
+        <v>["yes"]</v>
+      </c>
+      <c r="K240" t="str">
+        <v/>
+      </c>
+      <c r="L240" t="b">
+        <v>0</v>
+      </c>
+      <c r="M240" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B241" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C241" t="str">
+        <v>haitian-creole-words-practice-02-good-afternoon</v>
+      </c>
+      <c r="D241">
+        <v>2</v>
+      </c>
+      <c r="E241" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F241" t="str">
+        <v>Build the Haitian Creole phrase for "good afternoon".</v>
+      </c>
+      <c r="G241" t="str">
+        <v>Bon apremidi</v>
+      </c>
+      <c r="H241" t="str">
+        <v>["Wi","Kijan ou rele?","Ki kote ou soti?"]</v>
+      </c>
+      <c r="I241" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J241" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K241" t="str">
+        <v/>
+      </c>
+      <c r="L241" t="b">
+        <v>0</v>
+      </c>
+      <c r="M241" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B242" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C242" t="str">
+        <v>haitian-creole-words-practice-03-match</v>
+      </c>
+      <c r="D242">
+        <v>3</v>
+      </c>
+      <c r="E242" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F242" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G242" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H242" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I242" t="str">
+        <v/>
+      </c>
+      <c r="J242" t="str">
+        <v>["yes","good-afternoon","what-is-your-name","where-are-you-from"]</v>
+      </c>
+      <c r="K242" t="str">
+        <v/>
+      </c>
+      <c r="L242" t="b">
+        <v>0</v>
+      </c>
+      <c r="M242" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B243" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C243" t="str">
+        <v>haitian-creole-words-practice-04-where-are-you-from</v>
+      </c>
+      <c r="D243">
+        <v>4</v>
+      </c>
+      <c r="E243" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F243" t="str">
+        <v>Build the English meaning of "Ki kote ou soti?".</v>
+      </c>
+      <c r="G243" t="str">
+        <v>where are you from</v>
+      </c>
+      <c r="H243" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I243" t="str">
+        <v>where-are-you-from</v>
+      </c>
+      <c r="J243" t="str">
+        <v>["where-are-you-from"]</v>
+      </c>
+      <c r="K243" t="str">
+        <v/>
+      </c>
+      <c r="L243" t="b">
+        <v>0</v>
+      </c>
+      <c r="M243" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B244" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C244" t="str">
+        <v>haitian-creole-words-practice-05-family</v>
+      </c>
+      <c r="D244">
+        <v>5</v>
+      </c>
+      <c r="E244" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F244" t="str">
+        <v>Choose the Haitian Creole for "family".</v>
+      </c>
+      <c r="G244" t="str">
+        <v>Fanmi</v>
+      </c>
+      <c r="H244" t="str">
+        <v>["Wi","Bon apremidi","Kijan ou rele?"]</v>
+      </c>
+      <c r="I244" t="str">
+        <v>family</v>
+      </c>
+      <c r="J244" t="str">
+        <v>["family"]</v>
+      </c>
+      <c r="K244" t="str">
+        <v/>
+      </c>
+      <c r="L244" t="b">
+        <v>0</v>
+      </c>
+      <c r="M244" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B245" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C245" t="str">
+        <v>haitian-creole-words-practice-06-daughter</v>
+      </c>
+      <c r="D245">
+        <v>6</v>
+      </c>
+      <c r="E245" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F245" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G245" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="H245" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I245" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J245" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K245" t="str">
+        <v/>
+      </c>
+      <c r="L245" t="b">
+        <v>0</v>
+      </c>
+      <c r="M245" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B246" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C246" t="str">
+        <v>haitian-creole-words-practice-07-excuse-me</v>
+      </c>
+      <c r="D246">
+        <v>7</v>
+      </c>
+      <c r="E246" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F246" t="str">
+        <v>Choose the Haitian Creole for "excuse me".</v>
+      </c>
+      <c r="G246" t="str">
+        <v>Eskize m</v>
+      </c>
+      <c r="H246" t="str">
+        <v>["Wi","Bon apremidi","Kijan ou rele?"]</v>
+      </c>
+      <c r="I246" t="str">
+        <v>excuse-me</v>
+      </c>
+      <c r="J246" t="str">
+        <v>["excuse-me"]</v>
+      </c>
+      <c r="K246" t="str">
+        <v/>
+      </c>
+      <c r="L246" t="b">
+        <v>0</v>
+      </c>
+      <c r="M246" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B247" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C247" t="str">
+        <v>haitian-creole-words-practice-08-he-lives-here</v>
+      </c>
+      <c r="D247">
+        <v>8</v>
+      </c>
+      <c r="E247" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F247" t="str">
+        <v>What does "Li rete isit la" mean in Haitian Creole?</v>
+      </c>
+      <c r="G247" t="str">
+        <v>he lives here</v>
+      </c>
+      <c r="H247" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I247" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J247" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K247" t="str">
+        <v/>
+      </c>
+      <c r="L247" t="b">
+        <v>0</v>
+      </c>
+      <c r="M247" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B248" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C248" t="str">
+        <v>haitian-creole-words-practice-09-he-lives-here</v>
+      </c>
+      <c r="D248">
+        <v>9</v>
+      </c>
+      <c r="E248" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F248" t="str">
+        <v>Choose the Haitian Creole for "he lives here".</v>
+      </c>
+      <c r="G248" t="str">
+        <v>Li rete isit la</v>
+      </c>
+      <c r="H248" t="str">
+        <v>["Wi","Bon apremidi","Kijan ou rele?"]</v>
+      </c>
+      <c r="I248" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J248" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K248" t="str">
+        <v/>
+      </c>
+      <c r="L248" t="b">
+        <v>0</v>
+      </c>
+      <c r="M248" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B249" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C249" t="str">
+        <v>haitian-creole-practice-challenge-01-no</v>
+      </c>
+      <c r="D249">
+        <v>1</v>
+      </c>
+      <c r="E249" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F249" t="str">
+        <v>What does "Non" mean in Haitian Creole?</v>
+      </c>
+      <c r="G249" t="str">
+        <v>no</v>
+      </c>
+      <c r="H249" t="str">
+        <v>["good afternoon","have a good day","i am learning"]</v>
+      </c>
+      <c r="I249" t="str">
+        <v>no</v>
+      </c>
+      <c r="J249" t="str">
+        <v>["no"]</v>
+      </c>
+      <c r="K249" t="str">
+        <v/>
+      </c>
+      <c r="L249" t="b">
+        <v>0</v>
+      </c>
+      <c r="M249" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B250" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C250" t="str">
+        <v>haitian-creole-practice-challenge-02-good-afternoon</v>
+      </c>
+      <c r="D250">
+        <v>2</v>
+      </c>
+      <c r="E250" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F250" t="str">
+        <v>Build the Haitian Creole phrase for "good afternoon".</v>
+      </c>
+      <c r="G250" t="str">
+        <v>Bon apremidi</v>
+      </c>
+      <c r="H250" t="str">
+        <v>["Non","Pase yon bon jounen","M ap aprann..."]</v>
+      </c>
+      <c r="I250" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J250" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K250" t="str">
+        <v/>
+      </c>
+      <c r="L250" t="b">
+        <v>0</v>
+      </c>
+      <c r="M250" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B251" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C251" t="str">
+        <v>haitian-creole-practice-challenge-03-match</v>
+      </c>
+      <c r="D251">
+        <v>3</v>
+      </c>
+      <c r="E251" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F251" t="str">
+        <v>Match each Haitian Creole phrase to its meaning.</v>
+      </c>
+      <c r="G251" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H251" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I251" t="str">
+        <v/>
+      </c>
+      <c r="J251" t="str">
+        <v>["no","good-afternoon","have-a-good-day","i-am-learning"]</v>
+      </c>
+      <c r="K251" t="str">
+        <v/>
+      </c>
+      <c r="L251" t="b">
+        <v>0</v>
+      </c>
+      <c r="M251" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B252" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C252" t="str">
+        <v>haitian-creole-practice-challenge-04-i-am-learning</v>
+      </c>
+      <c r="D252">
+        <v>4</v>
+      </c>
+      <c r="E252" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F252" t="str">
+        <v>Build the English meaning of "M ap aprann...".</v>
+      </c>
+      <c r="G252" t="str">
+        <v>i am learning</v>
+      </c>
+      <c r="H252" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I252" t="str">
+        <v>i-am-learning</v>
+      </c>
+      <c r="J252" t="str">
+        <v>["i-am-learning"]</v>
+      </c>
+      <c r="K252" t="str">
+        <v/>
+      </c>
+      <c r="L252" t="b">
+        <v>0</v>
+      </c>
+      <c r="M252" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B253" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C253" t="str">
+        <v>haitian-creole-practice-challenge-05-where-do-you-live</v>
+      </c>
+      <c r="D253">
+        <v>5</v>
+      </c>
+      <c r="E253" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F253" t="str">
+        <v>Choose the Haitian Creole for "where do you live".</v>
+      </c>
+      <c r="G253" t="str">
+        <v>Ki kote ou rete?</v>
+      </c>
+      <c r="H253" t="str">
+        <v>["Non","Bon apremidi","Pase yon bon jounen"]</v>
+      </c>
+      <c r="I253" t="str">
+        <v>where-do-you-live</v>
+      </c>
+      <c r="J253" t="str">
+        <v>["where-do-you-live"]</v>
+      </c>
+      <c r="K253" t="str">
+        <v/>
+      </c>
+      <c r="L253" t="b">
+        <v>0</v>
+      </c>
+      <c r="M253" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B254" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C254" t="str">
+        <v>haitian-creole-practice-challenge-06-parents</v>
+      </c>
+      <c r="D254">
+        <v>6</v>
+      </c>
+      <c r="E254" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F254" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G254" t="str">
+        <v>parents</v>
+      </c>
+      <c r="H254" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I254" t="str">
+        <v>parents</v>
+      </c>
+      <c r="J254" t="str">
+        <v>["parents"]</v>
+      </c>
+      <c r="K254" t="str">
+        <v/>
+      </c>
+      <c r="L254" t="b">
+        <v>0</v>
+      </c>
+      <c r="M254" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B255" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C255" t="str">
+        <v>haitian-creole-practice-challenge-07-daughter</v>
+      </c>
+      <c r="D255">
+        <v>7</v>
+      </c>
+      <c r="E255" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F255" t="str">
+        <v>Choose the Haitian Creole for "daughter".</v>
+      </c>
+      <c r="G255" t="str">
+        <v>Pitit fi</v>
+      </c>
+      <c r="H255" t="str">
+        <v>["Non","Bon apremidi","Pase yon bon jounen"]</v>
+      </c>
+      <c r="I255" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J255" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K255" t="str">
+        <v/>
+      </c>
+      <c r="L255" t="b">
+        <v>0</v>
+      </c>
+      <c r="M255" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B256" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C256" t="str">
+        <v>haitian-creole-practice-challenge-08-no-problem</v>
+      </c>
+      <c r="D256">
+        <v>8</v>
+      </c>
+      <c r="E256" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F256" t="str">
+        <v>What does "Pa gen pwoblèm" mean in Haitian Creole?</v>
+      </c>
+      <c r="G256" t="str">
+        <v>no problem</v>
+      </c>
+      <c r="H256" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I256" t="str">
+        <v>no-problem</v>
+      </c>
+      <c r="J256" t="str">
+        <v>["no-problem"]</v>
+      </c>
+      <c r="K256" t="str">
+        <v/>
+      </c>
+      <c r="L256" t="b">
+        <v>0</v>
+      </c>
+      <c r="M256" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>haitian-creole</v>
+      </c>
+      <c r="B257" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C257" t="str">
+        <v>haitian-creole-practice-challenge-09-no-problem</v>
+      </c>
+      <c r="D257">
+        <v>9</v>
+      </c>
+      <c r="E257" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F257" t="str">
+        <v>Choose the Haitian Creole for "no problem".</v>
+      </c>
+      <c r="G257" t="str">
+        <v>Pa gen pwoblèm</v>
+      </c>
+      <c r="H257" t="str">
+        <v>["Non","Bon apremidi","Pase yon bon jounen"]</v>
+      </c>
+      <c r="I257" t="str">
+        <v>no-problem</v>
+      </c>
+      <c r="J257" t="str">
+        <v>["no-problem"]</v>
+      </c>
+      <c r="K257" t="str">
+        <v/>
+      </c>
+      <c r="L257" t="b">
+        <v>0</v>
+      </c>
+      <c r="M257" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M193"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M257"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Stage Sudanese Arabic candidate course artwork
</commit_message>
<xml_diff>
--- a/patois_learn_database_1.xlsx
+++ b/patois_learn_database_1.xlsx
@@ -6431,25 +6431,25 @@
         <v>yes</v>
       </c>
       <c r="C158" t="str">
-        <v/>
+        <v>أيوه</v>
       </c>
       <c r="D158" t="str">
-        <v/>
+        <v>aywa</v>
       </c>
       <c r="E158" t="str">
-        <v/>
+        <v>Khartoum colloquial yes</v>
       </c>
       <c r="F158" t="str">
         <v>assets/images/vocab/sudanese-arabic/yes.png</v>
       </c>
       <c r="G158" t="str">
-        <v>assets/audio/sudanese-arabic/yes.mp3</v>
+        <v/>
       </c>
       <c r="H158" t="str">
         <v/>
       </c>
       <c r="I158" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J158" t="str">
         <v>unavailable</v>
@@ -6463,25 +6463,25 @@
         <v>no</v>
       </c>
       <c r="C159" t="str">
-        <v/>
+        <v>لا</v>
       </c>
       <c r="D159" t="str">
-        <v/>
+        <v>la</v>
       </c>
       <c r="E159" t="str">
-        <v/>
+        <v>Arabic script</v>
       </c>
       <c r="F159" t="str">
         <v>assets/images/vocab/sudanese-arabic/no.png</v>
       </c>
       <c r="G159" t="str">
-        <v>assets/audio/sudanese-arabic/no.mp3</v>
+        <v/>
       </c>
       <c r="H159" t="str">
         <v/>
       </c>
       <c r="I159" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J159" t="str">
         <v>unavailable</v>
@@ -6495,25 +6495,25 @@
         <v>maybe</v>
       </c>
       <c r="C160" t="str">
-        <v/>
+        <v>يمكن</v>
       </c>
       <c r="D160" t="str">
-        <v/>
+        <v>yimkin</v>
       </c>
       <c r="E160" t="str">
-        <v/>
+        <v>Khartoum colloquial maybe</v>
       </c>
       <c r="F160" t="str">
         <v>assets/images/vocab/sudanese-arabic/maybe.png</v>
       </c>
       <c r="G160" t="str">
-        <v>assets/audio/sudanese-arabic/maybe.mp3</v>
+        <v/>
       </c>
       <c r="H160" t="str">
         <v/>
       </c>
       <c r="I160" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J160" t="str">
         <v>unavailable</v>
@@ -6527,25 +6527,25 @@
         <v>okay</v>
       </c>
       <c r="C161" t="str">
-        <v/>
+        <v>تمام</v>
       </c>
       <c r="D161" t="str">
-        <v/>
+        <v>tamam</v>
       </c>
       <c r="E161" t="str">
-        <v/>
+        <v>Common Sudanese agreement</v>
       </c>
       <c r="F161" t="str">
         <v>assets/images/vocab/sudanese-arabic/okay.png</v>
       </c>
       <c r="G161" t="str">
-        <v>assets/audio/sudanese-arabic/okay.mp3</v>
+        <v/>
       </c>
       <c r="H161" t="str">
         <v/>
       </c>
       <c r="I161" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J161" t="str">
         <v>unavailable</v>
@@ -6559,25 +6559,25 @@
         <v>again</v>
       </c>
       <c r="C162" t="str">
-        <v/>
+        <v>تاني</v>
       </c>
       <c r="D162" t="str">
-        <v/>
+        <v>tani</v>
       </c>
       <c r="E162" t="str">
-        <v/>
+        <v>Sudanese colloquial again</v>
       </c>
       <c r="F162" t="str">
         <v>assets/images/vocab/sudanese-arabic/again.png</v>
       </c>
       <c r="G162" t="str">
-        <v>assets/audio/sudanese-arabic/again.mp3</v>
+        <v/>
       </c>
       <c r="H162" t="str">
         <v/>
       </c>
       <c r="I162" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J162" t="str">
         <v>unavailable</v>
@@ -6591,25 +6591,25 @@
         <v>good-afternoon</v>
       </c>
       <c r="C163" t="str">
-        <v/>
+        <v>مساء الخير</v>
       </c>
       <c r="D163" t="str">
-        <v/>
+        <v>masa al-kheir</v>
       </c>
       <c r="E163" t="str">
-        <v/>
+        <v>Afternoon/evening greeting</v>
       </c>
       <c r="F163" t="str">
         <v>assets/images/vocab/sudanese-arabic/good-afternoon.png</v>
       </c>
       <c r="G163" t="str">
-        <v>assets/audio/sudanese-arabic/good-afternoon.mp3</v>
+        <v/>
       </c>
       <c r="H163" t="str">
         <v/>
       </c>
       <c r="I163" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J163" t="str">
         <v>unavailable</v>
@@ -6623,25 +6623,25 @@
         <v>nice-to-meet-you</v>
       </c>
       <c r="C164" t="str">
-        <v/>
+        <v>اتشرفت بيك</v>
       </c>
       <c r="D164" t="str">
-        <v/>
+        <v>it-sharraft beek</v>
       </c>
       <c r="E164" t="str">
-        <v/>
+        <v>Polite meeting phrase</v>
       </c>
       <c r="F164" t="str">
         <v>assets/images/vocab/sudanese-arabic/nice-to-meet-you.png</v>
       </c>
       <c r="G164" t="str">
-        <v>assets/audio/sudanese-arabic/nice-to-meet-you.mp3</v>
+        <v/>
       </c>
       <c r="H164" t="str">
         <v/>
       </c>
       <c r="I164" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J164" t="str">
         <v>unavailable</v>
@@ -6655,25 +6655,25 @@
         <v>long-time-no-see</v>
       </c>
       <c r="C165" t="str">
-        <v/>
+        <v>زمن ما شفناك</v>
       </c>
       <c r="D165" t="str">
-        <v/>
+        <v>zaman ma shufnak</v>
       </c>
       <c r="E165" t="str">
-        <v/>
+        <v>Long time no see</v>
       </c>
       <c r="F165" t="str">
         <v>assets/images/vocab/sudanese-arabic/long-time-no-see.png</v>
       </c>
       <c r="G165" t="str">
-        <v>assets/audio/sudanese-arabic/long-time-no-see.mp3</v>
+        <v/>
       </c>
       <c r="H165" t="str">
         <v/>
       </c>
       <c r="I165" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J165" t="str">
         <v>unavailable</v>
@@ -6687,25 +6687,25 @@
         <v>how-is-your-day</v>
       </c>
       <c r="C166" t="str">
-        <v/>
+        <v>يومك كيف؟</v>
       </c>
       <c r="D166" t="str">
-        <v/>
+        <v>yomak keef?</v>
       </c>
       <c r="E166" t="str">
-        <v/>
+        <v>How is your day?</v>
       </c>
       <c r="F166" t="str">
         <v>assets/images/vocab/sudanese-arabic/how-is-your-day.png</v>
       </c>
       <c r="G166" t="str">
-        <v>assets/audio/sudanese-arabic/how-is-your-day.mp3</v>
+        <v/>
       </c>
       <c r="H166" t="str">
         <v/>
       </c>
       <c r="I166" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J166" t="str">
         <v>unavailable</v>
@@ -6719,25 +6719,25 @@
         <v>have-a-good-day</v>
       </c>
       <c r="C167" t="str">
-        <v/>
+        <v>يومك سعيد</v>
       </c>
       <c r="D167" t="str">
-        <v/>
+        <v>yomak saeed</v>
       </c>
       <c r="E167" t="str">
-        <v/>
+        <v>Have a good day</v>
       </c>
       <c r="F167" t="str">
         <v>assets/images/vocab/sudanese-arabic/have-a-good-day.png</v>
       </c>
       <c r="G167" t="str">
-        <v>assets/audio/sudanese-arabic/have-a-good-day.mp3</v>
+        <v/>
       </c>
       <c r="H167" t="str">
         <v/>
       </c>
       <c r="I167" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J167" t="str">
         <v>unavailable</v>
@@ -6751,25 +6751,25 @@
         <v>what-is-your-name</v>
       </c>
       <c r="C168" t="str">
-        <v/>
+        <v>اسمك منو؟</v>
       </c>
       <c r="D168" t="str">
-        <v/>
+        <v>ismak minu?</v>
       </c>
       <c r="E168" t="str">
-        <v/>
+        <v>What is your name?</v>
       </c>
       <c r="F168" t="str">
         <v>assets/images/vocab/sudanese-arabic/what-is-your-name.png</v>
       </c>
       <c r="G168" t="str">
-        <v>assets/audio/sudanese-arabic/what-is-your-name.mp3</v>
+        <v/>
       </c>
       <c r="H168" t="str">
         <v/>
       </c>
       <c r="I168" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J168" t="str">
         <v>unavailable</v>
@@ -6783,25 +6783,25 @@
         <v>my-name-is</v>
       </c>
       <c r="C169" t="str">
-        <v/>
+        <v>اسمي...</v>
       </c>
       <c r="D169" t="str">
-        <v/>
+        <v>ismi...</v>
       </c>
       <c r="E169" t="str">
-        <v/>
+        <v>My name is...</v>
       </c>
       <c r="F169" t="str">
         <v>assets/images/vocab/sudanese-arabic/my-name-is.png</v>
       </c>
       <c r="G169" t="str">
-        <v>assets/audio/sudanese-arabic/my-name-is.mp3</v>
+        <v/>
       </c>
       <c r="H169" t="str">
         <v/>
       </c>
       <c r="I169" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J169" t="str">
         <v>unavailable</v>
@@ -6815,25 +6815,25 @@
         <v>i-am-a-student</v>
       </c>
       <c r="C170" t="str">
-        <v/>
+        <v>أنا طالب</v>
       </c>
       <c r="D170" t="str">
-        <v/>
+        <v>ana talib</v>
       </c>
       <c r="E170" t="str">
-        <v/>
+        <v>I am a student</v>
       </c>
       <c r="F170" t="str">
         <v>assets/images/vocab/sudanese-arabic/i-am-a-student.png</v>
       </c>
       <c r="G170" t="str">
-        <v>assets/audio/sudanese-arabic/i-am-a-student.mp3</v>
+        <v/>
       </c>
       <c r="H170" t="str">
         <v/>
       </c>
       <c r="I170" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J170" t="str">
         <v>unavailable</v>
@@ -6847,25 +6847,25 @@
         <v>i-am-learning</v>
       </c>
       <c r="C171" t="str">
-        <v/>
+        <v>أنا بتعلم...</v>
       </c>
       <c r="D171" t="str">
-        <v/>
+        <v>ana batallam...</v>
       </c>
       <c r="E171" t="str">
-        <v/>
+        <v>I am learning...</v>
       </c>
       <c r="F171" t="str">
         <v>assets/images/vocab/sudanese-arabic/i-am-learning.png</v>
       </c>
       <c r="G171" t="str">
-        <v>assets/audio/sudanese-arabic/i-am-learning.mp3</v>
+        <v/>
       </c>
       <c r="H171" t="str">
         <v/>
       </c>
       <c r="I171" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J171" t="str">
         <v>unavailable</v>
@@ -6879,25 +6879,25 @@
         <v>i-speak</v>
       </c>
       <c r="C172" t="str">
-        <v/>
+        <v>أنا بتكلم...</v>
       </c>
       <c r="D172" t="str">
-        <v/>
+        <v>ana batakallam...</v>
       </c>
       <c r="E172" t="str">
-        <v/>
+        <v>I speak...</v>
       </c>
       <c r="F172" t="str">
         <v>assets/images/vocab/sudanese-arabic/i-speak.png</v>
       </c>
       <c r="G172" t="str">
-        <v>assets/audio/sudanese-arabic/i-speak.mp3</v>
+        <v/>
       </c>
       <c r="H172" t="str">
         <v/>
       </c>
       <c r="I172" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J172" t="str">
         <v>unavailable</v>
@@ -6911,25 +6911,25 @@
         <v>where-are-you-from</v>
       </c>
       <c r="C173" t="str">
-        <v/>
+        <v>إنت من وين؟</v>
       </c>
       <c r="D173" t="str">
-        <v/>
+        <v>inta min wein?</v>
       </c>
       <c r="E173" t="str">
-        <v/>
+        <v>Where are you from?</v>
       </c>
       <c r="F173" t="str">
         <v>assets/images/vocab/sudanese-arabic/where-are-you-from.png</v>
       </c>
       <c r="G173" t="str">
-        <v>assets/audio/sudanese-arabic/where-are-you-from.mp3</v>
+        <v/>
       </c>
       <c r="H173" t="str">
         <v/>
       </c>
       <c r="I173" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J173" t="str">
         <v>unavailable</v>
@@ -6943,25 +6943,25 @@
         <v>i-am-from</v>
       </c>
       <c r="C174" t="str">
-        <v/>
+        <v>أنا من...</v>
       </c>
       <c r="D174" t="str">
-        <v/>
+        <v>ana min...</v>
       </c>
       <c r="E174" t="str">
-        <v/>
+        <v>I am from...</v>
       </c>
       <c r="F174" t="str">
         <v>assets/images/vocab/sudanese-arabic/i-am-from.png</v>
       </c>
       <c r="G174" t="str">
-        <v>assets/audio/sudanese-arabic/i-am-from.mp3</v>
+        <v/>
       </c>
       <c r="H174" t="str">
         <v/>
       </c>
       <c r="I174" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J174" t="str">
         <v>unavailable</v>
@@ -6975,25 +6975,25 @@
         <v>where-do-you-live</v>
       </c>
       <c r="C175" t="str">
-        <v/>
+        <v>ساكن وين؟</v>
       </c>
       <c r="D175" t="str">
-        <v/>
+        <v>sakin wein?</v>
       </c>
       <c r="E175" t="str">
-        <v/>
+        <v>Where do you live?</v>
       </c>
       <c r="F175" t="str">
         <v>assets/images/vocab/sudanese-arabic/where-do-you-live.png</v>
       </c>
       <c r="G175" t="str">
-        <v>assets/audio/sudanese-arabic/where-do-you-live.mp3</v>
+        <v/>
       </c>
       <c r="H175" t="str">
         <v/>
       </c>
       <c r="I175" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J175" t="str">
         <v>unavailable</v>
@@ -7007,25 +7007,25 @@
         <v>i-live-in</v>
       </c>
       <c r="C176" t="str">
-        <v/>
+        <v>ساكن في...</v>
       </c>
       <c r="D176" t="str">
-        <v/>
+        <v>sakin fi...</v>
       </c>
       <c r="E176" t="str">
-        <v/>
+        <v>I live in...</v>
       </c>
       <c r="F176" t="str">
         <v>assets/images/vocab/sudanese-arabic/i-live-in.png</v>
       </c>
       <c r="G176" t="str">
-        <v>assets/audio/sudanese-arabic/i-live-in.mp3</v>
+        <v/>
       </c>
       <c r="H176" t="str">
         <v/>
       </c>
       <c r="I176" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J176" t="str">
         <v>unavailable</v>
@@ -7039,25 +7039,25 @@
         <v>which-language-do-you-speak</v>
       </c>
       <c r="C177" t="str">
-        <v/>
+        <v>بتتكلم ياتو لغة؟</v>
       </c>
       <c r="D177" t="str">
-        <v/>
+        <v>bititkallam yatu lughah?</v>
       </c>
       <c r="E177" t="str">
-        <v/>
+        <v>Which language do you speak?</v>
       </c>
       <c r="F177" t="str">
         <v>assets/images/vocab/sudanese-arabic/which-language-do-you-speak.png</v>
       </c>
       <c r="G177" t="str">
-        <v>assets/audio/sudanese-arabic/which-language-do-you-speak.mp3</v>
+        <v/>
       </c>
       <c r="H177" t="str">
         <v/>
       </c>
       <c r="I177" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J177" t="str">
         <v>unavailable</v>
@@ -7071,25 +7071,25 @@
         <v>family</v>
       </c>
       <c r="C178" t="str">
-        <v/>
+        <v>أسرة</v>
       </c>
       <c r="D178" t="str">
-        <v/>
+        <v>usra</v>
       </c>
       <c r="E178" t="str">
-        <v/>
+        <v>Family</v>
       </c>
       <c r="F178" t="str">
         <v>assets/images/vocab/sudanese-arabic/family.png</v>
       </c>
       <c r="G178" t="str">
-        <v>assets/audio/sudanese-arabic/family.mp3</v>
+        <v/>
       </c>
       <c r="H178" t="str">
         <v/>
       </c>
       <c r="I178" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J178" t="str">
         <v>unavailable</v>
@@ -7103,25 +7103,25 @@
         <v>parents</v>
       </c>
       <c r="C179" t="str">
-        <v/>
+        <v>الأهل</v>
       </c>
       <c r="D179" t="str">
-        <v/>
+        <v>al-ahl</v>
       </c>
       <c r="E179" t="str">
-        <v/>
+        <v>Parents/family elders</v>
       </c>
       <c r="F179" t="str">
         <v>assets/images/vocab/sudanese-arabic/parents.png</v>
       </c>
       <c r="G179" t="str">
-        <v>assets/audio/sudanese-arabic/parents.mp3</v>
+        <v/>
       </c>
       <c r="H179" t="str">
         <v/>
       </c>
       <c r="I179" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J179" t="str">
         <v>unavailable</v>
@@ -7135,25 +7135,25 @@
         <v>husband</v>
       </c>
       <c r="C180" t="str">
-        <v/>
+        <v>زوج</v>
       </c>
       <c r="D180" t="str">
-        <v/>
+        <v>zawj</v>
       </c>
       <c r="E180" t="str">
-        <v/>
+        <v>Husband</v>
       </c>
       <c r="F180" t="str">
         <v>assets/images/vocab/sudanese-arabic/husband.png</v>
       </c>
       <c r="G180" t="str">
-        <v>assets/audio/sudanese-arabic/husband.mp3</v>
+        <v/>
       </c>
       <c r="H180" t="str">
         <v/>
       </c>
       <c r="I180" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J180" t="str">
         <v>unavailable</v>
@@ -7167,25 +7167,25 @@
         <v>wife</v>
       </c>
       <c r="C181" t="str">
-        <v/>
+        <v>زوجة</v>
       </c>
       <c r="D181" t="str">
-        <v/>
+        <v>zawjah</v>
       </c>
       <c r="E181" t="str">
-        <v/>
+        <v>Wife</v>
       </c>
       <c r="F181" t="str">
         <v>assets/images/vocab/sudanese-arabic/wife.png</v>
       </c>
       <c r="G181" t="str">
-        <v>assets/audio/sudanese-arabic/wife.mp3</v>
+        <v/>
       </c>
       <c r="H181" t="str">
         <v/>
       </c>
       <c r="I181" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J181" t="str">
         <v>unavailable</v>
@@ -7199,25 +7199,25 @@
         <v>son</v>
       </c>
       <c r="C182" t="str">
-        <v/>
+        <v>ولد</v>
       </c>
       <c r="D182" t="str">
-        <v/>
+        <v>walad</v>
       </c>
       <c r="E182" t="str">
-        <v/>
+        <v>Son/boy</v>
       </c>
       <c r="F182" t="str">
         <v>assets/images/vocab/sudanese-arabic/son.png</v>
       </c>
       <c r="G182" t="str">
-        <v>assets/audio/sudanese-arabic/son.mp3</v>
+        <v/>
       </c>
       <c r="H182" t="str">
         <v/>
       </c>
       <c r="I182" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J182" t="str">
         <v>unavailable</v>
@@ -7231,25 +7231,25 @@
         <v>daughter</v>
       </c>
       <c r="C183" t="str">
-        <v/>
+        <v>بنت</v>
       </c>
       <c r="D183" t="str">
-        <v/>
+        <v>bint</v>
       </c>
       <c r="E183" t="str">
-        <v/>
+        <v>Daughter/girl</v>
       </c>
       <c r="F183" t="str">
         <v>assets/images/vocab/sudanese-arabic/daughter.png</v>
       </c>
       <c r="G183" t="str">
-        <v>assets/audio/sudanese-arabic/daughter.mp3</v>
+        <v/>
       </c>
       <c r="H183" t="str">
         <v/>
       </c>
       <c r="I183" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J183" t="str">
         <v>unavailable</v>
@@ -7263,25 +7263,25 @@
         <v>grandfather</v>
       </c>
       <c r="C184" t="str">
-        <v/>
+        <v>جد</v>
       </c>
       <c r="D184" t="str">
-        <v/>
+        <v>jadd</v>
       </c>
       <c r="E184" t="str">
-        <v/>
+        <v>Grandfather</v>
       </c>
       <c r="F184" t="str">
         <v>assets/images/vocab/sudanese-arabic/grandfather.png</v>
       </c>
       <c r="G184" t="str">
-        <v>assets/audio/sudanese-arabic/grandfather.mp3</v>
+        <v/>
       </c>
       <c r="H184" t="str">
         <v/>
       </c>
       <c r="I184" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J184" t="str">
         <v>unavailable</v>
@@ -7295,25 +7295,25 @@
         <v>please</v>
       </c>
       <c r="C185" t="str">
-        <v/>
+        <v>لو سمحت</v>
       </c>
       <c r="D185" t="str">
-        <v/>
+        <v>law samaht</v>
       </c>
       <c r="E185" t="str">
-        <v/>
+        <v>Please</v>
       </c>
       <c r="F185" t="str">
         <v>assets/images/vocab/sudanese-arabic/please.png</v>
       </c>
       <c r="G185" t="str">
-        <v>assets/audio/sudanese-arabic/please.mp3</v>
+        <v/>
       </c>
       <c r="H185" t="str">
         <v/>
       </c>
       <c r="I185" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J185" t="str">
         <v>unavailable</v>
@@ -7327,25 +7327,25 @@
         <v>thank-you</v>
       </c>
       <c r="C186" t="str">
-        <v/>
+        <v>شكراً</v>
       </c>
       <c r="D186" t="str">
-        <v/>
+        <v>shukran</v>
       </c>
       <c r="E186" t="str">
-        <v/>
+        <v>Thank you</v>
       </c>
       <c r="F186" t="str">
         <v>assets/images/vocab/sudanese-arabic/thank-you.png</v>
       </c>
       <c r="G186" t="str">
-        <v>assets/audio/sudanese-arabic/thank-you.mp3</v>
+        <v/>
       </c>
       <c r="H186" t="str">
         <v/>
       </c>
       <c r="I186" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J186" t="str">
         <v>unavailable</v>
@@ -7359,25 +7359,25 @@
         <v>no-problem</v>
       </c>
       <c r="C187" t="str">
-        <v/>
+        <v>ما في مشكلة</v>
       </c>
       <c r="D187" t="str">
-        <v/>
+        <v>ma fi mushkila</v>
       </c>
       <c r="E187" t="str">
-        <v/>
+        <v>No problem</v>
       </c>
       <c r="F187" t="str">
         <v>assets/images/vocab/sudanese-arabic/no-problem.png</v>
       </c>
       <c r="G187" t="str">
-        <v>assets/audio/sudanese-arabic/no-problem.mp3</v>
+        <v/>
       </c>
       <c r="H187" t="str">
         <v/>
       </c>
       <c r="I187" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J187" t="str">
         <v>unavailable</v>
@@ -7391,25 +7391,25 @@
         <v>excuse-me</v>
       </c>
       <c r="C188" t="str">
-        <v/>
+        <v>عن إذنك</v>
       </c>
       <c r="D188" t="str">
-        <v/>
+        <v>an iznak</v>
       </c>
       <c r="E188" t="str">
-        <v/>
+        <v>Excuse me</v>
       </c>
       <c r="F188" t="str">
         <v>assets/images/vocab/sudanese-arabic/excuse-me.png</v>
       </c>
       <c r="G188" t="str">
-        <v>assets/audio/sudanese-arabic/excuse-me.mp3</v>
+        <v/>
       </c>
       <c r="H188" t="str">
         <v/>
       </c>
       <c r="I188" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J188" t="str">
         <v>unavailable</v>
@@ -7423,25 +7423,25 @@
         <v>sorry</v>
       </c>
       <c r="C189" t="str">
-        <v/>
+        <v>آسف</v>
       </c>
       <c r="D189" t="str">
-        <v/>
+        <v>asif</v>
       </c>
       <c r="E189" t="str">
-        <v/>
+        <v>Sorry</v>
       </c>
       <c r="F189" t="str">
         <v>assets/images/vocab/sudanese-arabic/sorry.png</v>
       </c>
       <c r="G189" t="str">
-        <v>assets/audio/sudanese-arabic/sorry.mp3</v>
+        <v/>
       </c>
       <c r="H189" t="str">
         <v/>
       </c>
       <c r="I189" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J189" t="str">
         <v>unavailable</v>
@@ -7455,25 +7455,25 @@
         <v>this-is-my-family</v>
       </c>
       <c r="C190" t="str">
-        <v/>
+        <v>دي أسرتي</v>
       </c>
       <c r="D190" t="str">
-        <v/>
+        <v>di usriti</v>
       </c>
       <c r="E190" t="str">
-        <v/>
+        <v>This is my family</v>
       </c>
       <c r="F190" t="str">
         <v>assets/images/vocab/sudanese-arabic/this-is-my-family.png</v>
       </c>
       <c r="G190" t="str">
-        <v>assets/audio/sudanese-arabic/this-is-my-family.mp3</v>
+        <v/>
       </c>
       <c r="H190" t="str">
         <v/>
       </c>
       <c r="I190" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J190" t="str">
         <v>unavailable</v>
@@ -7487,25 +7487,25 @@
         <v>this-is-my-husband</v>
       </c>
       <c r="C191" t="str">
-        <v/>
+        <v>دا زوجي</v>
       </c>
       <c r="D191" t="str">
-        <v/>
+        <v>da zawji</v>
       </c>
       <c r="E191" t="str">
-        <v/>
+        <v>This is my husband</v>
       </c>
       <c r="F191" t="str">
         <v>assets/images/vocab/sudanese-arabic/this-is-my-husband.png</v>
       </c>
       <c r="G191" t="str">
-        <v>assets/audio/sudanese-arabic/this-is-my-husband.mp3</v>
+        <v/>
       </c>
       <c r="H191" t="str">
         <v/>
       </c>
       <c r="I191" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J191" t="str">
         <v>unavailable</v>
@@ -7519,25 +7519,25 @@
         <v>this-is-my-wife</v>
       </c>
       <c r="C192" t="str">
-        <v/>
+        <v>دي زوجتي</v>
       </c>
       <c r="D192" t="str">
-        <v/>
+        <v>di zawjati</v>
       </c>
       <c r="E192" t="str">
-        <v/>
+        <v>This is my wife</v>
       </c>
       <c r="F192" t="str">
         <v>assets/images/vocab/sudanese-arabic/this-is-my-wife.png</v>
       </c>
       <c r="G192" t="str">
-        <v>assets/audio/sudanese-arabic/this-is-my-wife.mp3</v>
+        <v/>
       </c>
       <c r="H192" t="str">
         <v/>
       </c>
       <c r="I192" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J192" t="str">
         <v>unavailable</v>
@@ -7551,25 +7551,25 @@
         <v>he-lives-here</v>
       </c>
       <c r="C193" t="str">
-        <v/>
+        <v>هو ساكن هنا</v>
       </c>
       <c r="D193" t="str">
-        <v/>
+        <v>huwa sakin hina</v>
       </c>
       <c r="E193" t="str">
-        <v/>
+        <v>He lives here</v>
       </c>
       <c r="F193" t="str">
         <v>assets/images/vocab/sudanese-arabic/he-lives-here.png</v>
       </c>
       <c r="G193" t="str">
-        <v>assets/audio/sudanese-arabic/he-lives-here.mp3</v>
+        <v/>
       </c>
       <c r="H193" t="str">
         <v/>
       </c>
       <c r="I193" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J193" t="str">
         <v>unavailable</v>
@@ -7583,25 +7583,25 @@
         <v>she-works-here</v>
       </c>
       <c r="C194" t="str">
-        <v/>
+        <v>هي شغالة هنا</v>
       </c>
       <c r="D194" t="str">
-        <v/>
+        <v>hiya shaghala hina</v>
       </c>
       <c r="E194" t="str">
-        <v/>
+        <v>She works here</v>
       </c>
       <c r="F194" t="str">
         <v>assets/images/vocab/sudanese-arabic/she-works-here.png</v>
       </c>
       <c r="G194" t="str">
-        <v>assets/audio/sudanese-arabic/she-works-here.mp3</v>
+        <v/>
       </c>
       <c r="H194" t="str">
         <v/>
       </c>
       <c r="I194" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J194" t="str">
         <v>unavailable</v>
@@ -7615,25 +7615,25 @@
         <v>we-speak</v>
       </c>
       <c r="C195" t="str">
-        <v/>
+        <v>نحن بنتكلم...</v>
       </c>
       <c r="D195" t="str">
-        <v/>
+        <v>nahna binitkallam...</v>
       </c>
       <c r="E195" t="str">
-        <v/>
+        <v>We speak...</v>
       </c>
       <c r="F195" t="str">
         <v>assets/images/vocab/sudanese-arabic/we-speak.png</v>
       </c>
       <c r="G195" t="str">
-        <v>assets/audio/sudanese-arabic/we-speak.mp3</v>
+        <v/>
       </c>
       <c r="H195" t="str">
         <v/>
       </c>
       <c r="I195" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J195" t="str">
         <v>unavailable</v>
@@ -7647,25 +7647,25 @@
         <v>they-are-from</v>
       </c>
       <c r="C196" t="str">
-        <v/>
+        <v>هم من...</v>
       </c>
       <c r="D196" t="str">
-        <v/>
+        <v>hum min...</v>
       </c>
       <c r="E196" t="str">
-        <v/>
+        <v>They are from...</v>
       </c>
       <c r="F196" t="str">
         <v>assets/images/vocab/sudanese-arabic/they-are-from.png</v>
       </c>
       <c r="G196" t="str">
-        <v>assets/audio/sudanese-arabic/they-are-from.mp3</v>
+        <v/>
       </c>
       <c r="H196" t="str">
         <v/>
       </c>
       <c r="I196" t="str">
-        <v>backlog</v>
+        <v>needs-native-review</v>
       </c>
       <c r="J196" t="str">
         <v>unavailable</v>
@@ -14811,7 +14811,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M257"/>
+  <dimension ref="A1:M321"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25350,9 +25350,2633 @@
         <v>unavailable</v>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B258" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C258" t="str">
+        <v>sudanese-arabic-getting-started-01-yes</v>
+      </c>
+      <c r="D258">
+        <v>1</v>
+      </c>
+      <c r="E258" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F258" t="str">
+        <v>What does "أيوه" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G258" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H258" t="str">
+        <v>["no","maybe","okay"]</v>
+      </c>
+      <c r="I258" t="str">
+        <v>yes</v>
+      </c>
+      <c r="J258" t="str">
+        <v>["yes"]</v>
+      </c>
+      <c r="K258" t="str">
+        <v/>
+      </c>
+      <c r="L258" t="b">
+        <v>1</v>
+      </c>
+      <c r="M258" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B259" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C259" t="str">
+        <v>sudanese-arabic-getting-started-02-no</v>
+      </c>
+      <c r="D259">
+        <v>2</v>
+      </c>
+      <c r="E259" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F259" t="str">
+        <v>Build the Sudanese Arabic phrase for "no".</v>
+      </c>
+      <c r="G259" t="str">
+        <v>لا</v>
+      </c>
+      <c r="H259" t="str">
+        <v>["أيوه","يمكن","تمام"]</v>
+      </c>
+      <c r="I259" t="str">
+        <v>no</v>
+      </c>
+      <c r="J259" t="str">
+        <v>["no"]</v>
+      </c>
+      <c r="K259" t="str">
+        <v/>
+      </c>
+      <c r="L259" t="b">
+        <v>1</v>
+      </c>
+      <c r="M259" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B260" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C260" t="str">
+        <v>sudanese-arabic-getting-started-03-match</v>
+      </c>
+      <c r="D260">
+        <v>3</v>
+      </c>
+      <c r="E260" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F260" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G260" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H260" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I260" t="str">
+        <v/>
+      </c>
+      <c r="J260" t="str">
+        <v>["yes","no","maybe","okay"]</v>
+      </c>
+      <c r="K260" t="str">
+        <v/>
+      </c>
+      <c r="L260" t="b">
+        <v>0</v>
+      </c>
+      <c r="M260" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B261" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C261" t="str">
+        <v>sudanese-arabic-getting-started-04-okay</v>
+      </c>
+      <c r="D261">
+        <v>4</v>
+      </c>
+      <c r="E261" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F261" t="str">
+        <v>Build the English meaning of "تمام".</v>
+      </c>
+      <c r="G261" t="str">
+        <v>okay</v>
+      </c>
+      <c r="H261" t="str">
+        <v>["yes","no","maybe"]</v>
+      </c>
+      <c r="I261" t="str">
+        <v>okay</v>
+      </c>
+      <c r="J261" t="str">
+        <v>["okay"]</v>
+      </c>
+      <c r="K261" t="str">
+        <v/>
+      </c>
+      <c r="L261" t="b">
+        <v>1</v>
+      </c>
+      <c r="M261" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B262" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C262" t="str">
+        <v>sudanese-arabic-getting-started-05-again</v>
+      </c>
+      <c r="D262">
+        <v>5</v>
+      </c>
+      <c r="E262" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F262" t="str">
+        <v>Choose the Sudanese Arabic for "again".</v>
+      </c>
+      <c r="G262" t="str">
+        <v>تاني</v>
+      </c>
+      <c r="H262" t="str">
+        <v>["أيوه","لا","يمكن"]</v>
+      </c>
+      <c r="I262" t="str">
+        <v>again</v>
+      </c>
+      <c r="J262" t="str">
+        <v>["again"]</v>
+      </c>
+      <c r="K262" t="str">
+        <v/>
+      </c>
+      <c r="L262" t="b">
+        <v>1</v>
+      </c>
+      <c r="M262" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B263" t="str">
+        <v>getting-started</v>
+      </c>
+      <c r="C263" t="str">
+        <v>sudanese-arabic-getting-started-06-again</v>
+      </c>
+      <c r="D263">
+        <v>6</v>
+      </c>
+      <c r="E263" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F263" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G263" t="str">
+        <v>again</v>
+      </c>
+      <c r="H263" t="str">
+        <v>["yes","no","maybe"]</v>
+      </c>
+      <c r="I263" t="str">
+        <v>again</v>
+      </c>
+      <c r="J263" t="str">
+        <v>["again"]</v>
+      </c>
+      <c r="K263" t="str">
+        <v/>
+      </c>
+      <c r="L263" t="b">
+        <v>1</v>
+      </c>
+      <c r="M263" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B264" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C264" t="str">
+        <v>sudanese-arabic-easy-greetings-01-good-afternoon</v>
+      </c>
+      <c r="D264">
+        <v>1</v>
+      </c>
+      <c r="E264" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F264" t="str">
+        <v>What does "مساء الخير" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G264" t="str">
+        <v>good afternoon</v>
+      </c>
+      <c r="H264" t="str">
+        <v>["nice to meet you","long time no see","how is your day"]</v>
+      </c>
+      <c r="I264" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J264" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K264" t="str">
+        <v/>
+      </c>
+      <c r="L264" t="b">
+        <v>1</v>
+      </c>
+      <c r="M264" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B265" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C265" t="str">
+        <v>sudanese-arabic-easy-greetings-02-nice-to-meet-you</v>
+      </c>
+      <c r="D265">
+        <v>2</v>
+      </c>
+      <c r="E265" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F265" t="str">
+        <v>Build the Sudanese Arabic phrase for "nice to meet you".</v>
+      </c>
+      <c r="G265" t="str">
+        <v>اتشرفت بيك</v>
+      </c>
+      <c r="H265" t="str">
+        <v>["مساء الخير","زمن ما شفناك","يومك كيف؟"]</v>
+      </c>
+      <c r="I265" t="str">
+        <v>nice-to-meet-you</v>
+      </c>
+      <c r="J265" t="str">
+        <v>["nice-to-meet-you"]</v>
+      </c>
+      <c r="K265" t="str">
+        <v/>
+      </c>
+      <c r="L265" t="b">
+        <v>1</v>
+      </c>
+      <c r="M265" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B266" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C266" t="str">
+        <v>sudanese-arabic-easy-greetings-03-match</v>
+      </c>
+      <c r="D266">
+        <v>3</v>
+      </c>
+      <c r="E266" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F266" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G266" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H266" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I266" t="str">
+        <v/>
+      </c>
+      <c r="J266" t="str">
+        <v>["good-afternoon","nice-to-meet-you","long-time-no-see","how-is-your-day"]</v>
+      </c>
+      <c r="K266" t="str">
+        <v/>
+      </c>
+      <c r="L266" t="b">
+        <v>0</v>
+      </c>
+      <c r="M266" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B267" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C267" t="str">
+        <v>sudanese-arabic-easy-greetings-04-how-is-your-day</v>
+      </c>
+      <c r="D267">
+        <v>4</v>
+      </c>
+      <c r="E267" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F267" t="str">
+        <v>Build the English meaning of "يومك كيف؟".</v>
+      </c>
+      <c r="G267" t="str">
+        <v>how is your day</v>
+      </c>
+      <c r="H267" t="str">
+        <v>["good afternoon","nice to meet you","long time no see"]</v>
+      </c>
+      <c r="I267" t="str">
+        <v>how-is-your-day</v>
+      </c>
+      <c r="J267" t="str">
+        <v>["how-is-your-day"]</v>
+      </c>
+      <c r="K267" t="str">
+        <v/>
+      </c>
+      <c r="L267" t="b">
+        <v>1</v>
+      </c>
+      <c r="M267" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B268" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C268" t="str">
+        <v>sudanese-arabic-easy-greetings-05-have-a-good-day</v>
+      </c>
+      <c r="D268">
+        <v>5</v>
+      </c>
+      <c r="E268" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F268" t="str">
+        <v>Choose the Sudanese Arabic for "have a good day".</v>
+      </c>
+      <c r="G268" t="str">
+        <v>يومك سعيد</v>
+      </c>
+      <c r="H268" t="str">
+        <v>["مساء الخير","اتشرفت بيك","زمن ما شفناك"]</v>
+      </c>
+      <c r="I268" t="str">
+        <v>have-a-good-day</v>
+      </c>
+      <c r="J268" t="str">
+        <v>["have-a-good-day"]</v>
+      </c>
+      <c r="K268" t="str">
+        <v/>
+      </c>
+      <c r="L268" t="b">
+        <v>1</v>
+      </c>
+      <c r="M268" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B269" t="str">
+        <v>easy-greetings</v>
+      </c>
+      <c r="C269" t="str">
+        <v>sudanese-arabic-easy-greetings-06-have-a-good-day</v>
+      </c>
+      <c r="D269">
+        <v>6</v>
+      </c>
+      <c r="E269" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F269" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G269" t="str">
+        <v>have a good day</v>
+      </c>
+      <c r="H269" t="str">
+        <v>["good afternoon","nice to meet you","long time no see"]</v>
+      </c>
+      <c r="I269" t="str">
+        <v>have-a-good-day</v>
+      </c>
+      <c r="J269" t="str">
+        <v>["have-a-good-day"]</v>
+      </c>
+      <c r="K269" t="str">
+        <v/>
+      </c>
+      <c r="L269" t="b">
+        <v>1</v>
+      </c>
+      <c r="M269" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B270" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C270" t="str">
+        <v>sudanese-arabic-introducing-yourself-01-what-is-your-name</v>
+      </c>
+      <c r="D270">
+        <v>1</v>
+      </c>
+      <c r="E270" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F270" t="str">
+        <v>What does "اسمك منو؟" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G270" t="str">
+        <v>what is your name</v>
+      </c>
+      <c r="H270" t="str">
+        <v>["my name is","i am a student","i am learning"]</v>
+      </c>
+      <c r="I270" t="str">
+        <v>what-is-your-name</v>
+      </c>
+      <c r="J270" t="str">
+        <v>["what-is-your-name"]</v>
+      </c>
+      <c r="K270" t="str">
+        <v/>
+      </c>
+      <c r="L270" t="b">
+        <v>1</v>
+      </c>
+      <c r="M270" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B271" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C271" t="str">
+        <v>sudanese-arabic-introducing-yourself-02-my-name-is</v>
+      </c>
+      <c r="D271">
+        <v>2</v>
+      </c>
+      <c r="E271" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F271" t="str">
+        <v>Build the Sudanese Arabic phrase for "my name is".</v>
+      </c>
+      <c r="G271" t="str">
+        <v>اسمي...</v>
+      </c>
+      <c r="H271" t="str">
+        <v>["اسمك منو؟","أنا طالب","أنا بتعلم..."]</v>
+      </c>
+      <c r="I271" t="str">
+        <v>my-name-is</v>
+      </c>
+      <c r="J271" t="str">
+        <v>["my-name-is"]</v>
+      </c>
+      <c r="K271" t="str">
+        <v/>
+      </c>
+      <c r="L271" t="b">
+        <v>1</v>
+      </c>
+      <c r="M271" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B272" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C272" t="str">
+        <v>sudanese-arabic-introducing-yourself-03-match</v>
+      </c>
+      <c r="D272">
+        <v>3</v>
+      </c>
+      <c r="E272" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F272" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G272" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H272" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I272" t="str">
+        <v/>
+      </c>
+      <c r="J272" t="str">
+        <v>["what-is-your-name","my-name-is","i-am-a-student","i-am-learning"]</v>
+      </c>
+      <c r="K272" t="str">
+        <v/>
+      </c>
+      <c r="L272" t="b">
+        <v>0</v>
+      </c>
+      <c r="M272" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B273" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C273" t="str">
+        <v>sudanese-arabic-introducing-yourself-04-i-am-learning</v>
+      </c>
+      <c r="D273">
+        <v>4</v>
+      </c>
+      <c r="E273" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F273" t="str">
+        <v>Build the English meaning of "أنا بتعلم...".</v>
+      </c>
+      <c r="G273" t="str">
+        <v>i am learning</v>
+      </c>
+      <c r="H273" t="str">
+        <v>["what is your name","my name is","i am a student"]</v>
+      </c>
+      <c r="I273" t="str">
+        <v>i-am-learning</v>
+      </c>
+      <c r="J273" t="str">
+        <v>["i-am-learning"]</v>
+      </c>
+      <c r="K273" t="str">
+        <v/>
+      </c>
+      <c r="L273" t="b">
+        <v>1</v>
+      </c>
+      <c r="M273" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B274" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C274" t="str">
+        <v>sudanese-arabic-introducing-yourself-05-i-speak</v>
+      </c>
+      <c r="D274">
+        <v>5</v>
+      </c>
+      <c r="E274" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F274" t="str">
+        <v>Choose the Sudanese Arabic for "i speak".</v>
+      </c>
+      <c r="G274" t="str">
+        <v>أنا بتكلم...</v>
+      </c>
+      <c r="H274" t="str">
+        <v>["اسمك منو؟","اسمي...","أنا طالب"]</v>
+      </c>
+      <c r="I274" t="str">
+        <v>i-speak</v>
+      </c>
+      <c r="J274" t="str">
+        <v>["i-speak"]</v>
+      </c>
+      <c r="K274" t="str">
+        <v/>
+      </c>
+      <c r="L274" t="b">
+        <v>1</v>
+      </c>
+      <c r="M274" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B275" t="str">
+        <v>introducing-yourself</v>
+      </c>
+      <c r="C275" t="str">
+        <v>sudanese-arabic-introducing-yourself-06-i-speak</v>
+      </c>
+      <c r="D275">
+        <v>6</v>
+      </c>
+      <c r="E275" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F275" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G275" t="str">
+        <v>i speak</v>
+      </c>
+      <c r="H275" t="str">
+        <v>["what is your name","my name is","i am a student"]</v>
+      </c>
+      <c r="I275" t="str">
+        <v>i-speak</v>
+      </c>
+      <c r="J275" t="str">
+        <v>["i-speak"]</v>
+      </c>
+      <c r="K275" t="str">
+        <v/>
+      </c>
+      <c r="L275" t="b">
+        <v>1</v>
+      </c>
+      <c r="M275" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B276" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C276" t="str">
+        <v>sudanese-arabic-your-background-01-where-are-you-from</v>
+      </c>
+      <c r="D276">
+        <v>1</v>
+      </c>
+      <c r="E276" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F276" t="str">
+        <v>What does "إنت من وين؟" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G276" t="str">
+        <v>where are you from</v>
+      </c>
+      <c r="H276" t="str">
+        <v>["i am from","where do you live","i live in"]</v>
+      </c>
+      <c r="I276" t="str">
+        <v>where-are-you-from</v>
+      </c>
+      <c r="J276" t="str">
+        <v>["where-are-you-from"]</v>
+      </c>
+      <c r="K276" t="str">
+        <v/>
+      </c>
+      <c r="L276" t="b">
+        <v>1</v>
+      </c>
+      <c r="M276" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B277" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C277" t="str">
+        <v>sudanese-arabic-your-background-02-i-am-from</v>
+      </c>
+      <c r="D277">
+        <v>2</v>
+      </c>
+      <c r="E277" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F277" t="str">
+        <v>Build the Sudanese Arabic phrase for "i am from".</v>
+      </c>
+      <c r="G277" t="str">
+        <v>أنا من...</v>
+      </c>
+      <c r="H277" t="str">
+        <v>["إنت من وين؟","ساكن وين؟","ساكن في..."]</v>
+      </c>
+      <c r="I277" t="str">
+        <v>i-am-from</v>
+      </c>
+      <c r="J277" t="str">
+        <v>["i-am-from"]</v>
+      </c>
+      <c r="K277" t="str">
+        <v/>
+      </c>
+      <c r="L277" t="b">
+        <v>1</v>
+      </c>
+      <c r="M277" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B278" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C278" t="str">
+        <v>sudanese-arabic-your-background-03-match</v>
+      </c>
+      <c r="D278">
+        <v>3</v>
+      </c>
+      <c r="E278" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F278" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G278" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H278" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I278" t="str">
+        <v/>
+      </c>
+      <c r="J278" t="str">
+        <v>["where-are-you-from","i-am-from","where-do-you-live","i-live-in"]</v>
+      </c>
+      <c r="K278" t="str">
+        <v/>
+      </c>
+      <c r="L278" t="b">
+        <v>0</v>
+      </c>
+      <c r="M278" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B279" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C279" t="str">
+        <v>sudanese-arabic-your-background-04-i-live-in</v>
+      </c>
+      <c r="D279">
+        <v>4</v>
+      </c>
+      <c r="E279" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F279" t="str">
+        <v>Build the English meaning of "ساكن في...".</v>
+      </c>
+      <c r="G279" t="str">
+        <v>i live in</v>
+      </c>
+      <c r="H279" t="str">
+        <v>["where are you from","i am from","where do you live"]</v>
+      </c>
+      <c r="I279" t="str">
+        <v>i-live-in</v>
+      </c>
+      <c r="J279" t="str">
+        <v>["i-live-in"]</v>
+      </c>
+      <c r="K279" t="str">
+        <v/>
+      </c>
+      <c r="L279" t="b">
+        <v>1</v>
+      </c>
+      <c r="M279" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B280" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C280" t="str">
+        <v>sudanese-arabic-your-background-05-which-language-do-you-speak</v>
+      </c>
+      <c r="D280">
+        <v>5</v>
+      </c>
+      <c r="E280" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F280" t="str">
+        <v>Choose the Sudanese Arabic for "which language do you speak".</v>
+      </c>
+      <c r="G280" t="str">
+        <v>بتتكلم ياتو لغة؟</v>
+      </c>
+      <c r="H280" t="str">
+        <v>["إنت من وين؟","أنا من...","ساكن وين؟"]</v>
+      </c>
+      <c r="I280" t="str">
+        <v>which-language-do-you-speak</v>
+      </c>
+      <c r="J280" t="str">
+        <v>["which-language-do-you-speak"]</v>
+      </c>
+      <c r="K280" t="str">
+        <v/>
+      </c>
+      <c r="L280" t="b">
+        <v>1</v>
+      </c>
+      <c r="M280" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B281" t="str">
+        <v>your-background</v>
+      </c>
+      <c r="C281" t="str">
+        <v>sudanese-arabic-your-background-06-which-language-do-you-speak</v>
+      </c>
+      <c r="D281">
+        <v>6</v>
+      </c>
+      <c r="E281" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F281" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G281" t="str">
+        <v>which language do you speak</v>
+      </c>
+      <c r="H281" t="str">
+        <v>["where are you from","i am from","where do you live"]</v>
+      </c>
+      <c r="I281" t="str">
+        <v>which-language-do-you-speak</v>
+      </c>
+      <c r="J281" t="str">
+        <v>["which-language-do-you-speak"]</v>
+      </c>
+      <c r="K281" t="str">
+        <v/>
+      </c>
+      <c r="L281" t="b">
+        <v>1</v>
+      </c>
+      <c r="M281" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B282" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C282" t="str">
+        <v>sudanese-arabic-family-members-01-family</v>
+      </c>
+      <c r="D282">
+        <v>1</v>
+      </c>
+      <c r="E282" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F282" t="str">
+        <v>What does "أسرة" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G282" t="str">
+        <v>family</v>
+      </c>
+      <c r="H282" t="str">
+        <v>["parents","husband","wife"]</v>
+      </c>
+      <c r="I282" t="str">
+        <v>family</v>
+      </c>
+      <c r="J282" t="str">
+        <v>["family"]</v>
+      </c>
+      <c r="K282" t="str">
+        <v/>
+      </c>
+      <c r="L282" t="b">
+        <v>1</v>
+      </c>
+      <c r="M282" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B283" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C283" t="str">
+        <v>sudanese-arabic-family-members-02-parents</v>
+      </c>
+      <c r="D283">
+        <v>2</v>
+      </c>
+      <c r="E283" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F283" t="str">
+        <v>Build the Sudanese Arabic phrase for "parents".</v>
+      </c>
+      <c r="G283" t="str">
+        <v>الأهل</v>
+      </c>
+      <c r="H283" t="str">
+        <v>["أسرة","زوج","زوجة"]</v>
+      </c>
+      <c r="I283" t="str">
+        <v>parents</v>
+      </c>
+      <c r="J283" t="str">
+        <v>["parents"]</v>
+      </c>
+      <c r="K283" t="str">
+        <v/>
+      </c>
+      <c r="L283" t="b">
+        <v>1</v>
+      </c>
+      <c r="M283" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B284" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C284" t="str">
+        <v>sudanese-arabic-family-members-03-match</v>
+      </c>
+      <c r="D284">
+        <v>3</v>
+      </c>
+      <c r="E284" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F284" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G284" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H284" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I284" t="str">
+        <v/>
+      </c>
+      <c r="J284" t="str">
+        <v>["family","parents","husband","wife"]</v>
+      </c>
+      <c r="K284" t="str">
+        <v/>
+      </c>
+      <c r="L284" t="b">
+        <v>0</v>
+      </c>
+      <c r="M284" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B285" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C285" t="str">
+        <v>sudanese-arabic-family-members-04-wife</v>
+      </c>
+      <c r="D285">
+        <v>4</v>
+      </c>
+      <c r="E285" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F285" t="str">
+        <v>Build the English meaning of "زوجة".</v>
+      </c>
+      <c r="G285" t="str">
+        <v>wife</v>
+      </c>
+      <c r="H285" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I285" t="str">
+        <v>wife</v>
+      </c>
+      <c r="J285" t="str">
+        <v>["wife"]</v>
+      </c>
+      <c r="K285" t="str">
+        <v/>
+      </c>
+      <c r="L285" t="b">
+        <v>1</v>
+      </c>
+      <c r="M285" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B286" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C286" t="str">
+        <v>sudanese-arabic-family-members-05-son</v>
+      </c>
+      <c r="D286">
+        <v>5</v>
+      </c>
+      <c r="E286" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F286" t="str">
+        <v>Choose the Sudanese Arabic for "son".</v>
+      </c>
+      <c r="G286" t="str">
+        <v>ولد</v>
+      </c>
+      <c r="H286" t="str">
+        <v>["أسرة","الأهل","زوج"]</v>
+      </c>
+      <c r="I286" t="str">
+        <v>son</v>
+      </c>
+      <c r="J286" t="str">
+        <v>["son"]</v>
+      </c>
+      <c r="K286" t="str">
+        <v/>
+      </c>
+      <c r="L286" t="b">
+        <v>1</v>
+      </c>
+      <c r="M286" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B287" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C287" t="str">
+        <v>sudanese-arabic-family-members-06-daughter</v>
+      </c>
+      <c r="D287">
+        <v>6</v>
+      </c>
+      <c r="E287" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F287" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G287" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="H287" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I287" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J287" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K287" t="str">
+        <v/>
+      </c>
+      <c r="L287" t="b">
+        <v>1</v>
+      </c>
+      <c r="M287" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B288" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C288" t="str">
+        <v>sudanese-arabic-family-members-07-grandfather</v>
+      </c>
+      <c r="D288">
+        <v>7</v>
+      </c>
+      <c r="E288" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F288" t="str">
+        <v>Choose the Sudanese Arabic for "grandfather".</v>
+      </c>
+      <c r="G288" t="str">
+        <v>جد</v>
+      </c>
+      <c r="H288" t="str">
+        <v>["أسرة","الأهل","زوج"]</v>
+      </c>
+      <c r="I288" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="J288" t="str">
+        <v>["grandfather"]</v>
+      </c>
+      <c r="K288" t="str">
+        <v/>
+      </c>
+      <c r="L288" t="b">
+        <v>1</v>
+      </c>
+      <c r="M288" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B289" t="str">
+        <v>family-members</v>
+      </c>
+      <c r="C289" t="str">
+        <v>sudanese-arabic-family-members-08-grandfather</v>
+      </c>
+      <c r="D289">
+        <v>8</v>
+      </c>
+      <c r="E289" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F289" t="str">
+        <v>What does "جد" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G289" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="H289" t="str">
+        <v>["family","parents","husband"]</v>
+      </c>
+      <c r="I289" t="str">
+        <v>grandfather</v>
+      </c>
+      <c r="J289" t="str">
+        <v>["grandfather"]</v>
+      </c>
+      <c r="K289" t="str">
+        <v/>
+      </c>
+      <c r="L289" t="b">
+        <v>1</v>
+      </c>
+      <c r="M289" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B290" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C290" t="str">
+        <v>sudanese-arabic-polite-conversation-01-please</v>
+      </c>
+      <c r="D290">
+        <v>1</v>
+      </c>
+      <c r="E290" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F290" t="str">
+        <v>What does "لو سمحت" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G290" t="str">
+        <v>please</v>
+      </c>
+      <c r="H290" t="str">
+        <v>["thank you","no problem","excuse me"]</v>
+      </c>
+      <c r="I290" t="str">
+        <v>please</v>
+      </c>
+      <c r="J290" t="str">
+        <v>["please"]</v>
+      </c>
+      <c r="K290" t="str">
+        <v/>
+      </c>
+      <c r="L290" t="b">
+        <v>1</v>
+      </c>
+      <c r="M290" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B291" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C291" t="str">
+        <v>sudanese-arabic-polite-conversation-02-thank-you</v>
+      </c>
+      <c r="D291">
+        <v>2</v>
+      </c>
+      <c r="E291" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F291" t="str">
+        <v>Build the Sudanese Arabic phrase for "thank you".</v>
+      </c>
+      <c r="G291" t="str">
+        <v>شكراً</v>
+      </c>
+      <c r="H291" t="str">
+        <v>["لو سمحت","ما في مشكلة","عن إذنك"]</v>
+      </c>
+      <c r="I291" t="str">
+        <v>thank-you</v>
+      </c>
+      <c r="J291" t="str">
+        <v>["thank-you"]</v>
+      </c>
+      <c r="K291" t="str">
+        <v/>
+      </c>
+      <c r="L291" t="b">
+        <v>1</v>
+      </c>
+      <c r="M291" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B292" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C292" t="str">
+        <v>sudanese-arabic-polite-conversation-03-match</v>
+      </c>
+      <c r="D292">
+        <v>3</v>
+      </c>
+      <c r="E292" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F292" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G292" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H292" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I292" t="str">
+        <v/>
+      </c>
+      <c r="J292" t="str">
+        <v>["please","thank-you","no-problem","excuse-me"]</v>
+      </c>
+      <c r="K292" t="str">
+        <v/>
+      </c>
+      <c r="L292" t="b">
+        <v>0</v>
+      </c>
+      <c r="M292" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B293" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C293" t="str">
+        <v>sudanese-arabic-polite-conversation-04-excuse-me</v>
+      </c>
+      <c r="D293">
+        <v>4</v>
+      </c>
+      <c r="E293" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F293" t="str">
+        <v>Build the English meaning of "عن إذنك".</v>
+      </c>
+      <c r="G293" t="str">
+        <v>excuse me</v>
+      </c>
+      <c r="H293" t="str">
+        <v>["please","thank you","no problem"]</v>
+      </c>
+      <c r="I293" t="str">
+        <v>excuse-me</v>
+      </c>
+      <c r="J293" t="str">
+        <v>["excuse-me"]</v>
+      </c>
+      <c r="K293" t="str">
+        <v/>
+      </c>
+      <c r="L293" t="b">
+        <v>1</v>
+      </c>
+      <c r="M293" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B294" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C294" t="str">
+        <v>sudanese-arabic-polite-conversation-05-sorry</v>
+      </c>
+      <c r="D294">
+        <v>5</v>
+      </c>
+      <c r="E294" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F294" t="str">
+        <v>Choose the Sudanese Arabic for "sorry".</v>
+      </c>
+      <c r="G294" t="str">
+        <v>آسف</v>
+      </c>
+      <c r="H294" t="str">
+        <v>["لو سمحت","شكراً","ما في مشكلة"]</v>
+      </c>
+      <c r="I294" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="J294" t="str">
+        <v>["sorry"]</v>
+      </c>
+      <c r="K294" t="str">
+        <v/>
+      </c>
+      <c r="L294" t="b">
+        <v>1</v>
+      </c>
+      <c r="M294" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B295" t="str">
+        <v>polite-conversation</v>
+      </c>
+      <c r="C295" t="str">
+        <v>sudanese-arabic-polite-conversation-06-sorry</v>
+      </c>
+      <c r="D295">
+        <v>6</v>
+      </c>
+      <c r="E295" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F295" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G295" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="H295" t="str">
+        <v>["please","thank you","no problem"]</v>
+      </c>
+      <c r="I295" t="str">
+        <v>sorry</v>
+      </c>
+      <c r="J295" t="str">
+        <v>["sorry"]</v>
+      </c>
+      <c r="K295" t="str">
+        <v/>
+      </c>
+      <c r="L295" t="b">
+        <v>1</v>
+      </c>
+      <c r="M295" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B296" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C296" t="str">
+        <v>sudanese-arabic-introducing-others-01-this-is-my-family</v>
+      </c>
+      <c r="D296">
+        <v>1</v>
+      </c>
+      <c r="E296" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F296" t="str">
+        <v>What does "دي أسرتي" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G296" t="str">
+        <v>this is my family</v>
+      </c>
+      <c r="H296" t="str">
+        <v>["this is my husband","this is my wife","he lives here"]</v>
+      </c>
+      <c r="I296" t="str">
+        <v>this-is-my-family</v>
+      </c>
+      <c r="J296" t="str">
+        <v>["this-is-my-family"]</v>
+      </c>
+      <c r="K296" t="str">
+        <v/>
+      </c>
+      <c r="L296" t="b">
+        <v>1</v>
+      </c>
+      <c r="M296" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B297" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C297" t="str">
+        <v>sudanese-arabic-introducing-others-02-this-is-my-husband</v>
+      </c>
+      <c r="D297">
+        <v>2</v>
+      </c>
+      <c r="E297" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F297" t="str">
+        <v>Build the Sudanese Arabic phrase for "this is my husband".</v>
+      </c>
+      <c r="G297" t="str">
+        <v>دا زوجي</v>
+      </c>
+      <c r="H297" t="str">
+        <v>["دي أسرتي","دي زوجتي","هو ساكن هنا"]</v>
+      </c>
+      <c r="I297" t="str">
+        <v>this-is-my-husband</v>
+      </c>
+      <c r="J297" t="str">
+        <v>["this-is-my-husband"]</v>
+      </c>
+      <c r="K297" t="str">
+        <v/>
+      </c>
+      <c r="L297" t="b">
+        <v>1</v>
+      </c>
+      <c r="M297" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B298" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C298" t="str">
+        <v>sudanese-arabic-introducing-others-03-match</v>
+      </c>
+      <c r="D298">
+        <v>3</v>
+      </c>
+      <c r="E298" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F298" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G298" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H298" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I298" t="str">
+        <v/>
+      </c>
+      <c r="J298" t="str">
+        <v>["this-is-my-family","this-is-my-husband","this-is-my-wife","he-lives-here"]</v>
+      </c>
+      <c r="K298" t="str">
+        <v/>
+      </c>
+      <c r="L298" t="b">
+        <v>0</v>
+      </c>
+      <c r="M298" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B299" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C299" t="str">
+        <v>sudanese-arabic-introducing-others-04-he-lives-here</v>
+      </c>
+      <c r="D299">
+        <v>4</v>
+      </c>
+      <c r="E299" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F299" t="str">
+        <v>Build the English meaning of "هو ساكن هنا".</v>
+      </c>
+      <c r="G299" t="str">
+        <v>he lives here</v>
+      </c>
+      <c r="H299" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I299" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J299" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K299" t="str">
+        <v/>
+      </c>
+      <c r="L299" t="b">
+        <v>1</v>
+      </c>
+      <c r="M299" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B300" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C300" t="str">
+        <v>sudanese-arabic-introducing-others-05-she-works-here</v>
+      </c>
+      <c r="D300">
+        <v>5</v>
+      </c>
+      <c r="E300" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F300" t="str">
+        <v>Choose the Sudanese Arabic for "she works here".</v>
+      </c>
+      <c r="G300" t="str">
+        <v>هي شغالة هنا</v>
+      </c>
+      <c r="H300" t="str">
+        <v>["دي أسرتي","دا زوجي","دي زوجتي"]</v>
+      </c>
+      <c r="I300" t="str">
+        <v>she-works-here</v>
+      </c>
+      <c r="J300" t="str">
+        <v>["she-works-here"]</v>
+      </c>
+      <c r="K300" t="str">
+        <v/>
+      </c>
+      <c r="L300" t="b">
+        <v>1</v>
+      </c>
+      <c r="M300" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B301" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C301" t="str">
+        <v>sudanese-arabic-introducing-others-06-we-speak</v>
+      </c>
+      <c r="D301">
+        <v>6</v>
+      </c>
+      <c r="E301" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F301" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G301" t="str">
+        <v>we speak</v>
+      </c>
+      <c r="H301" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I301" t="str">
+        <v>we-speak</v>
+      </c>
+      <c r="J301" t="str">
+        <v>["we-speak"]</v>
+      </c>
+      <c r="K301" t="str">
+        <v/>
+      </c>
+      <c r="L301" t="b">
+        <v>1</v>
+      </c>
+      <c r="M301" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B302" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C302" t="str">
+        <v>sudanese-arabic-introducing-others-07-they-are-from</v>
+      </c>
+      <c r="D302">
+        <v>7</v>
+      </c>
+      <c r="E302" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F302" t="str">
+        <v>Choose the Sudanese Arabic for "they are from".</v>
+      </c>
+      <c r="G302" t="str">
+        <v>هم من...</v>
+      </c>
+      <c r="H302" t="str">
+        <v>["دي أسرتي","دا زوجي","دي زوجتي"]</v>
+      </c>
+      <c r="I302" t="str">
+        <v>they-are-from</v>
+      </c>
+      <c r="J302" t="str">
+        <v>["they-are-from"]</v>
+      </c>
+      <c r="K302" t="str">
+        <v/>
+      </c>
+      <c r="L302" t="b">
+        <v>1</v>
+      </c>
+      <c r="M302" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B303" t="str">
+        <v>introducing-others</v>
+      </c>
+      <c r="C303" t="str">
+        <v>sudanese-arabic-introducing-others-08-they-are-from</v>
+      </c>
+      <c r="D303">
+        <v>8</v>
+      </c>
+      <c r="E303" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F303" t="str">
+        <v>What does "هم من..." mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G303" t="str">
+        <v>they are from</v>
+      </c>
+      <c r="H303" t="str">
+        <v>["this is my family","this is my husband","this is my wife"]</v>
+      </c>
+      <c r="I303" t="str">
+        <v>they-are-from</v>
+      </c>
+      <c r="J303" t="str">
+        <v>["they-are-from"]</v>
+      </c>
+      <c r="K303" t="str">
+        <v/>
+      </c>
+      <c r="L303" t="b">
+        <v>1</v>
+      </c>
+      <c r="M303" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B304" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C304" t="str">
+        <v>sudanese-arabic-words-practice-01-yes</v>
+      </c>
+      <c r="D304">
+        <v>1</v>
+      </c>
+      <c r="E304" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F304" t="str">
+        <v>What does "أيوه" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G304" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H304" t="str">
+        <v>["good afternoon","what is your name","where are you from"]</v>
+      </c>
+      <c r="I304" t="str">
+        <v>yes</v>
+      </c>
+      <c r="J304" t="str">
+        <v>["yes"]</v>
+      </c>
+      <c r="K304" t="str">
+        <v/>
+      </c>
+      <c r="L304" t="b">
+        <v>0</v>
+      </c>
+      <c r="M304" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B305" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C305" t="str">
+        <v>sudanese-arabic-words-practice-02-good-afternoon</v>
+      </c>
+      <c r="D305">
+        <v>2</v>
+      </c>
+      <c r="E305" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F305" t="str">
+        <v>Build the Sudanese Arabic phrase for "good afternoon".</v>
+      </c>
+      <c r="G305" t="str">
+        <v>مساء الخير</v>
+      </c>
+      <c r="H305" t="str">
+        <v>["أيوه","اسمك منو؟","إنت من وين؟"]</v>
+      </c>
+      <c r="I305" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J305" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K305" t="str">
+        <v/>
+      </c>
+      <c r="L305" t="b">
+        <v>0</v>
+      </c>
+      <c r="M305" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B306" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C306" t="str">
+        <v>sudanese-arabic-words-practice-03-match</v>
+      </c>
+      <c r="D306">
+        <v>3</v>
+      </c>
+      <c r="E306" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G306" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H306" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I306" t="str">
+        <v/>
+      </c>
+      <c r="J306" t="str">
+        <v>["yes","good-afternoon","what-is-your-name","where-are-you-from"]</v>
+      </c>
+      <c r="K306" t="str">
+        <v/>
+      </c>
+      <c r="L306" t="b">
+        <v>0</v>
+      </c>
+      <c r="M306" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B307" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C307" t="str">
+        <v>sudanese-arabic-words-practice-04-where-are-you-from</v>
+      </c>
+      <c r="D307">
+        <v>4</v>
+      </c>
+      <c r="E307" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Build the English meaning of "إنت من وين؟".</v>
+      </c>
+      <c r="G307" t="str">
+        <v>where are you from</v>
+      </c>
+      <c r="H307" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I307" t="str">
+        <v>where-are-you-from</v>
+      </c>
+      <c r="J307" t="str">
+        <v>["where-are-you-from"]</v>
+      </c>
+      <c r="K307" t="str">
+        <v/>
+      </c>
+      <c r="L307" t="b">
+        <v>0</v>
+      </c>
+      <c r="M307" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B308" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C308" t="str">
+        <v>sudanese-arabic-words-practice-05-family</v>
+      </c>
+      <c r="D308">
+        <v>5</v>
+      </c>
+      <c r="E308" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Choose the Sudanese Arabic for "family".</v>
+      </c>
+      <c r="G308" t="str">
+        <v>أسرة</v>
+      </c>
+      <c r="H308" t="str">
+        <v>["أيوه","مساء الخير","اسمك منو؟"]</v>
+      </c>
+      <c r="I308" t="str">
+        <v>family</v>
+      </c>
+      <c r="J308" t="str">
+        <v>["family"]</v>
+      </c>
+      <c r="K308" t="str">
+        <v/>
+      </c>
+      <c r="L308" t="b">
+        <v>0</v>
+      </c>
+      <c r="M308" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B309" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C309" t="str">
+        <v>sudanese-arabic-words-practice-06-daughter</v>
+      </c>
+      <c r="D309">
+        <v>6</v>
+      </c>
+      <c r="E309" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G309" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="H309" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I309" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J309" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K309" t="str">
+        <v/>
+      </c>
+      <c r="L309" t="b">
+        <v>0</v>
+      </c>
+      <c r="M309" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B310" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C310" t="str">
+        <v>sudanese-arabic-words-practice-07-excuse-me</v>
+      </c>
+      <c r="D310">
+        <v>7</v>
+      </c>
+      <c r="E310" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Choose the Sudanese Arabic for "excuse me".</v>
+      </c>
+      <c r="G310" t="str">
+        <v>عن إذنك</v>
+      </c>
+      <c r="H310" t="str">
+        <v>["أيوه","مساء الخير","اسمك منو؟"]</v>
+      </c>
+      <c r="I310" t="str">
+        <v>excuse-me</v>
+      </c>
+      <c r="J310" t="str">
+        <v>["excuse-me"]</v>
+      </c>
+      <c r="K310" t="str">
+        <v/>
+      </c>
+      <c r="L310" t="b">
+        <v>0</v>
+      </c>
+      <c r="M310" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B311" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C311" t="str">
+        <v>sudanese-arabic-words-practice-08-he-lives-here</v>
+      </c>
+      <c r="D311">
+        <v>8</v>
+      </c>
+      <c r="E311" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F311" t="str">
+        <v>What does "هو ساكن هنا" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G311" t="str">
+        <v>he lives here</v>
+      </c>
+      <c r="H311" t="str">
+        <v>["yes","good afternoon","what is your name"]</v>
+      </c>
+      <c r="I311" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J311" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K311" t="str">
+        <v/>
+      </c>
+      <c r="L311" t="b">
+        <v>0</v>
+      </c>
+      <c r="M311" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B312" t="str">
+        <v>words-practice</v>
+      </c>
+      <c r="C312" t="str">
+        <v>sudanese-arabic-words-practice-09-he-lives-here</v>
+      </c>
+      <c r="D312">
+        <v>9</v>
+      </c>
+      <c r="E312" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Choose the Sudanese Arabic for "he lives here".</v>
+      </c>
+      <c r="G312" t="str">
+        <v>هو ساكن هنا</v>
+      </c>
+      <c r="H312" t="str">
+        <v>["أيوه","مساء الخير","اسمك منو؟"]</v>
+      </c>
+      <c r="I312" t="str">
+        <v>he-lives-here</v>
+      </c>
+      <c r="J312" t="str">
+        <v>["he-lives-here"]</v>
+      </c>
+      <c r="K312" t="str">
+        <v/>
+      </c>
+      <c r="L312" t="b">
+        <v>0</v>
+      </c>
+      <c r="M312" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B313" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C313" t="str">
+        <v>sudanese-arabic-practice-challenge-01-no</v>
+      </c>
+      <c r="D313">
+        <v>1</v>
+      </c>
+      <c r="E313" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F313" t="str">
+        <v>What does "لا" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G313" t="str">
+        <v>no</v>
+      </c>
+      <c r="H313" t="str">
+        <v>["good afternoon","have a good day","i am learning"]</v>
+      </c>
+      <c r="I313" t="str">
+        <v>no</v>
+      </c>
+      <c r="J313" t="str">
+        <v>["no"]</v>
+      </c>
+      <c r="K313" t="str">
+        <v/>
+      </c>
+      <c r="L313" t="b">
+        <v>0</v>
+      </c>
+      <c r="M313" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B314" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C314" t="str">
+        <v>sudanese-arabic-practice-challenge-02-good-afternoon</v>
+      </c>
+      <c r="D314">
+        <v>2</v>
+      </c>
+      <c r="E314" t="str">
+        <v>sentence-build-target</v>
+      </c>
+      <c r="F314" t="str">
+        <v>Build the Sudanese Arabic phrase for "good afternoon".</v>
+      </c>
+      <c r="G314" t="str">
+        <v>مساء الخير</v>
+      </c>
+      <c r="H314" t="str">
+        <v>["لا","يومك سعيد","أنا بتعلم..."]</v>
+      </c>
+      <c r="I314" t="str">
+        <v>good-afternoon</v>
+      </c>
+      <c r="J314" t="str">
+        <v>["good-afternoon"]</v>
+      </c>
+      <c r="K314" t="str">
+        <v/>
+      </c>
+      <c r="L314" t="b">
+        <v>0</v>
+      </c>
+      <c r="M314" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B315" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C315" t="str">
+        <v>sudanese-arabic-practice-challenge-03-match</v>
+      </c>
+      <c r="D315">
+        <v>3</v>
+      </c>
+      <c r="E315" t="str">
+        <v>match-pairs</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Match each Sudanese Arabic phrase to its meaning.</v>
+      </c>
+      <c r="G315" t="str">
+        <v>__matched__</v>
+      </c>
+      <c r="H315" t="str">
+        <v>[]</v>
+      </c>
+      <c r="I315" t="str">
+        <v/>
+      </c>
+      <c r="J315" t="str">
+        <v>["no","good-afternoon","have-a-good-day","i-am-learning"]</v>
+      </c>
+      <c r="K315" t="str">
+        <v/>
+      </c>
+      <c r="L315" t="b">
+        <v>0</v>
+      </c>
+      <c r="M315" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B316" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C316" t="str">
+        <v>sudanese-arabic-practice-challenge-04-i-am-learning</v>
+      </c>
+      <c r="D316">
+        <v>4</v>
+      </c>
+      <c r="E316" t="str">
+        <v>word-tray-meaning</v>
+      </c>
+      <c r="F316" t="str">
+        <v>Build the English meaning of "أنا بتعلم...".</v>
+      </c>
+      <c r="G316" t="str">
+        <v>i am learning</v>
+      </c>
+      <c r="H316" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I316" t="str">
+        <v>i-am-learning</v>
+      </c>
+      <c r="J316" t="str">
+        <v>["i-am-learning"]</v>
+      </c>
+      <c r="K316" t="str">
+        <v/>
+      </c>
+      <c r="L316" t="b">
+        <v>0</v>
+      </c>
+      <c r="M316" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B317" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C317" t="str">
+        <v>sudanese-arabic-practice-challenge-05-where-do-you-live</v>
+      </c>
+      <c r="D317">
+        <v>5</v>
+      </c>
+      <c r="E317" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F317" t="str">
+        <v>Choose the Sudanese Arabic for "where do you live".</v>
+      </c>
+      <c r="G317" t="str">
+        <v>ساكن وين؟</v>
+      </c>
+      <c r="H317" t="str">
+        <v>["لا","مساء الخير","يومك سعيد"]</v>
+      </c>
+      <c r="I317" t="str">
+        <v>where-do-you-live</v>
+      </c>
+      <c r="J317" t="str">
+        <v>["where-do-you-live"]</v>
+      </c>
+      <c r="K317" t="str">
+        <v/>
+      </c>
+      <c r="L317" t="b">
+        <v>0</v>
+      </c>
+      <c r="M317" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B318" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C318" t="str">
+        <v>sudanese-arabic-practice-challenge-06-parents</v>
+      </c>
+      <c r="D318">
+        <v>6</v>
+      </c>
+      <c r="E318" t="str">
+        <v>listen-choice</v>
+      </c>
+      <c r="F318" t="str">
+        <v>Listen, then choose the English meaning.</v>
+      </c>
+      <c r="G318" t="str">
+        <v>parents</v>
+      </c>
+      <c r="H318" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I318" t="str">
+        <v>parents</v>
+      </c>
+      <c r="J318" t="str">
+        <v>["parents"]</v>
+      </c>
+      <c r="K318" t="str">
+        <v/>
+      </c>
+      <c r="L318" t="b">
+        <v>0</v>
+      </c>
+      <c r="M318" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B319" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C319" t="str">
+        <v>sudanese-arabic-practice-challenge-07-daughter</v>
+      </c>
+      <c r="D319">
+        <v>7</v>
+      </c>
+      <c r="E319" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Choose the Sudanese Arabic for "daughter".</v>
+      </c>
+      <c r="G319" t="str">
+        <v>بنت</v>
+      </c>
+      <c r="H319" t="str">
+        <v>["لا","مساء الخير","يومك سعيد"]</v>
+      </c>
+      <c r="I319" t="str">
+        <v>daughter</v>
+      </c>
+      <c r="J319" t="str">
+        <v>["daughter"]</v>
+      </c>
+      <c r="K319" t="str">
+        <v/>
+      </c>
+      <c r="L319" t="b">
+        <v>0</v>
+      </c>
+      <c r="M319" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B320" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C320" t="str">
+        <v>sudanese-arabic-practice-challenge-08-no-problem</v>
+      </c>
+      <c r="D320">
+        <v>8</v>
+      </c>
+      <c r="E320" t="str">
+        <v>translate-to-meaning</v>
+      </c>
+      <c r="F320" t="str">
+        <v>What does "ما في مشكلة" mean in Sudanese Arabic?</v>
+      </c>
+      <c r="G320" t="str">
+        <v>no problem</v>
+      </c>
+      <c r="H320" t="str">
+        <v>["no","good afternoon","have a good day"]</v>
+      </c>
+      <c r="I320" t="str">
+        <v>no-problem</v>
+      </c>
+      <c r="J320" t="str">
+        <v>["no-problem"]</v>
+      </c>
+      <c r="K320" t="str">
+        <v/>
+      </c>
+      <c r="L320" t="b">
+        <v>0</v>
+      </c>
+      <c r="M320" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>sudanese-arabic</v>
+      </c>
+      <c r="B321" t="str">
+        <v>practice-challenge</v>
+      </c>
+      <c r="C321" t="str">
+        <v>sudanese-arabic-practice-challenge-09-no-problem</v>
+      </c>
+      <c r="D321">
+        <v>9</v>
+      </c>
+      <c r="E321" t="str">
+        <v>translate-to-target</v>
+      </c>
+      <c r="F321" t="str">
+        <v>Choose the Sudanese Arabic for "no problem".</v>
+      </c>
+      <c r="G321" t="str">
+        <v>ما في مشكلة</v>
+      </c>
+      <c r="H321" t="str">
+        <v>["لا","مساء الخير","يومك سعيد"]</v>
+      </c>
+      <c r="I321" t="str">
+        <v>no-problem</v>
+      </c>
+      <c r="J321" t="str">
+        <v>["no-problem"]</v>
+      </c>
+      <c r="K321" t="str">
+        <v/>
+      </c>
+      <c r="L321" t="b">
+        <v>0</v>
+      </c>
+      <c r="M321" t="str">
+        <v>unavailable</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M257"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M321"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>